<commit_message>
state: bot run 2026-09-14T21:53 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K853"/>
+  <dimension ref="A1:K953"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37104,6 +37104,4306 @@
         <v>0</v>
       </c>
       <c r="K853" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1134.64 &lt;= EMA21 1138.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D854" t="n">
+        <v>7274</v>
+      </c>
+      <c r="E854" t="n">
+        <v>7702.71</v>
+      </c>
+      <c r="F854" t="n">
+        <v>7702.71</v>
+      </c>
+      <c r="G854" t="n">
+        <v>7393.78</v>
+      </c>
+      <c r="H854" t="n">
+        <v>7439.32</v>
+      </c>
+      <c r="I854" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J854" t="b">
+        <v>0</v>
+      </c>
+      <c r="K854" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7393.78 &lt;= EMA21 7439.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D855" t="n">
+        <v>1373</v>
+      </c>
+      <c r="E855" t="n">
+        <v>1672.08</v>
+      </c>
+      <c r="F855" t="n">
+        <v>1672.08</v>
+      </c>
+      <c r="G855" t="n">
+        <v>1415.65</v>
+      </c>
+      <c r="H855" t="n">
+        <v>1474.41</v>
+      </c>
+      <c r="I855" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J855" t="b">
+        <v>0</v>
+      </c>
+      <c r="K855" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1415.65 &lt;= EMA21 1474.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D856" t="n">
+        <v>3060</v>
+      </c>
+      <c r="E856" t="n">
+        <v>3196.42</v>
+      </c>
+      <c r="F856" t="n">
+        <v>3196.42</v>
+      </c>
+      <c r="G856" t="n">
+        <v>3016.07</v>
+      </c>
+      <c r="H856" t="n">
+        <v>3011.12</v>
+      </c>
+      <c r="I856" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J856" t="b">
+        <v>0</v>
+      </c>
+      <c r="K856" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3060.00 &lt;= Upper 3196.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D857" t="n">
+        <v>1281.3</v>
+      </c>
+      <c r="E857" t="n">
+        <v>1350.01</v>
+      </c>
+      <c r="F857" t="n">
+        <v>1350.01</v>
+      </c>
+      <c r="G857" t="n">
+        <v>1293.89</v>
+      </c>
+      <c r="H857" t="n">
+        <v>1309.64</v>
+      </c>
+      <c r="I857" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J857" t="b">
+        <v>0</v>
+      </c>
+      <c r="K857" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1293.89 &lt;= EMA21 1309.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D858" t="n">
+        <v>1764.6</v>
+      </c>
+      <c r="E858" t="n">
+        <v>1780.47</v>
+      </c>
+      <c r="F858" t="n">
+        <v>1780.47</v>
+      </c>
+      <c r="G858" t="n">
+        <v>1727.91</v>
+      </c>
+      <c r="H858" t="n">
+        <v>1712.62</v>
+      </c>
+      <c r="I858" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J858" t="b">
+        <v>0</v>
+      </c>
+      <c r="K858" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1764.60 &lt;= Upper 1780.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D859" t="n">
+        <v>209.97</v>
+      </c>
+      <c r="E859" t="n">
+        <v>215.83</v>
+      </c>
+      <c r="F859" t="n">
+        <v>215.83</v>
+      </c>
+      <c r="G859" t="n">
+        <v>209.54</v>
+      </c>
+      <c r="H859" t="n">
+        <v>208.76</v>
+      </c>
+      <c r="I859" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J859" t="b">
+        <v>0</v>
+      </c>
+      <c r="K859" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 209.97 &lt;= Upper 215.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D860" t="n">
+        <v>391.85</v>
+      </c>
+      <c r="E860" t="n">
+        <v>421.15</v>
+      </c>
+      <c r="F860" t="n">
+        <v>421.15</v>
+      </c>
+      <c r="G860" t="n">
+        <v>399.32</v>
+      </c>
+      <c r="H860" t="n">
+        <v>406.64</v>
+      </c>
+      <c r="I860" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J860" t="b">
+        <v>0</v>
+      </c>
+      <c r="K860" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 399.32 &lt;= EMA21 406.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D861" t="n">
+        <v>8836</v>
+      </c>
+      <c r="E861" t="n">
+        <v>8975.4</v>
+      </c>
+      <c r="F861" t="n">
+        <v>8975.4</v>
+      </c>
+      <c r="G861" t="n">
+        <v>8825.41</v>
+      </c>
+      <c r="H861" t="n">
+        <v>8809.1</v>
+      </c>
+      <c r="I861" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J861" t="b">
+        <v>0</v>
+      </c>
+      <c r="K861" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8836.00 &lt;= Upper 8975.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D862" t="n">
+        <v>2472.5</v>
+      </c>
+      <c r="E862" t="n">
+        <v>2718.87</v>
+      </c>
+      <c r="F862" t="n">
+        <v>2718.87</v>
+      </c>
+      <c r="G862" t="n">
+        <v>2517.86</v>
+      </c>
+      <c r="H862" t="n">
+        <v>2574.77</v>
+      </c>
+      <c r="I862" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J862" t="b">
+        <v>0</v>
+      </c>
+      <c r="K862" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2517.86 &lt;= EMA21 2574.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D863" t="n">
+        <v>3688</v>
+      </c>
+      <c r="E863" t="n">
+        <v>4042.24</v>
+      </c>
+      <c r="F863" t="n">
+        <v>4042.24</v>
+      </c>
+      <c r="G863" t="n">
+        <v>3746.7</v>
+      </c>
+      <c r="H863" t="n">
+        <v>3821.78</v>
+      </c>
+      <c r="I863" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J863" t="b">
+        <v>0</v>
+      </c>
+      <c r="K863" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3746.70 &lt;= EMA21 3821.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D864" t="n">
+        <v>1246</v>
+      </c>
+      <c r="E864" t="n">
+        <v>1285.71</v>
+      </c>
+      <c r="F864" t="n">
+        <v>1285.71</v>
+      </c>
+      <c r="G864" t="n">
+        <v>1251.58</v>
+      </c>
+      <c r="H864" t="n">
+        <v>1252.5</v>
+      </c>
+      <c r="I864" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J864" t="b">
+        <v>0</v>
+      </c>
+      <c r="K864" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1251.58 &lt;= EMA21 1252.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D865" t="n">
+        <v>11678</v>
+      </c>
+      <c r="E865" t="n">
+        <v>12220.66</v>
+      </c>
+      <c r="F865" t="n">
+        <v>12220.66</v>
+      </c>
+      <c r="G865" t="n">
+        <v>11829.92</v>
+      </c>
+      <c r="H865" t="n">
+        <v>11780.49</v>
+      </c>
+      <c r="I865" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J865" t="b">
+        <v>0</v>
+      </c>
+      <c r="K865" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11678.00 &lt;= Upper 12220.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D866" t="n">
+        <v>1034.5</v>
+      </c>
+      <c r="E866" t="n">
+        <v>1108.54</v>
+      </c>
+      <c r="F866" t="n">
+        <v>1108.54</v>
+      </c>
+      <c r="G866" t="n">
+        <v>1050.8</v>
+      </c>
+      <c r="H866" t="n">
+        <v>1062.63</v>
+      </c>
+      <c r="I866" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J866" t="b">
+        <v>0</v>
+      </c>
+      <c r="K866" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1050.80 &lt;= EMA21 1062.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D867" t="n">
+        <v>1913.5</v>
+      </c>
+      <c r="E867" t="n">
+        <v>2056.25</v>
+      </c>
+      <c r="F867" t="n">
+        <v>2056.25</v>
+      </c>
+      <c r="G867" t="n">
+        <v>1950.38</v>
+      </c>
+      <c r="H867" t="n">
+        <v>1970.38</v>
+      </c>
+      <c r="I867" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J867" t="b">
+        <v>0</v>
+      </c>
+      <c r="K867" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1950.38 &lt;= EMA21 1970.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D868" t="n">
+        <v>11134</v>
+      </c>
+      <c r="E868" t="n">
+        <v>11609.91</v>
+      </c>
+      <c r="F868" t="n">
+        <v>11609.91</v>
+      </c>
+      <c r="G868" t="n">
+        <v>11126.48</v>
+      </c>
+      <c r="H868" t="n">
+        <v>11186.8</v>
+      </c>
+      <c r="I868" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J868" t="b">
+        <v>0</v>
+      </c>
+      <c r="K868" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11126.48 &lt;= EMA21 11186.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D869" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="E869" t="n">
+        <v>247.72</v>
+      </c>
+      <c r="F869" t="n">
+        <v>247.72</v>
+      </c>
+      <c r="G869" t="n">
+        <v>238.13</v>
+      </c>
+      <c r="H869" t="n">
+        <v>240.63</v>
+      </c>
+      <c r="I869" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J869" t="b">
+        <v>0</v>
+      </c>
+      <c r="K869" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 238.13 &lt;= EMA21 240.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D870" t="n">
+        <v>404.35</v>
+      </c>
+      <c r="E870" t="n">
+        <v>415.91</v>
+      </c>
+      <c r="F870" t="n">
+        <v>415.91</v>
+      </c>
+      <c r="G870" t="n">
+        <v>406.73</v>
+      </c>
+      <c r="H870" t="n">
+        <v>407.22</v>
+      </c>
+      <c r="I870" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J870" t="b">
+        <v>0</v>
+      </c>
+      <c r="K870" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 406.73 &lt;= EMA21 407.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D871" t="n">
+        <v>304.5</v>
+      </c>
+      <c r="E871" t="n">
+        <v>326.04</v>
+      </c>
+      <c r="F871" t="n">
+        <v>326.04</v>
+      </c>
+      <c r="G871" t="n">
+        <v>309.16</v>
+      </c>
+      <c r="H871" t="n">
+        <v>312.58</v>
+      </c>
+      <c r="I871" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J871" t="b">
+        <v>0</v>
+      </c>
+      <c r="K871" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 309.16 &lt;= EMA21 312.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D872" t="n">
+        <v>1831.1</v>
+      </c>
+      <c r="E872" t="n">
+        <v>1982.75</v>
+      </c>
+      <c r="F872" t="n">
+        <v>1982.75</v>
+      </c>
+      <c r="G872" t="n">
+        <v>1847.48</v>
+      </c>
+      <c r="H872" t="n">
+        <v>1874.66</v>
+      </c>
+      <c r="I872" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J872" t="b">
+        <v>0</v>
+      </c>
+      <c r="K872" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1847.48 &lt;= EMA21 1874.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D873" t="n">
+        <v>48385</v>
+      </c>
+      <c r="E873" t="n">
+        <v>49944.45</v>
+      </c>
+      <c r="F873" t="n">
+        <v>49944.45</v>
+      </c>
+      <c r="G873" t="n">
+        <v>48352.85</v>
+      </c>
+      <c r="H873" t="n">
+        <v>47573.2</v>
+      </c>
+      <c r="I873" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J873" t="b">
+        <v>0</v>
+      </c>
+      <c r="K873" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 48385.00 &lt;= Upper 49944.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D874" t="n">
+        <v>4962</v>
+      </c>
+      <c r="E874" t="n">
+        <v>5604.87</v>
+      </c>
+      <c r="F874" t="n">
+        <v>5604.87</v>
+      </c>
+      <c r="G874" t="n">
+        <v>5088.56</v>
+      </c>
+      <c r="H874" t="n">
+        <v>5206.69</v>
+      </c>
+      <c r="I874" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J874" t="b">
+        <v>0</v>
+      </c>
+      <c r="K874" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5088.56 &lt;= EMA21 5206.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D875" t="n">
+        <v>909</v>
+      </c>
+      <c r="E875" t="n">
+        <v>927.35</v>
+      </c>
+      <c r="F875" t="n">
+        <v>927.35</v>
+      </c>
+      <c r="G875" t="n">
+        <v>904.46</v>
+      </c>
+      <c r="H875" t="n">
+        <v>895.64</v>
+      </c>
+      <c r="I875" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J875" t="b">
+        <v>0</v>
+      </c>
+      <c r="K875" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 909.00 &lt;= Upper 927.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D876" t="n">
+        <v>124</v>
+      </c>
+      <c r="E876" t="n">
+        <v>131.64</v>
+      </c>
+      <c r="F876" t="n">
+        <v>131.64</v>
+      </c>
+      <c r="G876" t="n">
+        <v>125.13</v>
+      </c>
+      <c r="H876" t="n">
+        <v>126.46</v>
+      </c>
+      <c r="I876" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J876" t="b">
+        <v>0</v>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 125.13 &lt;= EMA21 126.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D877" t="n">
+        <v>1845.9</v>
+      </c>
+      <c r="E877" t="n">
+        <v>1902.18</v>
+      </c>
+      <c r="F877" t="n">
+        <v>1902.18</v>
+      </c>
+      <c r="G877" t="n">
+        <v>1844.61</v>
+      </c>
+      <c r="H877" t="n">
+        <v>1849.23</v>
+      </c>
+      <c r="I877" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J877" t="b">
+        <v>0</v>
+      </c>
+      <c r="K877" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1844.61 &lt;= EMA21 1849.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D878" t="n">
+        <v>1366</v>
+      </c>
+      <c r="E878" t="n">
+        <v>1462.1</v>
+      </c>
+      <c r="F878" t="n">
+        <v>1462.1</v>
+      </c>
+      <c r="G878" t="n">
+        <v>1386.54</v>
+      </c>
+      <c r="H878" t="n">
+        <v>1406.74</v>
+      </c>
+      <c r="I878" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="J878" t="b">
+        <v>0</v>
+      </c>
+      <c r="K878" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1386.54 &lt;= EMA21 1406.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D879" t="n">
+        <v>426.4</v>
+      </c>
+      <c r="E879" t="n">
+        <v>432.82</v>
+      </c>
+      <c r="F879" t="n">
+        <v>432.82</v>
+      </c>
+      <c r="G879" t="n">
+        <v>419.96</v>
+      </c>
+      <c r="H879" t="n">
+        <v>413.04</v>
+      </c>
+      <c r="I879" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J879" t="b">
+        <v>0</v>
+      </c>
+      <c r="K879" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 426.40 &lt;= Upper 432.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D880" t="n">
+        <v>5070</v>
+      </c>
+      <c r="E880" t="n">
+        <v>5407.25</v>
+      </c>
+      <c r="F880" t="n">
+        <v>5407.25</v>
+      </c>
+      <c r="G880" t="n">
+        <v>5115.57</v>
+      </c>
+      <c r="H880" t="n">
+        <v>5186.39</v>
+      </c>
+      <c r="I880" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J880" t="b">
+        <v>0</v>
+      </c>
+      <c r="K880" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5115.57 &lt;= EMA21 5186.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D881" t="n">
+        <v>644.5</v>
+      </c>
+      <c r="E881" t="n">
+        <v>695.92</v>
+      </c>
+      <c r="F881" t="n">
+        <v>695.92</v>
+      </c>
+      <c r="G881" t="n">
+        <v>664.84</v>
+      </c>
+      <c r="H881" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="I881" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J881" t="b">
+        <v>0</v>
+      </c>
+      <c r="K881" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 664.84 &lt;= EMA21 667.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D882" t="n">
+        <v>9322</v>
+      </c>
+      <c r="E882" t="n">
+        <v>9784.209999999999</v>
+      </c>
+      <c r="F882" t="n">
+        <v>9784.209999999999</v>
+      </c>
+      <c r="G882" t="n">
+        <v>9310.49</v>
+      </c>
+      <c r="H882" t="n">
+        <v>9019.92</v>
+      </c>
+      <c r="I882" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J882" t="b">
+        <v>0</v>
+      </c>
+      <c r="K882" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9322.00 &lt;= Upper 9784.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D883" t="n">
+        <v>1165.5</v>
+      </c>
+      <c r="E883" t="n">
+        <v>1200.7</v>
+      </c>
+      <c r="F883" t="n">
+        <v>1200.7</v>
+      </c>
+      <c r="G883" t="n">
+        <v>1155.83</v>
+      </c>
+      <c r="H883" t="n">
+        <v>1165.86</v>
+      </c>
+      <c r="I883" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="J883" t="b">
+        <v>0</v>
+      </c>
+      <c r="K883" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1155.83 &lt;= EMA21 1165.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D884" t="n">
+        <v>7530</v>
+      </c>
+      <c r="E884" t="n">
+        <v>8268.68</v>
+      </c>
+      <c r="F884" t="n">
+        <v>8268.68</v>
+      </c>
+      <c r="G884" t="n">
+        <v>7735.32</v>
+      </c>
+      <c r="H884" t="n">
+        <v>7822.06</v>
+      </c>
+      <c r="I884" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J884" t="b">
+        <v>0</v>
+      </c>
+      <c r="K884" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7735.32 &lt;= EMA21 7822.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D885" t="n">
+        <v>323.5</v>
+      </c>
+      <c r="E885" t="n">
+        <v>332.95</v>
+      </c>
+      <c r="F885" t="n">
+        <v>332.95</v>
+      </c>
+      <c r="G885" t="n">
+        <v>323.56</v>
+      </c>
+      <c r="H885" t="n">
+        <v>321.37</v>
+      </c>
+      <c r="I885" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J885" t="b">
+        <v>0</v>
+      </c>
+      <c r="K885" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 323.50 &lt;= Upper 332.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D886" t="n">
+        <v>173.62</v>
+      </c>
+      <c r="E886" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="F886" t="n">
+        <v>176.8</v>
+      </c>
+      <c r="G886" t="n">
+        <v>174.22</v>
+      </c>
+      <c r="H886" t="n">
+        <v>173.94</v>
+      </c>
+      <c r="I886" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J886" t="b">
+        <v>0</v>
+      </c>
+      <c r="K886" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 173.62 &lt;= Upper 176.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D887" t="n">
+        <v>865</v>
+      </c>
+      <c r="E887" t="n">
+        <v>961.48</v>
+      </c>
+      <c r="F887" t="n">
+        <v>961.48</v>
+      </c>
+      <c r="G887" t="n">
+        <v>878.22</v>
+      </c>
+      <c r="H887" t="n">
+        <v>909.62</v>
+      </c>
+      <c r="I887" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J887" t="b">
+        <v>0</v>
+      </c>
+      <c r="K887" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 878.22 &lt;= EMA21 909.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D888" t="n">
+        <v>3281.9</v>
+      </c>
+      <c r="E888" t="n">
+        <v>3349.74</v>
+      </c>
+      <c r="F888" t="n">
+        <v>3349.74</v>
+      </c>
+      <c r="G888" t="n">
+        <v>3302.47</v>
+      </c>
+      <c r="H888" t="n">
+        <v>3286.59</v>
+      </c>
+      <c r="I888" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J888" t="b">
+        <v>0</v>
+      </c>
+      <c r="K888" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3281.90 &lt;= Upper 3349.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D889" t="n">
+        <v>1206.1</v>
+      </c>
+      <c r="E889" t="n">
+        <v>1375.06</v>
+      </c>
+      <c r="F889" t="n">
+        <v>1375.06</v>
+      </c>
+      <c r="G889" t="n">
+        <v>1258.84</v>
+      </c>
+      <c r="H889" t="n">
+        <v>1284.78</v>
+      </c>
+      <c r="I889" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J889" t="b">
+        <v>0</v>
+      </c>
+      <c r="K889" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1258.84 &lt;= EMA21 1284.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D890" t="n">
+        <v>2403.9</v>
+      </c>
+      <c r="E890" t="n">
+        <v>2705.79</v>
+      </c>
+      <c r="F890" t="n">
+        <v>2705.79</v>
+      </c>
+      <c r="G890" t="n">
+        <v>2474.74</v>
+      </c>
+      <c r="H890" t="n">
+        <v>2520.27</v>
+      </c>
+      <c r="I890" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J890" t="b">
+        <v>0</v>
+      </c>
+      <c r="K890" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2474.74 &lt;= EMA21 2520.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D891" t="n">
+        <v>708.25</v>
+      </c>
+      <c r="E891" t="n">
+        <v>738.48</v>
+      </c>
+      <c r="F891" t="n">
+        <v>738.48</v>
+      </c>
+      <c r="G891" t="n">
+        <v>704.51</v>
+      </c>
+      <c r="H891" t="n">
+        <v>714.47</v>
+      </c>
+      <c r="I891" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J891" t="b">
+        <v>0</v>
+      </c>
+      <c r="K891" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 704.51 &lt;= EMA21 714.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D892" t="n">
+        <v>530</v>
+      </c>
+      <c r="E892" t="n">
+        <v>560.12</v>
+      </c>
+      <c r="F892" t="n">
+        <v>560.12</v>
+      </c>
+      <c r="G892" t="n">
+        <v>531.9299999999999</v>
+      </c>
+      <c r="H892" t="n">
+        <v>537.8</v>
+      </c>
+      <c r="I892" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J892" t="b">
+        <v>0</v>
+      </c>
+      <c r="K892" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 531.93 &lt;= EMA21 537.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D893" t="n">
+        <v>981.5</v>
+      </c>
+      <c r="E893" t="n">
+        <v>1065.39</v>
+      </c>
+      <c r="F893" t="n">
+        <v>1065.39</v>
+      </c>
+      <c r="G893" t="n">
+        <v>1011.48</v>
+      </c>
+      <c r="H893" t="n">
+        <v>1017.9</v>
+      </c>
+      <c r="I893" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J893" t="b">
+        <v>0</v>
+      </c>
+      <c r="K893" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1011.48 &lt;= EMA21 1017.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D894" t="n">
+        <v>4905</v>
+      </c>
+      <c r="E894" t="n">
+        <v>5124.52</v>
+      </c>
+      <c r="F894" t="n">
+        <v>5124.52</v>
+      </c>
+      <c r="G894" t="n">
+        <v>4911.27</v>
+      </c>
+      <c r="H894" t="n">
+        <v>4880.9</v>
+      </c>
+      <c r="I894" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J894" t="b">
+        <v>0</v>
+      </c>
+      <c r="K894" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4905.00 &lt;= Upper 5124.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D895" t="n">
+        <v>1927</v>
+      </c>
+      <c r="E895" t="n">
+        <v>2078.66</v>
+      </c>
+      <c r="F895" t="n">
+        <v>2078.66</v>
+      </c>
+      <c r="G895" t="n">
+        <v>1963.32</v>
+      </c>
+      <c r="H895" t="n">
+        <v>1998.98</v>
+      </c>
+      <c r="I895" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J895" t="b">
+        <v>0</v>
+      </c>
+      <c r="K895" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1963.32 &lt;= EMA21 1998.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D896" t="n">
+        <v>576.45</v>
+      </c>
+      <c r="E896" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="F896" t="n">
+        <v>628.73</v>
+      </c>
+      <c r="G896" t="n">
+        <v>592.39</v>
+      </c>
+      <c r="H896" t="n">
+        <v>589.0599999999999</v>
+      </c>
+      <c r="I896" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J896" t="b">
+        <v>0</v>
+      </c>
+      <c r="K896" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 576.45 &lt;= Upper 628.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D897" t="n">
+        <v>2174</v>
+      </c>
+      <c r="E897" t="n">
+        <v>2267.66</v>
+      </c>
+      <c r="F897" t="n">
+        <v>2267.66</v>
+      </c>
+      <c r="G897" t="n">
+        <v>2195.03</v>
+      </c>
+      <c r="H897" t="n">
+        <v>2188.67</v>
+      </c>
+      <c r="I897" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J897" t="b">
+        <v>0</v>
+      </c>
+      <c r="K897" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 2174.00 &lt;= Upper 2267.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D898" t="n">
+        <v>1379.3</v>
+      </c>
+      <c r="E898" t="n">
+        <v>1455.66</v>
+      </c>
+      <c r="F898" t="n">
+        <v>1455.66</v>
+      </c>
+      <c r="G898" t="n">
+        <v>1403.74</v>
+      </c>
+      <c r="H898" t="n">
+        <v>1413.97</v>
+      </c>
+      <c r="I898" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J898" t="b">
+        <v>0</v>
+      </c>
+      <c r="K898" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1403.74 &lt;= EMA21 1413.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D899" t="n">
+        <v>259.85</v>
+      </c>
+      <c r="E899" t="n">
+        <v>275.47</v>
+      </c>
+      <c r="F899" t="n">
+        <v>275.47</v>
+      </c>
+      <c r="G899" t="n">
+        <v>262.51</v>
+      </c>
+      <c r="H899" t="n">
+        <v>266.83</v>
+      </c>
+      <c r="I899" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J899" t="b">
+        <v>0</v>
+      </c>
+      <c r="K899" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.51 &lt;= EMA21 266.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D900" t="n">
+        <v>718.5</v>
+      </c>
+      <c r="E900" t="n">
+        <v>738.38</v>
+      </c>
+      <c r="F900" t="n">
+        <v>738.38</v>
+      </c>
+      <c r="G900" t="n">
+        <v>720.5700000000001</v>
+      </c>
+      <c r="H900" t="n">
+        <v>723.12</v>
+      </c>
+      <c r="I900" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J900" t="b">
+        <v>0</v>
+      </c>
+      <c r="K900" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 720.57 &lt;= EMA21 723.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D901" t="n">
+        <v>135.11</v>
+      </c>
+      <c r="E901" t="n">
+        <v>140.04</v>
+      </c>
+      <c r="F901" t="n">
+        <v>140.04</v>
+      </c>
+      <c r="G901" t="n">
+        <v>135.92</v>
+      </c>
+      <c r="H901" t="n">
+        <v>137.01</v>
+      </c>
+      <c r="I901" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J901" t="b">
+        <v>0</v>
+      </c>
+      <c r="K901" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.92 &lt;= EMA21 137.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D902" t="n">
+        <v>81.09</v>
+      </c>
+      <c r="E902" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="F902" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="G902" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H902" t="n">
+        <v>84.05</v>
+      </c>
+      <c r="I902" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J902" t="b">
+        <v>0</v>
+      </c>
+      <c r="K902" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 82.32 &lt;= EMA21 84.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D903" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="E903" t="n">
+        <v>1186.43</v>
+      </c>
+      <c r="F903" t="n">
+        <v>1186.43</v>
+      </c>
+      <c r="G903" t="n">
+        <v>1077.73</v>
+      </c>
+      <c r="H903" t="n">
+        <v>1104.02</v>
+      </c>
+      <c r="I903" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J903" t="b">
+        <v>0</v>
+      </c>
+      <c r="K903" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1077.73 &lt;= EMA21 1104.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D904" t="n">
+        <v>4973</v>
+      </c>
+      <c r="E904" t="n">
+        <v>5355.29</v>
+      </c>
+      <c r="F904" t="n">
+        <v>5355.29</v>
+      </c>
+      <c r="G904" t="n">
+        <v>5017.37</v>
+      </c>
+      <c r="H904" t="n">
+        <v>5096.4</v>
+      </c>
+      <c r="I904" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J904" t="b">
+        <v>0</v>
+      </c>
+      <c r="K904" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5017.37 &lt;= EMA21 5096.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D905" t="n">
+        <v>1265</v>
+      </c>
+      <c r="E905" t="n">
+        <v>1349.19</v>
+      </c>
+      <c r="F905" t="n">
+        <v>1349.19</v>
+      </c>
+      <c r="G905" t="n">
+        <v>1299.69</v>
+      </c>
+      <c r="H905" t="n">
+        <v>1300.58</v>
+      </c>
+      <c r="I905" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J905" t="b">
+        <v>0</v>
+      </c>
+      <c r="K905" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1299.69 &lt;= EMA21 1300.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D906" t="n">
+        <v>1120.5</v>
+      </c>
+      <c r="E906" t="n">
+        <v>1198.33</v>
+      </c>
+      <c r="F906" t="n">
+        <v>1198.33</v>
+      </c>
+      <c r="G906" t="n">
+        <v>1143.37</v>
+      </c>
+      <c r="H906" t="n">
+        <v>1137.54</v>
+      </c>
+      <c r="I906" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J906" t="b">
+        <v>0</v>
+      </c>
+      <c r="K906" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1120.50 &lt;= Upper 1198.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D907" t="n">
+        <v>229.9</v>
+      </c>
+      <c r="E907" t="n">
+        <v>251.3</v>
+      </c>
+      <c r="F907" t="n">
+        <v>251.3</v>
+      </c>
+      <c r="G907" t="n">
+        <v>234.41</v>
+      </c>
+      <c r="H907" t="n">
+        <v>238.89</v>
+      </c>
+      <c r="I907" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="J907" t="b">
+        <v>0</v>
+      </c>
+      <c r="K907" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.41 &lt;= EMA21 238.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D908" t="n">
+        <v>419</v>
+      </c>
+      <c r="E908" t="n">
+        <v>437.64</v>
+      </c>
+      <c r="F908" t="n">
+        <v>437.64</v>
+      </c>
+      <c r="G908" t="n">
+        <v>418.07</v>
+      </c>
+      <c r="H908" t="n">
+        <v>412.51</v>
+      </c>
+      <c r="I908" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J908" t="b">
+        <v>0</v>
+      </c>
+      <c r="K908" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 419.00 &lt;= Upper 437.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D909" t="n">
+        <v>4275</v>
+      </c>
+      <c r="E909" t="n">
+        <v>4718.38</v>
+      </c>
+      <c r="F909" t="n">
+        <v>4718.38</v>
+      </c>
+      <c r="G909" t="n">
+        <v>4434.19</v>
+      </c>
+      <c r="H909" t="n">
+        <v>4478.92</v>
+      </c>
+      <c r="I909" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J909" t="b">
+        <v>0</v>
+      </c>
+      <c r="K909" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4434.19 &lt;= EMA21 4478.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D910" t="n">
+        <v>3930.7</v>
+      </c>
+      <c r="E910" t="n">
+        <v>4138.99</v>
+      </c>
+      <c r="F910" t="n">
+        <v>4138.99</v>
+      </c>
+      <c r="G910" t="n">
+        <v>3965.73</v>
+      </c>
+      <c r="H910" t="n">
+        <v>3991.39</v>
+      </c>
+      <c r="I910" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J910" t="b">
+        <v>0</v>
+      </c>
+      <c r="K910" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3965.73 &lt;= EMA21 3991.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D911" t="n">
+        <v>1116.9</v>
+      </c>
+      <c r="E911" t="n">
+        <v>1303.91</v>
+      </c>
+      <c r="F911" t="n">
+        <v>1303.91</v>
+      </c>
+      <c r="G911" t="n">
+        <v>1185.75</v>
+      </c>
+      <c r="H911" t="n">
+        <v>1205.13</v>
+      </c>
+      <c r="I911" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="J911" t="b">
+        <v>0</v>
+      </c>
+      <c r="K911" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1185.75 &lt;= EMA21 1205.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D912" t="n">
+        <v>3107</v>
+      </c>
+      <c r="E912" t="n">
+        <v>3533.62</v>
+      </c>
+      <c r="F912" t="n">
+        <v>3533.62</v>
+      </c>
+      <c r="G912" t="n">
+        <v>3174.63</v>
+      </c>
+      <c r="H912" t="n">
+        <v>3244.86</v>
+      </c>
+      <c r="I912" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J912" t="b">
+        <v>0</v>
+      </c>
+      <c r="K912" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3174.63 &lt;= EMA21 3244.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D913" t="n">
+        <v>12400</v>
+      </c>
+      <c r="E913" t="n">
+        <v>14168.62</v>
+      </c>
+      <c r="F913" t="n">
+        <v>14168.62</v>
+      </c>
+      <c r="G913" t="n">
+        <v>12750.8</v>
+      </c>
+      <c r="H913" t="n">
+        <v>13094.55</v>
+      </c>
+      <c r="I913" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J913" t="b">
+        <v>0</v>
+      </c>
+      <c r="K913" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12750.80 &lt;= EMA21 13094.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D914" t="n">
+        <v>1037.7</v>
+      </c>
+      <c r="E914" t="n">
+        <v>1043.88</v>
+      </c>
+      <c r="F914" t="n">
+        <v>1043.88</v>
+      </c>
+      <c r="G914" t="n">
+        <v>1018.88</v>
+      </c>
+      <c r="H914" t="n">
+        <v>1021.62</v>
+      </c>
+      <c r="I914" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J914" t="b">
+        <v>0</v>
+      </c>
+      <c r="K914" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1018.88 &lt;= EMA21 1021.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D915" t="n">
+        <v>2339</v>
+      </c>
+      <c r="E915" t="n">
+        <v>2671.05</v>
+      </c>
+      <c r="F915" t="n">
+        <v>2671.05</v>
+      </c>
+      <c r="G915" t="n">
+        <v>2436.36</v>
+      </c>
+      <c r="H915" t="n">
+        <v>2472.92</v>
+      </c>
+      <c r="I915" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J915" t="b">
+        <v>0</v>
+      </c>
+      <c r="K915" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2436.36 &lt;= EMA21 2472.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D916" t="n">
+        <v>2792.1</v>
+      </c>
+      <c r="E916" t="n">
+        <v>3224.19</v>
+      </c>
+      <c r="F916" t="n">
+        <v>3224.19</v>
+      </c>
+      <c r="G916" t="n">
+        <v>2881.14</v>
+      </c>
+      <c r="H916" t="n">
+        <v>2931.33</v>
+      </c>
+      <c r="I916" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J916" t="b">
+        <v>0</v>
+      </c>
+      <c r="K916" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2881.14 &lt;= EMA21 2931.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D917" t="n">
+        <v>333.4</v>
+      </c>
+      <c r="E917" t="n">
+        <v>339.17</v>
+      </c>
+      <c r="F917" t="n">
+        <v>339.17</v>
+      </c>
+      <c r="G917" t="n">
+        <v>332.37</v>
+      </c>
+      <c r="H917" t="n">
+        <v>333.14</v>
+      </c>
+      <c r="I917" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J917" t="b">
+        <v>0</v>
+      </c>
+      <c r="K917" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 332.37 &lt;= EMA21 333.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D918" t="n">
+        <v>1383.3</v>
+      </c>
+      <c r="E918" t="n">
+        <v>1509.16</v>
+      </c>
+      <c r="F918" t="n">
+        <v>1509.16</v>
+      </c>
+      <c r="G918" t="n">
+        <v>1406.97</v>
+      </c>
+      <c r="H918" t="n">
+        <v>1433.45</v>
+      </c>
+      <c r="I918" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J918" t="b">
+        <v>0</v>
+      </c>
+      <c r="K918" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1406.97 &lt;= EMA21 1433.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D919" t="n">
+        <v>232.5</v>
+      </c>
+      <c r="E919" t="n">
+        <v>239.51</v>
+      </c>
+      <c r="F919" t="n">
+        <v>239.51</v>
+      </c>
+      <c r="G919" t="n">
+        <v>234.54</v>
+      </c>
+      <c r="H919" t="n">
+        <v>235.37</v>
+      </c>
+      <c r="I919" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="J919" t="b">
+        <v>0</v>
+      </c>
+      <c r="K919" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.54 &lt;= EMA21 235.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D920" t="n">
+        <v>1566.9</v>
+      </c>
+      <c r="E920" t="n">
+        <v>1707.64</v>
+      </c>
+      <c r="F920" t="n">
+        <v>1707.64</v>
+      </c>
+      <c r="G920" t="n">
+        <v>1597</v>
+      </c>
+      <c r="H920" t="n">
+        <v>1619.73</v>
+      </c>
+      <c r="I920" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J920" t="b">
+        <v>0</v>
+      </c>
+      <c r="K920" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1597.00 &lt;= EMA21 1619.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D921" t="n">
+        <v>353.45</v>
+      </c>
+      <c r="E921" t="n">
+        <v>373.59</v>
+      </c>
+      <c r="F921" t="n">
+        <v>373.59</v>
+      </c>
+      <c r="G921" t="n">
+        <v>352.94</v>
+      </c>
+      <c r="H921" t="n">
+        <v>360.12</v>
+      </c>
+      <c r="I921" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J921" t="b">
+        <v>0</v>
+      </c>
+      <c r="K921" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 352.94 &lt;= EMA21 360.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D922" t="n">
+        <v>269.1</v>
+      </c>
+      <c r="E922" t="n">
+        <v>272.41</v>
+      </c>
+      <c r="F922" t="n">
+        <v>272.41</v>
+      </c>
+      <c r="G922" t="n">
+        <v>267.58</v>
+      </c>
+      <c r="H922" t="n">
+        <v>268.76</v>
+      </c>
+      <c r="I922" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J922" t="b">
+        <v>0</v>
+      </c>
+      <c r="K922" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 267.58 &lt;= EMA21 268.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D923" t="n">
+        <v>116.75</v>
+      </c>
+      <c r="E923" t="n">
+        <v>118.09</v>
+      </c>
+      <c r="F923" t="n">
+        <v>118.09</v>
+      </c>
+      <c r="G923" t="n">
+        <v>116.26</v>
+      </c>
+      <c r="H923" t="n">
+        <v>115.76</v>
+      </c>
+      <c r="I923" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J923" t="b">
+        <v>0</v>
+      </c>
+      <c r="K923" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.75 &lt;= Upper 118.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D924" t="n">
+        <v>312.7</v>
+      </c>
+      <c r="E924" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="F924" t="n">
+        <v>339.4</v>
+      </c>
+      <c r="G924" t="n">
+        <v>316.38</v>
+      </c>
+      <c r="H924" t="n">
+        <v>323.82</v>
+      </c>
+      <c r="I924" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J924" t="b">
+        <v>0</v>
+      </c>
+      <c r="K924" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 316.38 &lt;= EMA21 323.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D925" t="n">
+        <v>1257.5</v>
+      </c>
+      <c r="E925" t="n">
+        <v>1337.45</v>
+      </c>
+      <c r="F925" t="n">
+        <v>1337.45</v>
+      </c>
+      <c r="G925" t="n">
+        <v>1286.91</v>
+      </c>
+      <c r="H925" t="n">
+        <v>1296.38</v>
+      </c>
+      <c r="I925" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J925" t="b">
+        <v>0</v>
+      </c>
+      <c r="K925" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1286.91 &lt;= EMA21 1296.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D926" t="n">
+        <v>1684.7</v>
+      </c>
+      <c r="E926" t="n">
+        <v>1818.08</v>
+      </c>
+      <c r="F926" t="n">
+        <v>1818.08</v>
+      </c>
+      <c r="G926" t="n">
+        <v>1714.46</v>
+      </c>
+      <c r="H926" t="n">
+        <v>1746.98</v>
+      </c>
+      <c r="I926" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J926" t="b">
+        <v>0</v>
+      </c>
+      <c r="K926" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1714.46 &lt;= EMA21 1746.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D927" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="E927" t="n">
+        <v>172.22</v>
+      </c>
+      <c r="F927" t="n">
+        <v>172.22</v>
+      </c>
+      <c r="G927" t="n">
+        <v>163.91</v>
+      </c>
+      <c r="H927" t="n">
+        <v>163.63</v>
+      </c>
+      <c r="I927" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J927" t="b">
+        <v>0</v>
+      </c>
+      <c r="K927" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 164.45 &lt;= Upper 172.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D928" t="n">
+        <v>22570</v>
+      </c>
+      <c r="E928" t="n">
+        <v>25190.51</v>
+      </c>
+      <c r="F928" t="n">
+        <v>25190.51</v>
+      </c>
+      <c r="G928" t="n">
+        <v>23235.17</v>
+      </c>
+      <c r="H928" t="n">
+        <v>23911.45</v>
+      </c>
+      <c r="I928" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J928" t="b">
+        <v>0</v>
+      </c>
+      <c r="K928" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 23235.17 &lt;= EMA21 23911.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D929" t="n">
+        <v>1028.6</v>
+      </c>
+      <c r="E929" t="n">
+        <v>1162.54</v>
+      </c>
+      <c r="F929" t="n">
+        <v>1162.54</v>
+      </c>
+      <c r="G929" t="n">
+        <v>1045.38</v>
+      </c>
+      <c r="H929" t="n">
+        <v>1065.7</v>
+      </c>
+      <c r="I929" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J929" t="b">
+        <v>0</v>
+      </c>
+      <c r="K929" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1045.38 &lt;= EMA21 1065.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D930" t="n">
+        <v>3181.3</v>
+      </c>
+      <c r="E930" t="n">
+        <v>3616.86</v>
+      </c>
+      <c r="F930" t="n">
+        <v>3616.86</v>
+      </c>
+      <c r="G930" t="n">
+        <v>3191.39</v>
+      </c>
+      <c r="H930" t="n">
+        <v>3259.74</v>
+      </c>
+      <c r="I930" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J930" t="b">
+        <v>0</v>
+      </c>
+      <c r="K930" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3191.39 &lt;= EMA21 3259.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D931" t="n">
+        <v>3957</v>
+      </c>
+      <c r="E931" t="n">
+        <v>4132.57</v>
+      </c>
+      <c r="F931" t="n">
+        <v>4132.57</v>
+      </c>
+      <c r="G931" t="n">
+        <v>3972.69</v>
+      </c>
+      <c r="H931" t="n">
+        <v>3965.16</v>
+      </c>
+      <c r="I931" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J931" t="b">
+        <v>0</v>
+      </c>
+      <c r="K931" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3957.00 &lt;= Upper 4132.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D932" t="n">
+        <v>22290</v>
+      </c>
+      <c r="E932" t="n">
+        <v>22809.23</v>
+      </c>
+      <c r="F932" t="n">
+        <v>22809.23</v>
+      </c>
+      <c r="G932" t="n">
+        <v>21758.36</v>
+      </c>
+      <c r="H932" t="n">
+        <v>20904.42</v>
+      </c>
+      <c r="I932" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J932" t="b">
+        <v>0</v>
+      </c>
+      <c r="K932" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 22290.00 &lt;= Upper 22809.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D933" t="n">
+        <v>995.7</v>
+      </c>
+      <c r="E933" t="n">
+        <v>1075.39</v>
+      </c>
+      <c r="F933" t="n">
+        <v>1075.39</v>
+      </c>
+      <c r="G933" t="n">
+        <v>1013.32</v>
+      </c>
+      <c r="H933" t="n">
+        <v>1027.66</v>
+      </c>
+      <c r="I933" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J933" t="b">
+        <v>0</v>
+      </c>
+      <c r="K933" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1013.32 &lt;= EMA21 1027.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D934" t="n">
+        <v>1840</v>
+      </c>
+      <c r="E934" t="n">
+        <v>1963.23</v>
+      </c>
+      <c r="F934" t="n">
+        <v>1963.23</v>
+      </c>
+      <c r="G934" t="n">
+        <v>1882.15</v>
+      </c>
+      <c r="H934" t="n">
+        <v>1902.01</v>
+      </c>
+      <c r="I934" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J934" t="b">
+        <v>0</v>
+      </c>
+      <c r="K934" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1882.15 &lt;= EMA21 1902.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D935" t="n">
+        <v>4125</v>
+      </c>
+      <c r="E935" t="n">
+        <v>4521.64</v>
+      </c>
+      <c r="F935" t="n">
+        <v>4521.64</v>
+      </c>
+      <c r="G935" t="n">
+        <v>4172.4</v>
+      </c>
+      <c r="H935" t="n">
+        <v>4215.96</v>
+      </c>
+      <c r="I935" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J935" t="b">
+        <v>0</v>
+      </c>
+      <c r="K935" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4172.40 &lt;= EMA21 4215.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D936" t="n">
+        <v>362.9</v>
+      </c>
+      <c r="E936" t="n">
+        <v>376.61</v>
+      </c>
+      <c r="F936" t="n">
+        <v>376.61</v>
+      </c>
+      <c r="G936" t="n">
+        <v>366.4</v>
+      </c>
+      <c r="H936" t="n">
+        <v>366.47</v>
+      </c>
+      <c r="I936" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J936" t="b">
+        <v>0</v>
+      </c>
+      <c r="K936" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 366.40 &lt;= EMA21 366.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D937" t="n">
+        <v>2200.8</v>
+      </c>
+      <c r="E937" t="n">
+        <v>2394.77</v>
+      </c>
+      <c r="F937" t="n">
+        <v>2394.77</v>
+      </c>
+      <c r="G937" t="n">
+        <v>2254.69</v>
+      </c>
+      <c r="H937" t="n">
+        <v>2286.71</v>
+      </c>
+      <c r="I937" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J937" t="b">
+        <v>0</v>
+      </c>
+      <c r="K937" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2254.69 &lt;= EMA21 2286.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D938" t="n">
+        <v>991</v>
+      </c>
+      <c r="E938" t="n">
+        <v>1084.99</v>
+      </c>
+      <c r="F938" t="n">
+        <v>1084.99</v>
+      </c>
+      <c r="G938" t="n">
+        <v>1010.97</v>
+      </c>
+      <c r="H938" t="n">
+        <v>1032.19</v>
+      </c>
+      <c r="I938" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J938" t="b">
+        <v>0</v>
+      </c>
+      <c r="K938" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1010.97 &lt;= EMA21 1032.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D939" t="n">
+        <v>434.55</v>
+      </c>
+      <c r="E939" t="n">
+        <v>491.42</v>
+      </c>
+      <c r="F939" t="n">
+        <v>491.42</v>
+      </c>
+      <c r="G939" t="n">
+        <v>450.34</v>
+      </c>
+      <c r="H939" t="n">
+        <v>455.2</v>
+      </c>
+      <c r="I939" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J939" t="b">
+        <v>0</v>
+      </c>
+      <c r="K939" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 450.34 &lt;= EMA21 455.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D940" t="n">
+        <v>301.1</v>
+      </c>
+      <c r="E940" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="F940" t="n">
+        <v>328.33</v>
+      </c>
+      <c r="G940" t="n">
+        <v>306.56</v>
+      </c>
+      <c r="H940" t="n">
+        <v>314.37</v>
+      </c>
+      <c r="I940" t="n">
+        <v>1</v>
+      </c>
+      <c r="J940" t="b">
+        <v>0</v>
+      </c>
+      <c r="K940" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 306.56 &lt;= EMA21 314.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D941" t="n">
+        <v>364.65</v>
+      </c>
+      <c r="E941" t="n">
+        <v>386.47</v>
+      </c>
+      <c r="F941" t="n">
+        <v>386.47</v>
+      </c>
+      <c r="G941" t="n">
+        <v>365.32</v>
+      </c>
+      <c r="H941" t="n">
+        <v>367.36</v>
+      </c>
+      <c r="I941" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J941" t="b">
+        <v>0</v>
+      </c>
+      <c r="K941" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 365.32 &lt;= EMA21 367.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D942" t="n">
+        <v>183</v>
+      </c>
+      <c r="E942" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="F942" t="n">
+        <v>189.16</v>
+      </c>
+      <c r="G942" t="n">
+        <v>185.57</v>
+      </c>
+      <c r="H942" t="n">
+        <v>185.89</v>
+      </c>
+      <c r="I942" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J942" t="b">
+        <v>0</v>
+      </c>
+      <c r="K942" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.57 &lt;= EMA21 185.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D943" t="n">
+        <v>1541</v>
+      </c>
+      <c r="E943" t="n">
+        <v>1656.32</v>
+      </c>
+      <c r="F943" t="n">
+        <v>1656.32</v>
+      </c>
+      <c r="G943" t="n">
+        <v>1560.35</v>
+      </c>
+      <c r="H943" t="n">
+        <v>1579.68</v>
+      </c>
+      <c r="I943" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J943" t="b">
+        <v>0</v>
+      </c>
+      <c r="K943" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1560.35 &lt;= EMA21 1579.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D944" t="n">
+        <v>5009.5</v>
+      </c>
+      <c r="E944" t="n">
+        <v>5161.3</v>
+      </c>
+      <c r="F944" t="n">
+        <v>5161.3</v>
+      </c>
+      <c r="G944" t="n">
+        <v>5025.8</v>
+      </c>
+      <c r="H944" t="n">
+        <v>5022.47</v>
+      </c>
+      <c r="I944" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J944" t="b">
+        <v>0</v>
+      </c>
+      <c r="K944" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 5009.50 &lt;= Upper 5161.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D945" t="n">
+        <v>4965.5</v>
+      </c>
+      <c r="E945" t="n">
+        <v>5068.18</v>
+      </c>
+      <c r="F945" t="n">
+        <v>5068.18</v>
+      </c>
+      <c r="G945" t="n">
+        <v>4944.35</v>
+      </c>
+      <c r="H945" t="n">
+        <v>4944.08</v>
+      </c>
+      <c r="I945" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J945" t="b">
+        <v>0</v>
+      </c>
+      <c r="K945" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4965.50 &lt;= Upper 5068.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D946" t="n">
+        <v>2802.4</v>
+      </c>
+      <c r="E946" t="n">
+        <v>2989.58</v>
+      </c>
+      <c r="F946" t="n">
+        <v>2989.58</v>
+      </c>
+      <c r="G946" t="n">
+        <v>2830.16</v>
+      </c>
+      <c r="H946" t="n">
+        <v>2873.65</v>
+      </c>
+      <c r="I946" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J946" t="b">
+        <v>0</v>
+      </c>
+      <c r="K946" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2830.16 &lt;= EMA21 2873.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D947" t="n">
+        <v>11000</v>
+      </c>
+      <c r="E947" t="n">
+        <v>11899.48</v>
+      </c>
+      <c r="F947" t="n">
+        <v>11899.48</v>
+      </c>
+      <c r="G947" t="n">
+        <v>11150.11</v>
+      </c>
+      <c r="H947" t="n">
+        <v>11348.94</v>
+      </c>
+      <c r="I947" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J947" t="b">
+        <v>0</v>
+      </c>
+      <c r="K947" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11150.11 &lt;= EMA21 11348.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D948" t="n">
+        <v>178.1</v>
+      </c>
+      <c r="E948" t="n">
+        <v>191.02</v>
+      </c>
+      <c r="F948" t="n">
+        <v>191.02</v>
+      </c>
+      <c r="G948" t="n">
+        <v>183.02</v>
+      </c>
+      <c r="H948" t="n">
+        <v>183.36</v>
+      </c>
+      <c r="I948" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J948" t="b">
+        <v>0</v>
+      </c>
+      <c r="K948" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 183.02 &lt;= EMA21 183.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D949" t="n">
+        <v>1395</v>
+      </c>
+      <c r="E949" t="n">
+        <v>1598.82</v>
+      </c>
+      <c r="F949" t="n">
+        <v>1598.82</v>
+      </c>
+      <c r="G949" t="n">
+        <v>1438.19</v>
+      </c>
+      <c r="H949" t="n">
+        <v>1468.95</v>
+      </c>
+      <c r="I949" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J949" t="b">
+        <v>0</v>
+      </c>
+      <c r="K949" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1438.19 &lt;= EMA21 1468.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D950" t="n">
+        <v>416.5</v>
+      </c>
+      <c r="E950" t="n">
+        <v>444.46</v>
+      </c>
+      <c r="F950" t="n">
+        <v>444.46</v>
+      </c>
+      <c r="G950" t="n">
+        <v>411.52</v>
+      </c>
+      <c r="H950" t="n">
+        <v>419.37</v>
+      </c>
+      <c r="I950" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J950" t="b">
+        <v>0</v>
+      </c>
+      <c r="K950" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 411.52 &lt;= EMA21 419.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D951" t="n">
+        <v>263.7</v>
+      </c>
+      <c r="E951" t="n">
+        <v>286.99</v>
+      </c>
+      <c r="F951" t="n">
+        <v>286.99</v>
+      </c>
+      <c r="G951" t="n">
+        <v>270.44</v>
+      </c>
+      <c r="H951" t="n">
+        <v>272.22</v>
+      </c>
+      <c r="I951" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J951" t="b">
+        <v>0</v>
+      </c>
+      <c r="K951" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 270.44 &lt;= EMA21 272.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>167.4</v>
+      </c>
+      <c r="E952" t="n">
+        <v>187.56</v>
+      </c>
+      <c r="F952" t="n">
+        <v>187.56</v>
+      </c>
+      <c r="G952" t="n">
+        <v>171.75</v>
+      </c>
+      <c r="H952" t="n">
+        <v>175.66</v>
+      </c>
+      <c r="I952" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J952" t="b">
+        <v>0</v>
+      </c>
+      <c r="K952" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 171.75 &lt;= EMA21 175.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>1119.1</v>
+      </c>
+      <c r="E953" t="n">
+        <v>1190.18</v>
+      </c>
+      <c r="F953" t="n">
+        <v>1190.18</v>
+      </c>
+      <c r="G953" t="n">
+        <v>1134.64</v>
+      </c>
+      <c r="H953" t="n">
+        <v>1138.08</v>
+      </c>
+      <c r="I953" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J953" t="b">
+        <v>0</v>
+      </c>
+      <c r="K953" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1134.64 &lt;= EMA21 1138.08)</t>
         </is>
@@ -37512,7 +41812,7 @@
         <v>436.2999877929688</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -37553,7 +41853,7 @@
         <v>1780</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -37594,7 +41894,7 @@
         <v>215.2799987792969</v>
       </c>
       <c r="J4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -43929,7 +48229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44375,6 +48675,39 @@
         <v>3</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>21:52:56</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>138772.28</v>
+      </c>
+      <c r="D14" t="n">
+        <v>59196.65</v>
+      </c>
+      <c r="E14" t="n">
+        <v>197968.93</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-1945.43</v>
+      </c>
+      <c r="G14" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>18</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-15T20:31 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K953"/>
+  <dimension ref="A1:K1053"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41406,6 +41406,4306 @@
       <c r="K953" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1134.64 &lt;= EMA21 1138.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>7005</v>
+      </c>
+      <c r="E954" t="n">
+        <v>7743.79</v>
+      </c>
+      <c r="F954" t="n">
+        <v>7743.79</v>
+      </c>
+      <c r="G954" t="n">
+        <v>7316.02</v>
+      </c>
+      <c r="H954" t="n">
+        <v>7399.84</v>
+      </c>
+      <c r="I954" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J954" t="b">
+        <v>0</v>
+      </c>
+      <c r="K954" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7316.02 &lt;= EMA21 7399.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D955" t="n">
+        <v>1347.5</v>
+      </c>
+      <c r="E955" t="n">
+        <v>1663.15</v>
+      </c>
+      <c r="F955" t="n">
+        <v>1663.15</v>
+      </c>
+      <c r="G955" t="n">
+        <v>1402.02</v>
+      </c>
+      <c r="H955" t="n">
+        <v>1462.87</v>
+      </c>
+      <c r="I955" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J955" t="b">
+        <v>0</v>
+      </c>
+      <c r="K955" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1402.02 &lt;= EMA21 1462.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D956" t="n">
+        <v>2928.6</v>
+      </c>
+      <c r="E956" t="n">
+        <v>3195.75</v>
+      </c>
+      <c r="F956" t="n">
+        <v>3195.75</v>
+      </c>
+      <c r="G956" t="n">
+        <v>2998.57</v>
+      </c>
+      <c r="H956" t="n">
+        <v>3003.61</v>
+      </c>
+      <c r="I956" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J956" t="b">
+        <v>0</v>
+      </c>
+      <c r="K956" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2998.57 &lt;= EMA21 3003.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D957" t="n">
+        <v>1255</v>
+      </c>
+      <c r="E957" t="n">
+        <v>1347.91</v>
+      </c>
+      <c r="F957" t="n">
+        <v>1347.91</v>
+      </c>
+      <c r="G957" t="n">
+        <v>1286.11</v>
+      </c>
+      <c r="H957" t="n">
+        <v>1304.68</v>
+      </c>
+      <c r="I957" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J957" t="b">
+        <v>0</v>
+      </c>
+      <c r="K957" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1286.11 &lt;= EMA21 1304.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D958" t="n">
+        <v>1713.8</v>
+      </c>
+      <c r="E958" t="n">
+        <v>1781.42</v>
+      </c>
+      <c r="F958" t="n">
+        <v>1781.42</v>
+      </c>
+      <c r="G958" t="n">
+        <v>1725.08</v>
+      </c>
+      <c r="H958" t="n">
+        <v>1712.73</v>
+      </c>
+      <c r="I958" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J958" t="b">
+        <v>0</v>
+      </c>
+      <c r="K958" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1713.80 &lt;= Upper 1781.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D959" t="n">
+        <v>202</v>
+      </c>
+      <c r="E959" t="n">
+        <v>215.91</v>
+      </c>
+      <c r="F959" t="n">
+        <v>215.91</v>
+      </c>
+      <c r="G959" t="n">
+        <v>208.04</v>
+      </c>
+      <c r="H959" t="n">
+        <v>208.15</v>
+      </c>
+      <c r="I959" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J959" t="b">
+        <v>0</v>
+      </c>
+      <c r="K959" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 208.04 &lt;= EMA21 208.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D960" t="n">
+        <v>381.75</v>
+      </c>
+      <c r="E960" t="n">
+        <v>422.37</v>
+      </c>
+      <c r="F960" t="n">
+        <v>422.37</v>
+      </c>
+      <c r="G960" t="n">
+        <v>395.81</v>
+      </c>
+      <c r="H960" t="n">
+        <v>404.37</v>
+      </c>
+      <c r="I960" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J960" t="b">
+        <v>0</v>
+      </c>
+      <c r="K960" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 395.81 &lt;= EMA21 404.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D961" t="n">
+        <v>8714</v>
+      </c>
+      <c r="E961" t="n">
+        <v>8959.34</v>
+      </c>
+      <c r="F961" t="n">
+        <v>8959.34</v>
+      </c>
+      <c r="G961" t="n">
+        <v>8803.120000000001</v>
+      </c>
+      <c r="H961" t="n">
+        <v>8800.450000000001</v>
+      </c>
+      <c r="I961" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J961" t="b">
+        <v>0</v>
+      </c>
+      <c r="K961" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8714.00 &lt;= Upper 8959.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D962" t="n">
+        <v>2402.8</v>
+      </c>
+      <c r="E962" t="n">
+        <v>2716.76</v>
+      </c>
+      <c r="F962" t="n">
+        <v>2716.76</v>
+      </c>
+      <c r="G962" t="n">
+        <v>2494.85</v>
+      </c>
+      <c r="H962" t="n">
+        <v>2559.14</v>
+      </c>
+      <c r="I962" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J962" t="b">
+        <v>0</v>
+      </c>
+      <c r="K962" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2494.85 &lt;= EMA21 2559.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D963" t="n">
+        <v>3680</v>
+      </c>
+      <c r="E963" t="n">
+        <v>4024.33</v>
+      </c>
+      <c r="F963" t="n">
+        <v>4024.33</v>
+      </c>
+      <c r="G963" t="n">
+        <v>3733.36</v>
+      </c>
+      <c r="H963" t="n">
+        <v>3808.89</v>
+      </c>
+      <c r="I963" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J963" t="b">
+        <v>0</v>
+      </c>
+      <c r="K963" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3733.36 &lt;= EMA21 3808.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D964" t="n">
+        <v>1222.9</v>
+      </c>
+      <c r="E964" t="n">
+        <v>1285.02</v>
+      </c>
+      <c r="F964" t="n">
+        <v>1285.02</v>
+      </c>
+      <c r="G964" t="n">
+        <v>1245.84</v>
+      </c>
+      <c r="H964" t="n">
+        <v>1249.81</v>
+      </c>
+      <c r="I964" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J964" t="b">
+        <v>0</v>
+      </c>
+      <c r="K964" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1245.84 &lt;= EMA21 1249.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D965" t="n">
+        <v>11424</v>
+      </c>
+      <c r="E965" t="n">
+        <v>12246.03</v>
+      </c>
+      <c r="F965" t="n">
+        <v>12246.03</v>
+      </c>
+      <c r="G965" t="n">
+        <v>11748.74</v>
+      </c>
+      <c r="H965" t="n">
+        <v>11748.08</v>
+      </c>
+      <c r="I965" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J965" t="b">
+        <v>0</v>
+      </c>
+      <c r="K965" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 11424.00 &lt;= Upper 12246.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D966" t="n">
+        <v>1009.2</v>
+      </c>
+      <c r="E966" t="n">
+        <v>1111.33</v>
+      </c>
+      <c r="F966" t="n">
+        <v>1111.33</v>
+      </c>
+      <c r="G966" t="n">
+        <v>1042.48</v>
+      </c>
+      <c r="H966" t="n">
+        <v>1057.77</v>
+      </c>
+      <c r="I966" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J966" t="b">
+        <v>0</v>
+      </c>
+      <c r="K966" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1042.48 &lt;= EMA21 1057.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D967" t="n">
+        <v>1855.5</v>
+      </c>
+      <c r="E967" t="n">
+        <v>2068.79</v>
+      </c>
+      <c r="F967" t="n">
+        <v>2068.79</v>
+      </c>
+      <c r="G967" t="n">
+        <v>1931.4</v>
+      </c>
+      <c r="H967" t="n">
+        <v>1959.94</v>
+      </c>
+      <c r="I967" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J967" t="b">
+        <v>0</v>
+      </c>
+      <c r="K967" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1931.40 &lt;= EMA21 1959.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>11100</v>
+      </c>
+      <c r="E968" t="n">
+        <v>11596.34</v>
+      </c>
+      <c r="F968" t="n">
+        <v>11596.34</v>
+      </c>
+      <c r="G968" t="n">
+        <v>11121.18</v>
+      </c>
+      <c r="H968" t="n">
+        <v>11178.91</v>
+      </c>
+      <c r="I968" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J968" t="b">
+        <v>0</v>
+      </c>
+      <c r="K968" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11121.18 &lt;= EMA21 11178.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D969" t="n">
+        <v>232.7</v>
+      </c>
+      <c r="E969" t="n">
+        <v>247.36</v>
+      </c>
+      <c r="F969" t="n">
+        <v>247.36</v>
+      </c>
+      <c r="G969" t="n">
+        <v>237.04</v>
+      </c>
+      <c r="H969" t="n">
+        <v>239.91</v>
+      </c>
+      <c r="I969" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J969" t="b">
+        <v>0</v>
+      </c>
+      <c r="K969" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 237.04 &lt;= EMA21 239.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D970" t="n">
+        <v>382.9</v>
+      </c>
+      <c r="E970" t="n">
+        <v>421.13</v>
+      </c>
+      <c r="F970" t="n">
+        <v>421.13</v>
+      </c>
+      <c r="G970" t="n">
+        <v>401.97</v>
+      </c>
+      <c r="H970" t="n">
+        <v>405.01</v>
+      </c>
+      <c r="I970" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J970" t="b">
+        <v>0</v>
+      </c>
+      <c r="K970" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 401.97 &lt;= EMA21 405.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D971" t="n">
+        <v>298.65</v>
+      </c>
+      <c r="E971" t="n">
+        <v>326.56</v>
+      </c>
+      <c r="F971" t="n">
+        <v>326.56</v>
+      </c>
+      <c r="G971" t="n">
+        <v>307.06</v>
+      </c>
+      <c r="H971" t="n">
+        <v>311.31</v>
+      </c>
+      <c r="I971" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J971" t="b">
+        <v>0</v>
+      </c>
+      <c r="K971" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 307.06 &lt;= EMA21 311.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>1830.4</v>
+      </c>
+      <c r="E972" t="n">
+        <v>1970.18</v>
+      </c>
+      <c r="F972" t="n">
+        <v>1970.18</v>
+      </c>
+      <c r="G972" t="n">
+        <v>1844.07</v>
+      </c>
+      <c r="H972" t="n">
+        <v>1870.64</v>
+      </c>
+      <c r="I972" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J972" t="b">
+        <v>0</v>
+      </c>
+      <c r="K972" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1844.07 &lt;= EMA21 1870.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D973" t="n">
+        <v>47070</v>
+      </c>
+      <c r="E973" t="n">
+        <v>49931.88</v>
+      </c>
+      <c r="F973" t="n">
+        <v>49931.88</v>
+      </c>
+      <c r="G973" t="n">
+        <v>48096.28</v>
+      </c>
+      <c r="H973" t="n">
+        <v>47527.45</v>
+      </c>
+      <c r="I973" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J973" t="b">
+        <v>0</v>
+      </c>
+      <c r="K973" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47070.00 &lt;= Upper 49931.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D974" t="n">
+        <v>4947.5</v>
+      </c>
+      <c r="E974" t="n">
+        <v>5576.37</v>
+      </c>
+      <c r="F974" t="n">
+        <v>5576.37</v>
+      </c>
+      <c r="G974" t="n">
+        <v>5060.34</v>
+      </c>
+      <c r="H974" t="n">
+        <v>5183.13</v>
+      </c>
+      <c r="I974" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J974" t="b">
+        <v>0</v>
+      </c>
+      <c r="K974" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5060.34 &lt;= EMA21 5183.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D975" t="n">
+        <v>858</v>
+      </c>
+      <c r="E975" t="n">
+        <v>928.08</v>
+      </c>
+      <c r="F975" t="n">
+        <v>928.08</v>
+      </c>
+      <c r="G975" t="n">
+        <v>895.17</v>
+      </c>
+      <c r="H975" t="n">
+        <v>892.22</v>
+      </c>
+      <c r="I975" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J975" t="b">
+        <v>0</v>
+      </c>
+      <c r="K975" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 858.00 &lt;= Upper 928.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D976" t="n">
+        <v>122.37</v>
+      </c>
+      <c r="E976" t="n">
+        <v>131.27</v>
+      </c>
+      <c r="F976" t="n">
+        <v>131.27</v>
+      </c>
+      <c r="G976" t="n">
+        <v>124.57</v>
+      </c>
+      <c r="H976" t="n">
+        <v>126.08</v>
+      </c>
+      <c r="I976" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J976" t="b">
+        <v>0</v>
+      </c>
+      <c r="K976" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.57 &lt;= EMA21 126.08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D977" t="n">
+        <v>1791.6</v>
+      </c>
+      <c r="E977" t="n">
+        <v>1902.27</v>
+      </c>
+      <c r="F977" t="n">
+        <v>1902.27</v>
+      </c>
+      <c r="G977" t="n">
+        <v>1834.01</v>
+      </c>
+      <c r="H977" t="n">
+        <v>1843.99</v>
+      </c>
+      <c r="I977" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J977" t="b">
+        <v>0</v>
+      </c>
+      <c r="K977" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1834.01 &lt;= EMA21 1843.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D978" t="n">
+        <v>1351</v>
+      </c>
+      <c r="E978" t="n">
+        <v>1460.37</v>
+      </c>
+      <c r="F978" t="n">
+        <v>1460.37</v>
+      </c>
+      <c r="G978" t="n">
+        <v>1379.43</v>
+      </c>
+      <c r="H978" t="n">
+        <v>1401.67</v>
+      </c>
+      <c r="I978" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="J978" t="b">
+        <v>0</v>
+      </c>
+      <c r="K978" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1379.43 &lt;= EMA21 1401.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D979" t="n">
+        <v>419.25</v>
+      </c>
+      <c r="E979" t="n">
+        <v>434.04</v>
+      </c>
+      <c r="F979" t="n">
+        <v>434.04</v>
+      </c>
+      <c r="G979" t="n">
+        <v>419.82</v>
+      </c>
+      <c r="H979" t="n">
+        <v>413.61</v>
+      </c>
+      <c r="I979" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J979" t="b">
+        <v>0</v>
+      </c>
+      <c r="K979" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 419.25 &lt;= Upper 434.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D980" t="n">
+        <v>4874</v>
+      </c>
+      <c r="E980" t="n">
+        <v>5394.67</v>
+      </c>
+      <c r="F980" t="n">
+        <v>5394.67</v>
+      </c>
+      <c r="G980" t="n">
+        <v>5067.26</v>
+      </c>
+      <c r="H980" t="n">
+        <v>5157.99</v>
+      </c>
+      <c r="I980" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J980" t="b">
+        <v>0</v>
+      </c>
+      <c r="K980" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5067.26 &lt;= EMA21 5157.99)</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D981" t="n">
+        <v>620.85</v>
+      </c>
+      <c r="E981" t="n">
+        <v>703.41</v>
+      </c>
+      <c r="F981" t="n">
+        <v>703.41</v>
+      </c>
+      <c r="G981" t="n">
+        <v>656.04</v>
+      </c>
+      <c r="H981" t="n">
+        <v>663.26</v>
+      </c>
+      <c r="I981" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J981" t="b">
+        <v>0</v>
+      </c>
+      <c r="K981" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 656.04 &lt;= EMA21 663.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>9198</v>
+      </c>
+      <c r="E982" t="n">
+        <v>9775.790000000001</v>
+      </c>
+      <c r="F982" t="n">
+        <v>9775.790000000001</v>
+      </c>
+      <c r="G982" t="n">
+        <v>9287.99</v>
+      </c>
+      <c r="H982" t="n">
+        <v>9036.110000000001</v>
+      </c>
+      <c r="I982" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J982" t="b">
+        <v>0</v>
+      </c>
+      <c r="K982" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9198.00 &lt;= Upper 9775.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>1145</v>
+      </c>
+      <c r="E983" t="n">
+        <v>1197.73</v>
+      </c>
+      <c r="F983" t="n">
+        <v>1197.73</v>
+      </c>
+      <c r="G983" t="n">
+        <v>1153.66</v>
+      </c>
+      <c r="H983" t="n">
+        <v>1163.96</v>
+      </c>
+      <c r="I983" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="J983" t="b">
+        <v>0</v>
+      </c>
+      <c r="K983" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1153.66 &lt;= EMA21 1163.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>7452.5</v>
+      </c>
+      <c r="E984" t="n">
+        <v>8282.43</v>
+      </c>
+      <c r="F984" t="n">
+        <v>8282.43</v>
+      </c>
+      <c r="G984" t="n">
+        <v>7678.75</v>
+      </c>
+      <c r="H984" t="n">
+        <v>7788.46</v>
+      </c>
+      <c r="I984" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J984" t="b">
+        <v>0</v>
+      </c>
+      <c r="K984" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7678.75 &lt;= EMA21 7788.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>315.25</v>
+      </c>
+      <c r="E985" t="n">
+        <v>333.37</v>
+      </c>
+      <c r="F985" t="n">
+        <v>333.37</v>
+      </c>
+      <c r="G985" t="n">
+        <v>321.9</v>
+      </c>
+      <c r="H985" t="n">
+        <v>320.82</v>
+      </c>
+      <c r="I985" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J985" t="b">
+        <v>0</v>
+      </c>
+      <c r="K985" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 315.25 &lt;= Upper 333.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>170.88</v>
+      </c>
+      <c r="E986" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="F986" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="G986" t="n">
+        <v>173.56</v>
+      </c>
+      <c r="H986" t="n">
+        <v>173.66</v>
+      </c>
+      <c r="I986" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J986" t="b">
+        <v>0</v>
+      </c>
+      <c r="K986" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 173.56 &lt;= EMA21 173.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>857</v>
+      </c>
+      <c r="E987" t="n">
+        <v>960.4400000000001</v>
+      </c>
+      <c r="F987" t="n">
+        <v>960.4400000000001</v>
+      </c>
+      <c r="G987" t="n">
+        <v>873.98</v>
+      </c>
+      <c r="H987" t="n">
+        <v>904.84</v>
+      </c>
+      <c r="I987" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J987" t="b">
+        <v>0</v>
+      </c>
+      <c r="K987" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 873.98 &lt;= EMA21 904.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D988" t="n">
+        <v>3171</v>
+      </c>
+      <c r="E988" t="n">
+        <v>3366.54</v>
+      </c>
+      <c r="F988" t="n">
+        <v>3366.54</v>
+      </c>
+      <c r="G988" t="n">
+        <v>3276.18</v>
+      </c>
+      <c r="H988" t="n">
+        <v>3276.09</v>
+      </c>
+      <c r="I988" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J988" t="b">
+        <v>0</v>
+      </c>
+      <c r="K988" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 3171.00 &lt;= Upper 3366.54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D989" t="n">
+        <v>1253.7</v>
+      </c>
+      <c r="E989" t="n">
+        <v>1372.34</v>
+      </c>
+      <c r="F989" t="n">
+        <v>1372.34</v>
+      </c>
+      <c r="G989" t="n">
+        <v>1257.81</v>
+      </c>
+      <c r="H989" t="n">
+        <v>1281.96</v>
+      </c>
+      <c r="I989" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J989" t="b">
+        <v>0</v>
+      </c>
+      <c r="K989" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1257.81 &lt;= EMA21 1281.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D990" t="n">
+        <v>2409</v>
+      </c>
+      <c r="E990" t="n">
+        <v>2710.8</v>
+      </c>
+      <c r="F990" t="n">
+        <v>2710.8</v>
+      </c>
+      <c r="G990" t="n">
+        <v>2461.59</v>
+      </c>
+      <c r="H990" t="n">
+        <v>2510.16</v>
+      </c>
+      <c r="I990" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J990" t="b">
+        <v>0</v>
+      </c>
+      <c r="K990" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2461.59 &lt;= EMA21 2510.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D991" t="n">
+        <v>716.55</v>
+      </c>
+      <c r="E991" t="n">
+        <v>736.87</v>
+      </c>
+      <c r="F991" t="n">
+        <v>736.87</v>
+      </c>
+      <c r="G991" t="n">
+        <v>706.92</v>
+      </c>
+      <c r="H991" t="n">
+        <v>714.66</v>
+      </c>
+      <c r="I991" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="J991" t="b">
+        <v>0</v>
+      </c>
+      <c r="K991" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 706.92 &lt;= EMA21 714.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D992" t="n">
+        <v>516.1</v>
+      </c>
+      <c r="E992" t="n">
+        <v>561.3</v>
+      </c>
+      <c r="F992" t="n">
+        <v>561.3</v>
+      </c>
+      <c r="G992" t="n">
+        <v>528.76</v>
+      </c>
+      <c r="H992" t="n">
+        <v>535.83</v>
+      </c>
+      <c r="I992" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J992" t="b">
+        <v>0</v>
+      </c>
+      <c r="K992" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 528.76 &lt;= EMA21 535.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D993" t="n">
+        <v>958.7</v>
+      </c>
+      <c r="E993" t="n">
+        <v>1072.46</v>
+      </c>
+      <c r="F993" t="n">
+        <v>1072.46</v>
+      </c>
+      <c r="G993" t="n">
+        <v>1000.92</v>
+      </c>
+      <c r="H993" t="n">
+        <v>1012.52</v>
+      </c>
+      <c r="I993" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J993" t="b">
+        <v>0</v>
+      </c>
+      <c r="K993" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1000.92 &lt;= EMA21 1012.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D994" t="n">
+        <v>4695</v>
+      </c>
+      <c r="E994" t="n">
+        <v>5126.73</v>
+      </c>
+      <c r="F994" t="n">
+        <v>5126.73</v>
+      </c>
+      <c r="G994" t="n">
+        <v>4868.02</v>
+      </c>
+      <c r="H994" t="n">
+        <v>4864</v>
+      </c>
+      <c r="I994" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J994" t="b">
+        <v>0</v>
+      </c>
+      <c r="K994" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 4695.00 &lt;= Upper 5126.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D995" t="n">
+        <v>1938.1</v>
+      </c>
+      <c r="E995" t="n">
+        <v>2067.37</v>
+      </c>
+      <c r="F995" t="n">
+        <v>2067.37</v>
+      </c>
+      <c r="G995" t="n">
+        <v>1958.27</v>
+      </c>
+      <c r="H995" t="n">
+        <v>1993.45</v>
+      </c>
+      <c r="I995" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J995" t="b">
+        <v>0</v>
+      </c>
+      <c r="K995" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1958.27 &lt;= EMA21 1993.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D996" t="n">
+        <v>560.9</v>
+      </c>
+      <c r="E996" t="n">
+        <v>629.42</v>
+      </c>
+      <c r="F996" t="n">
+        <v>629.42</v>
+      </c>
+      <c r="G996" t="n">
+        <v>586.09</v>
+      </c>
+      <c r="H996" t="n">
+        <v>586.5</v>
+      </c>
+      <c r="I996" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J996" t="b">
+        <v>0</v>
+      </c>
+      <c r="K996" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 586.09 &lt;= EMA21 586.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D997" t="n">
+        <v>2140</v>
+      </c>
+      <c r="E997" t="n">
+        <v>2271.28</v>
+      </c>
+      <c r="F997" t="n">
+        <v>2271.28</v>
+      </c>
+      <c r="G997" t="n">
+        <v>2184.03</v>
+      </c>
+      <c r="H997" t="n">
+        <v>2184.25</v>
+      </c>
+      <c r="I997" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J997" t="b">
+        <v>0</v>
+      </c>
+      <c r="K997" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2184.03 &lt;= EMA21 2184.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D998" t="n">
+        <v>1350.4</v>
+      </c>
+      <c r="E998" t="n">
+        <v>1462.73</v>
+      </c>
+      <c r="F998" t="n">
+        <v>1462.73</v>
+      </c>
+      <c r="G998" t="n">
+        <v>1393.07</v>
+      </c>
+      <c r="H998" t="n">
+        <v>1408.19</v>
+      </c>
+      <c r="I998" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J998" t="b">
+        <v>0</v>
+      </c>
+      <c r="K998" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1393.07 &lt;= EMA21 1408.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D999" t="n">
+        <v>258</v>
+      </c>
+      <c r="E999" t="n">
+        <v>274.74</v>
+      </c>
+      <c r="F999" t="n">
+        <v>274.74</v>
+      </c>
+      <c r="G999" t="n">
+        <v>261.61</v>
+      </c>
+      <c r="H999" t="n">
+        <v>266.02</v>
+      </c>
+      <c r="I999" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J999" t="b">
+        <v>0</v>
+      </c>
+      <c r="K999" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 261.61 &lt;= EMA21 266.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D1000" t="n">
+        <v>715</v>
+      </c>
+      <c r="E1000" t="n">
+        <v>738.5</v>
+      </c>
+      <c r="F1000" t="n">
+        <v>738.5</v>
+      </c>
+      <c r="G1000" t="n">
+        <v>719.46</v>
+      </c>
+      <c r="H1000" t="n">
+        <v>722.38</v>
+      </c>
+      <c r="I1000" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="J1000" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1000" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 719.46 &lt;= EMA21 722.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D1001" t="n">
+        <v>132.03</v>
+      </c>
+      <c r="E1001" t="n">
+        <v>140.32</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>140.32</v>
+      </c>
+      <c r="G1001" t="n">
+        <v>135.14</v>
+      </c>
+      <c r="H1001" t="n">
+        <v>136.56</v>
+      </c>
+      <c r="I1001" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J1001" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1001" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.14 &lt;= EMA21 136.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D1002" t="n">
+        <v>79.15000000000001</v>
+      </c>
+      <c r="E1002" t="n">
+        <v>88.25</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>88.25</v>
+      </c>
+      <c r="G1002" t="n">
+        <v>81.69</v>
+      </c>
+      <c r="H1002" t="n">
+        <v>83.61</v>
+      </c>
+      <c r="I1002" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1002" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1002" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 81.69 &lt;= EMA21 83.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1003" t="n">
+        <v>1077</v>
+      </c>
+      <c r="E1003" t="n">
+        <v>1183.66</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>1183.66</v>
+      </c>
+      <c r="G1003" t="n">
+        <v>1077.58</v>
+      </c>
+      <c r="H1003" t="n">
+        <v>1101.57</v>
+      </c>
+      <c r="I1003" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J1003" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1003" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1077.58 &lt;= EMA21 1101.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D1004" t="n">
+        <v>4776</v>
+      </c>
+      <c r="E1004" t="n">
+        <v>5356.4</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>5356.4</v>
+      </c>
+      <c r="G1004" t="n">
+        <v>4969.1</v>
+      </c>
+      <c r="H1004" t="n">
+        <v>5067.27</v>
+      </c>
+      <c r="I1004" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J1004" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1004" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4969.10 &lt;= EMA21 5067.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D1005" t="n">
+        <v>1229.2</v>
+      </c>
+      <c r="E1005" t="n">
+        <v>1357.63</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>1357.63</v>
+      </c>
+      <c r="G1005" t="n">
+        <v>1285.59</v>
+      </c>
+      <c r="H1005" t="n">
+        <v>1294.09</v>
+      </c>
+      <c r="I1005" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1005" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1005" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1285.59 &lt;= EMA21 1294.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D1006" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E1006" t="n">
+        <v>1197.55</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>1197.55</v>
+      </c>
+      <c r="G1006" t="n">
+        <v>1133.7</v>
+      </c>
+      <c r="H1006" t="n">
+        <v>1133.67</v>
+      </c>
+      <c r="I1006" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1006" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1006" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1095.00 &lt;= Upper 1197.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D1007" t="n">
+        <v>225.6</v>
+      </c>
+      <c r="E1007" t="n">
+        <v>250.88</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>250.88</v>
+      </c>
+      <c r="G1007" t="n">
+        <v>232.65</v>
+      </c>
+      <c r="H1007" t="n">
+        <v>237.68</v>
+      </c>
+      <c r="I1007" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J1007" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1007" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 232.65 &lt;= EMA21 237.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D1008" t="n">
+        <v>409.8</v>
+      </c>
+      <c r="E1008" t="n">
+        <v>436.85</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>436.85</v>
+      </c>
+      <c r="G1008" t="n">
+        <v>416.42</v>
+      </c>
+      <c r="H1008" t="n">
+        <v>412.26</v>
+      </c>
+      <c r="I1008" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J1008" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1008" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 409.80 &lt;= Upper 436.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D1009" t="n">
+        <v>4346.6</v>
+      </c>
+      <c r="E1009" t="n">
+        <v>4694.79</v>
+      </c>
+      <c r="F1009" t="n">
+        <v>4694.79</v>
+      </c>
+      <c r="G1009" t="n">
+        <v>4416.68</v>
+      </c>
+      <c r="H1009" t="n">
+        <v>4466.89</v>
+      </c>
+      <c r="I1009" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J1009" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1009" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4416.68 &lt;= EMA21 4466.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D1010" t="n">
+        <v>3850.7</v>
+      </c>
+      <c r="E1010" t="n">
+        <v>4144.46</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>4144.46</v>
+      </c>
+      <c r="G1010" t="n">
+        <v>3942.73</v>
+      </c>
+      <c r="H1010" t="n">
+        <v>3978.6</v>
+      </c>
+      <c r="I1010" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="J1010" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1010" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3942.73 &lt;= EMA21 3978.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D1011" t="n">
+        <v>1064.8</v>
+      </c>
+      <c r="E1011" t="n">
+        <v>1320.19</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>1320.19</v>
+      </c>
+      <c r="G1011" t="n">
+        <v>1161.56</v>
+      </c>
+      <c r="H1011" t="n">
+        <v>1192.38</v>
+      </c>
+      <c r="I1011" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1011" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1011" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1161.56 &lt;= EMA21 1192.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D1012" t="n">
+        <v>3029.5</v>
+      </c>
+      <c r="E1012" t="n">
+        <v>3535.62</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>3535.62</v>
+      </c>
+      <c r="G1012" t="n">
+        <v>3145.61</v>
+      </c>
+      <c r="H1012" t="n">
+        <v>3225.28</v>
+      </c>
+      <c r="I1012" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J1012" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1012" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3145.61 &lt;= EMA21 3225.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D1013" t="n">
+        <v>12231</v>
+      </c>
+      <c r="E1013" t="n">
+        <v>14146.95</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>14146.95</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>12646.84</v>
+      </c>
+      <c r="H1013" t="n">
+        <v>13016.04</v>
+      </c>
+      <c r="I1013" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1013" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1013" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12646.84 &lt;= EMA21 13016.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D1014" t="n">
+        <v>1030</v>
+      </c>
+      <c r="E1014" t="n">
+        <v>1046.18</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>1046.18</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>1021.1</v>
+      </c>
+      <c r="H1014" t="n">
+        <v>1022.38</v>
+      </c>
+      <c r="I1014" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J1014" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1014" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1021.10 &lt;= EMA21 1022.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D1015" t="n">
+        <v>2236</v>
+      </c>
+      <c r="E1015" t="n">
+        <v>2694.69</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>2694.69</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>2396.29</v>
+      </c>
+      <c r="H1015" t="n">
+        <v>2451.38</v>
+      </c>
+      <c r="I1015" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1015" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1015" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2396.29 &lt;= EMA21 2451.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D1016" t="n">
+        <v>2722.3</v>
+      </c>
+      <c r="E1016" t="n">
+        <v>3236.24</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>3236.24</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>2849.37</v>
+      </c>
+      <c r="H1016" t="n">
+        <v>2912.33</v>
+      </c>
+      <c r="I1016" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J1016" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1016" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2849.37 &lt;= EMA21 2912.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D1017" t="n">
+        <v>329.5</v>
+      </c>
+      <c r="E1017" t="n">
+        <v>339</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>339</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>331.79</v>
+      </c>
+      <c r="H1017" t="n">
+        <v>332.81</v>
+      </c>
+      <c r="I1017" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1017" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1017" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 331.79 &lt;= EMA21 332.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D1018" t="n">
+        <v>1362</v>
+      </c>
+      <c r="E1018" t="n">
+        <v>1510.18</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>1510.18</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>1397.97</v>
+      </c>
+      <c r="H1018" t="n">
+        <v>1426.96</v>
+      </c>
+      <c r="I1018" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1018" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1018" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1397.97 &lt;= EMA21 1426.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D1019" t="n">
+        <v>235.95</v>
+      </c>
+      <c r="E1019" t="n">
+        <v>239.29</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>239.29</v>
+      </c>
+      <c r="G1019" t="n">
+        <v>234.82</v>
+      </c>
+      <c r="H1019" t="n">
+        <v>235.42</v>
+      </c>
+      <c r="I1019" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1019" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1019" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.82 &lt;= EMA21 235.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D1020" t="n">
+        <v>1521.1</v>
+      </c>
+      <c r="E1020" t="n">
+        <v>1713.39</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>1713.39</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>1581.82</v>
+      </c>
+      <c r="H1020" t="n">
+        <v>1610.77</v>
+      </c>
+      <c r="I1020" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1020" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1581.82 &lt;= EMA21 1610.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D1021" t="n">
+        <v>344</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>371.65</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>371.65</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>351.16</v>
+      </c>
+      <c r="H1021" t="n">
+        <v>358.66</v>
+      </c>
+      <c r="I1021" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1021" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1021" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 351.16 &lt;= EMA21 358.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D1022" t="n">
+        <v>262.8</v>
+      </c>
+      <c r="E1022" t="n">
+        <v>272.55</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>272.55</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>266.63</v>
+      </c>
+      <c r="H1022" t="n">
+        <v>268.22</v>
+      </c>
+      <c r="I1022" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1022" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1022" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.63 &lt;= EMA21 268.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D1023" t="n">
+        <v>114.7</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>118.03</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>118.03</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>115.95</v>
+      </c>
+      <c r="H1023" t="n">
+        <v>115.66</v>
+      </c>
+      <c r="I1023" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="J1023" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1023" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 114.70 &lt;= Upper 118.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D1024" t="n">
+        <v>308.5</v>
+      </c>
+      <c r="E1024" t="n">
+        <v>336.72</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>336.72</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>314.81</v>
+      </c>
+      <c r="H1024" t="n">
+        <v>322.42</v>
+      </c>
+      <c r="I1024" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1024" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 314.81 &lt;= EMA21 322.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D1025" t="n">
+        <v>1235.3</v>
+      </c>
+      <c r="E1025" t="n">
+        <v>1342.75</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>1342.75</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>1276.59</v>
+      </c>
+      <c r="H1025" t="n">
+        <v>1290.83</v>
+      </c>
+      <c r="I1025" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1025" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1025" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1276.59 &lt;= EMA21 1290.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D1026" t="n">
+        <v>1654.1</v>
+      </c>
+      <c r="E1026" t="n">
+        <v>1819.2</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>1819.2</v>
+      </c>
+      <c r="G1026" t="n">
+        <v>1702.39</v>
+      </c>
+      <c r="H1026" t="n">
+        <v>1738.53</v>
+      </c>
+      <c r="I1026" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1026" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1026" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1702.39 &lt;= EMA21 1738.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D1027" t="n">
+        <v>158.15</v>
+      </c>
+      <c r="E1027" t="n">
+        <v>172.54</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>172.54</v>
+      </c>
+      <c r="G1027" t="n">
+        <v>162.76</v>
+      </c>
+      <c r="H1027" t="n">
+        <v>163.13</v>
+      </c>
+      <c r="I1027" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="J1027" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1027" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 162.76 &lt;= EMA21 163.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D1028" t="n">
+        <v>21905</v>
+      </c>
+      <c r="E1028" t="n">
+        <v>25273.48</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>25273.48</v>
+      </c>
+      <c r="G1028" t="n">
+        <v>22969.14</v>
+      </c>
+      <c r="H1028" t="n">
+        <v>23729.05</v>
+      </c>
+      <c r="I1028" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J1028" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1028" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 22969.14 &lt;= EMA21 23729.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D1029" t="n">
+        <v>979.8</v>
+      </c>
+      <c r="E1029" t="n">
+        <v>1164.66</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>1164.66</v>
+      </c>
+      <c r="G1029" t="n">
+        <v>1032.27</v>
+      </c>
+      <c r="H1029" t="n">
+        <v>1057.89</v>
+      </c>
+      <c r="I1029" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J1029" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1029" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1032.27 &lt;= EMA21 1057.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D1030" t="n">
+        <v>3028.7</v>
+      </c>
+      <c r="E1030" t="n">
+        <v>3574.07</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>3574.07</v>
+      </c>
+      <c r="G1030" t="n">
+        <v>3158.86</v>
+      </c>
+      <c r="H1030" t="n">
+        <v>3238.73</v>
+      </c>
+      <c r="I1030" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1030" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1030" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3158.86 &lt;= EMA21 3238.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D1031" t="n">
+        <v>3770</v>
+      </c>
+      <c r="E1031" t="n">
+        <v>4154.86</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>4154.86</v>
+      </c>
+      <c r="G1031" t="n">
+        <v>3932.15</v>
+      </c>
+      <c r="H1031" t="n">
+        <v>3947.42</v>
+      </c>
+      <c r="I1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1031" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1031" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3932.15 &lt;= EMA21 3947.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D1032" t="n">
+        <v>19250</v>
+      </c>
+      <c r="E1032" t="n">
+        <v>22858.28</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>22858.28</v>
+      </c>
+      <c r="G1032" t="n">
+        <v>21256.69</v>
+      </c>
+      <c r="H1032" t="n">
+        <v>20754.02</v>
+      </c>
+      <c r="I1032" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="J1032" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1032" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 19250.00 &lt;= Upper 22858.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D1033" t="n">
+        <v>968</v>
+      </c>
+      <c r="E1033" t="n">
+        <v>1077.72</v>
+      </c>
+      <c r="F1033" t="n">
+        <v>1077.72</v>
+      </c>
+      <c r="G1033" t="n">
+        <v>1004.25</v>
+      </c>
+      <c r="H1033" t="n">
+        <v>1022.24</v>
+      </c>
+      <c r="I1033" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J1033" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1033" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1004.25 &lt;= EMA21 1022.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D1034" t="n">
+        <v>1835</v>
+      </c>
+      <c r="E1034" t="n">
+        <v>1967.32</v>
+      </c>
+      <c r="F1034" t="n">
+        <v>1967.32</v>
+      </c>
+      <c r="G1034" t="n">
+        <v>1872.72</v>
+      </c>
+      <c r="H1034" t="n">
+        <v>1895.92</v>
+      </c>
+      <c r="I1034" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J1034" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1034" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1872.72 &lt;= EMA21 1895.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D1035" t="n">
+        <v>4050</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>4519.83</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>4519.83</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>4147.92</v>
+      </c>
+      <c r="H1035" t="n">
+        <v>4200.88</v>
+      </c>
+      <c r="I1035" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J1035" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1035" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4147.92 &lt;= EMA21 4200.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D1036" t="n">
+        <v>353.35</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>377.64</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>377.64</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>363.79</v>
+      </c>
+      <c r="H1036" t="n">
+        <v>365.28</v>
+      </c>
+      <c r="I1036" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J1036" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1036" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.79 &lt;= EMA21 365.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D1037" t="n">
+        <v>2251</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>2392.46</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>2392.46</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>2253.95</v>
+      </c>
+      <c r="H1037" t="n">
+        <v>2283.46</v>
+      </c>
+      <c r="I1037" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="J1037" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1037" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2253.95 &lt;= EMA21 2283.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D1038" t="n">
+        <v>986.1</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>1081.73</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>1081.73</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>1006</v>
+      </c>
+      <c r="H1038" t="n">
+        <v>1028</v>
+      </c>
+      <c r="I1038" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1038" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1038" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1006.00 &lt;= EMA21 1028.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D1039" t="n">
+        <v>427.15</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>493.6</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>493.6</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>445.7</v>
+      </c>
+      <c r="H1039" t="n">
+        <v>452.65</v>
+      </c>
+      <c r="I1039" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J1039" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1039" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 445.70 &lt;= EMA21 452.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D1040" t="n">
+        <v>303.6</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>325.27</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>325.27</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>305.97</v>
+      </c>
+      <c r="H1040" t="n">
+        <v>313.39</v>
+      </c>
+      <c r="I1040" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J1040" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 305.97 &lt;= EMA21 313.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D1041" t="n">
+        <v>363</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>384.3</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>384.3</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>364.85</v>
+      </c>
+      <c r="H1041" t="n">
+        <v>366.97</v>
+      </c>
+      <c r="I1041" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1041" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 364.85 &lt;= EMA21 366.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D1042" t="n">
+        <v>183.65</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>189.12</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>189.12</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>185.19</v>
+      </c>
+      <c r="H1042" t="n">
+        <v>185.69</v>
+      </c>
+      <c r="I1042" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1042" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.19 &lt;= EMA21 185.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D1043" t="n">
+        <v>1575.9</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>1653.87</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>1653.87</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>1563.46</v>
+      </c>
+      <c r="H1043" t="n">
+        <v>1579.34</v>
+      </c>
+      <c r="I1043" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J1043" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1563.46 &lt;= EMA21 1579.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D1044" t="n">
+        <v>4856</v>
+      </c>
+      <c r="E1044" t="n">
+        <v>5186.76</v>
+      </c>
+      <c r="F1044" t="n">
+        <v>5186.76</v>
+      </c>
+      <c r="G1044" t="n">
+        <v>4991.84</v>
+      </c>
+      <c r="H1044" t="n">
+        <v>5007.34</v>
+      </c>
+      <c r="I1044" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1044" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1044" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4991.84 &lt;= EMA21 5007.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D1045" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>5072.41</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>5072.41</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>4925.48</v>
+      </c>
+      <c r="H1045" t="n">
+        <v>4935.53</v>
+      </c>
+      <c r="I1045" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J1045" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1045" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4925.48 &lt;= EMA21 4935.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D1046" t="n">
+        <v>2730</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>2992.08</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>2992.08</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>2810.12</v>
+      </c>
+      <c r="H1046" t="n">
+        <v>2860.59</v>
+      </c>
+      <c r="I1046" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1046" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1046" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2810.12 &lt;= EMA21 2860.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D1047" t="n">
+        <v>10697</v>
+      </c>
+      <c r="E1047" t="n">
+        <v>11918.3</v>
+      </c>
+      <c r="F1047" t="n">
+        <v>11918.3</v>
+      </c>
+      <c r="G1047" t="n">
+        <v>11059.49</v>
+      </c>
+      <c r="H1047" t="n">
+        <v>11289.67</v>
+      </c>
+      <c r="I1047" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J1047" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1047" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11059.49 &lt;= EMA21 11289.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D1048" t="n">
+        <v>175</v>
+      </c>
+      <c r="E1048" t="n">
+        <v>191.67</v>
+      </c>
+      <c r="F1048" t="n">
+        <v>191.67</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>181.41</v>
+      </c>
+      <c r="H1048" t="n">
+        <v>182.6</v>
+      </c>
+      <c r="I1048" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1048" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1048" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 181.41 &lt;= EMA21 182.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D1049" t="n">
+        <v>1370.6</v>
+      </c>
+      <c r="E1049" t="n">
+        <v>1599.82</v>
+      </c>
+      <c r="F1049" t="n">
+        <v>1599.82</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>1424.67</v>
+      </c>
+      <c r="H1049" t="n">
+        <v>1460.01</v>
+      </c>
+      <c r="I1049" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J1049" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1049" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1424.67 &lt;= EMA21 1460.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D1050" t="n">
+        <v>409.6</v>
+      </c>
+      <c r="E1050" t="n">
+        <v>442.52</v>
+      </c>
+      <c r="F1050" t="n">
+        <v>442.52</v>
+      </c>
+      <c r="G1050" t="n">
+        <v>411.13</v>
+      </c>
+      <c r="H1050" t="n">
+        <v>418.48</v>
+      </c>
+      <c r="I1050" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J1050" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1050" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 411.13 &lt;= EMA21 418.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D1051" t="n">
+        <v>257</v>
+      </c>
+      <c r="E1051" t="n">
+        <v>288.06</v>
+      </c>
+      <c r="F1051" t="n">
+        <v>288.06</v>
+      </c>
+      <c r="G1051" t="n">
+        <v>267.75</v>
+      </c>
+      <c r="H1051" t="n">
+        <v>270.84</v>
+      </c>
+      <c r="I1051" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1051" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1051" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 267.75 &lt;= EMA21 270.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D1052" t="n">
+        <v>170</v>
+      </c>
+      <c r="E1052" t="n">
+        <v>187.12</v>
+      </c>
+      <c r="F1052" t="n">
+        <v>187.12</v>
+      </c>
+      <c r="G1052" t="n">
+        <v>171.4</v>
+      </c>
+      <c r="H1052" t="n">
+        <v>175.15</v>
+      </c>
+      <c r="I1052" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J1052" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1052" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 171.40 &lt;= EMA21 175.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D1053" t="n">
+        <v>1099</v>
+      </c>
+      <c r="E1053" t="n">
+        <v>1191.28</v>
+      </c>
+      <c r="F1053" t="n">
+        <v>1191.28</v>
+      </c>
+      <c r="G1053" t="n">
+        <v>1127.51</v>
+      </c>
+      <c r="H1053" t="n">
+        <v>1134.52</v>
+      </c>
+      <c r="I1053" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J1053" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1053" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1127.51 &lt;= EMA21 1134.52)</t>
         </is>
       </c>
     </row>
@@ -41719,7 +46019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41800,10 +46100,10 @@
         <v>19685.95</v>
       </c>
       <c r="F2" t="n">
-        <v>426.4</v>
+        <v>419.25</v>
       </c>
       <c r="G2" t="n">
-        <v>1.8</v>
+        <v>0.1</v>
       </c>
       <c r="H2" t="n">
         <v>416.67</v>
@@ -41812,7 +46112,7 @@
         <v>436.2999877929688</v>
       </c>
       <c r="J2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -41841,62 +46141,21 @@
         <v>19525</v>
       </c>
       <c r="F3" t="n">
-        <v>1764.6</v>
+        <v>1713.8</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.59</v>
+        <v>-3.45</v>
       </c>
       <c r="H3" t="n">
-        <v>1699.9</v>
+        <v>1710.79</v>
       </c>
       <c r="I3" t="n">
-        <v>1780</v>
+        <v>1791.400024414062</v>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K3" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ADANIPOWER</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>214.9</v>
-      </c>
-      <c r="D4" t="n">
-        <v>93</v>
-      </c>
-      <c r="E4" t="n">
-        <v>19985.7</v>
-      </c>
-      <c r="F4" t="n">
-        <v>209.97</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-2.29</v>
-      </c>
-      <c r="H4" t="n">
-        <v>205.59</v>
-      </c>
-      <c r="I4" t="n">
-        <v>215.2799987792969</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -41913,7 +46172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42845,6 +47104,57 @@
         <v>2</v>
       </c>
       <c r="M19" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>214.9</v>
+      </c>
+      <c r="E20" t="n">
+        <v>205.59</v>
+      </c>
+      <c r="F20" t="n">
+        <v>93</v>
+      </c>
+      <c r="G20" t="n">
+        <v>19985.7</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-4.332</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-4.632</v>
+      </c>
+      <c r="J20" t="n">
+        <v>-925.74</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>4</v>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -42861,7 +47171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K148"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48145,6 +52455,55 @@
         </is>
       </c>
       <c r="K148" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-15 20:31:29</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>3BD88DF392</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>205.59</v>
+      </c>
+      <c r="G149" t="n">
+        <v>205.59</v>
+      </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" t="n">
+        <v>93</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
         <is>
           <t>HARD_STOP_LOSS</t>
         </is>
@@ -48229,7 +52588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48708,6 +53067,39 @@
         <v>3</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20:31:29</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>157832.24</v>
+      </c>
+      <c r="D15" t="n">
+        <v>39210.95</v>
+      </c>
+      <c r="E15" t="n">
+        <v>197043.19</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-2871.17</v>
+      </c>
+      <c r="G15" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-16T20:29 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1053"/>
+  <dimension ref="A1:K1153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45706,6 +45706,4306 @@
       <c r="K1053" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1127.51 &lt;= EMA21 1134.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D1054" t="n">
+        <v>6980</v>
+      </c>
+      <c r="E1054" t="n">
+        <v>7746.69</v>
+      </c>
+      <c r="F1054" t="n">
+        <v>7746.69</v>
+      </c>
+      <c r="G1054" t="n">
+        <v>7233.49</v>
+      </c>
+      <c r="H1054" t="n">
+        <v>7349.25</v>
+      </c>
+      <c r="I1054" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1054" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1054" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7233.49 &lt;= EMA21 7349.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D1055" t="n">
+        <v>1349.2</v>
+      </c>
+      <c r="E1055" t="n">
+        <v>1639.67</v>
+      </c>
+      <c r="F1055" t="n">
+        <v>1639.67</v>
+      </c>
+      <c r="G1055" t="n">
+        <v>1385.99</v>
+      </c>
+      <c r="H1055" t="n">
+        <v>1444.92</v>
+      </c>
+      <c r="I1055" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J1055" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1055" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1385.99 &lt;= EMA21 1444.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D1056" t="n">
+        <v>2920</v>
+      </c>
+      <c r="E1056" t="n">
+        <v>3200.5</v>
+      </c>
+      <c r="F1056" t="n">
+        <v>3200.5</v>
+      </c>
+      <c r="G1056" t="n">
+        <v>2988.48</v>
+      </c>
+      <c r="H1056" t="n">
+        <v>2999.69</v>
+      </c>
+      <c r="I1056" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="J1056" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1056" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2988.48 &lt;= EMA21 2999.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D1057" t="n">
+        <v>1270.2</v>
+      </c>
+      <c r="E1057" t="n">
+        <v>1346.38</v>
+      </c>
+      <c r="F1057" t="n">
+        <v>1346.38</v>
+      </c>
+      <c r="G1057" t="n">
+        <v>1281.32</v>
+      </c>
+      <c r="H1057" t="n">
+        <v>1299.41</v>
+      </c>
+      <c r="I1057" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J1057" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1057" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1281.32 &lt;= EMA21 1299.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D1058" t="n">
+        <v>1723.8</v>
+      </c>
+      <c r="E1058" t="n">
+        <v>1791.83</v>
+      </c>
+      <c r="F1058" t="n">
+        <v>1791.83</v>
+      </c>
+      <c r="G1058" t="n">
+        <v>1729.52</v>
+      </c>
+      <c r="H1058" t="n">
+        <v>1717.64</v>
+      </c>
+      <c r="I1058" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J1058" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1058" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1723.80 &lt;= Upper 1791.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D1059" t="n">
+        <v>202.34</v>
+      </c>
+      <c r="E1059" t="n">
+        <v>216.27</v>
+      </c>
+      <c r="F1059" t="n">
+        <v>216.27</v>
+      </c>
+      <c r="G1059" t="n">
+        <v>206.95</v>
+      </c>
+      <c r="H1059" t="n">
+        <v>207.71</v>
+      </c>
+      <c r="I1059" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J1059" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1059" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 206.95 &lt;= EMA21 207.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D1060" t="n">
+        <v>381.05</v>
+      </c>
+      <c r="E1060" t="n">
+        <v>422.86</v>
+      </c>
+      <c r="F1060" t="n">
+        <v>422.86</v>
+      </c>
+      <c r="G1060" t="n">
+        <v>391.9</v>
+      </c>
+      <c r="H1060" t="n">
+        <v>401.14</v>
+      </c>
+      <c r="I1060" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J1060" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1060" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 391.90 &lt;= EMA21 401.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D1061" t="n">
+        <v>8696.5</v>
+      </c>
+      <c r="E1061" t="n">
+        <v>8958.790000000001</v>
+      </c>
+      <c r="F1061" t="n">
+        <v>8958.790000000001</v>
+      </c>
+      <c r="G1061" t="n">
+        <v>8783.16</v>
+      </c>
+      <c r="H1061" t="n">
+        <v>8793.030000000001</v>
+      </c>
+      <c r="I1061" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1061" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1061" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8783.16 &lt;= EMA21 8793.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D1062" t="n">
+        <v>2416.6</v>
+      </c>
+      <c r="E1062" t="n">
+        <v>2709.71</v>
+      </c>
+      <c r="F1062" t="n">
+        <v>2709.71</v>
+      </c>
+      <c r="G1062" t="n">
+        <v>2473.39</v>
+      </c>
+      <c r="H1062" t="n">
+        <v>2538.5</v>
+      </c>
+      <c r="I1062" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1062" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1062" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2473.39 &lt;= EMA21 2538.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D1063" t="n">
+        <v>3720</v>
+      </c>
+      <c r="E1063" t="n">
+        <v>3980.64</v>
+      </c>
+      <c r="F1063" t="n">
+        <v>3980.64</v>
+      </c>
+      <c r="G1063" t="n">
+        <v>3723.17</v>
+      </c>
+      <c r="H1063" t="n">
+        <v>3790.76</v>
+      </c>
+      <c r="I1063" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1063" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1063" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3723.17 &lt;= EMA21 3790.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D1064" t="n">
+        <v>1241</v>
+      </c>
+      <c r="E1064" t="n">
+        <v>1284.38</v>
+      </c>
+      <c r="F1064" t="n">
+        <v>1284.38</v>
+      </c>
+      <c r="G1064" t="n">
+        <v>1244.16</v>
+      </c>
+      <c r="H1064" t="n">
+        <v>1248.52</v>
+      </c>
+      <c r="I1064" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J1064" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1064" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1244.16 &lt;= EMA21 1248.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D1065" t="n">
+        <v>11593</v>
+      </c>
+      <c r="E1065" t="n">
+        <v>12245.77</v>
+      </c>
+      <c r="F1065" t="n">
+        <v>12245.77</v>
+      </c>
+      <c r="G1065" t="n">
+        <v>11698.14</v>
+      </c>
+      <c r="H1065" t="n">
+        <v>11726.28</v>
+      </c>
+      <c r="I1065" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J1065" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1065" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11698.14 &lt;= EMA21 11726.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D1066" t="n">
+        <v>1006.2</v>
+      </c>
+      <c r="E1066" t="n">
+        <v>1109.61</v>
+      </c>
+      <c r="F1066" t="n">
+        <v>1109.61</v>
+      </c>
+      <c r="G1066" t="n">
+        <v>1033.14</v>
+      </c>
+      <c r="H1066" t="n">
+        <v>1050.97</v>
+      </c>
+      <c r="I1066" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J1066" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1066" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1033.14 &lt;= EMA21 1050.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D1067" t="n">
+        <v>1837</v>
+      </c>
+      <c r="E1067" t="n">
+        <v>2078.24</v>
+      </c>
+      <c r="F1067" t="n">
+        <v>2078.24</v>
+      </c>
+      <c r="G1067" t="n">
+        <v>1912.52</v>
+      </c>
+      <c r="H1067" t="n">
+        <v>1948.76</v>
+      </c>
+      <c r="I1067" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1067" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1067" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1912.52 &lt;= EMA21 1948.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D1068" t="n">
+        <v>10930</v>
+      </c>
+      <c r="E1068" t="n">
+        <v>11586.43</v>
+      </c>
+      <c r="F1068" t="n">
+        <v>11586.43</v>
+      </c>
+      <c r="G1068" t="n">
+        <v>11083.91</v>
+      </c>
+      <c r="H1068" t="n">
+        <v>11152.31</v>
+      </c>
+      <c r="I1068" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J1068" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1068" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11083.91 &lt;= EMA21 11152.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D1069" t="n">
+        <v>234.98</v>
+      </c>
+      <c r="E1069" t="n">
+        <v>246.23</v>
+      </c>
+      <c r="F1069" t="n">
+        <v>246.23</v>
+      </c>
+      <c r="G1069" t="n">
+        <v>236.63</v>
+      </c>
+      <c r="H1069" t="n">
+        <v>239.27</v>
+      </c>
+      <c r="I1069" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1069" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1069" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 236.63 &lt;= EMA21 239.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D1070" t="n">
+        <v>385.75</v>
+      </c>
+      <c r="E1070" t="n">
+        <v>422.59</v>
+      </c>
+      <c r="F1070" t="n">
+        <v>422.59</v>
+      </c>
+      <c r="G1070" t="n">
+        <v>398.42</v>
+      </c>
+      <c r="H1070" t="n">
+        <v>403.04</v>
+      </c>
+      <c r="I1070" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1070" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1070" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 398.42 &lt;= EMA21 403.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D1071" t="n">
+        <v>303.35</v>
+      </c>
+      <c r="E1071" t="n">
+        <v>326.83</v>
+      </c>
+      <c r="F1071" t="n">
+        <v>326.83</v>
+      </c>
+      <c r="G1071" t="n">
+        <v>305.72</v>
+      </c>
+      <c r="H1071" t="n">
+        <v>309.98</v>
+      </c>
+      <c r="I1071" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1071" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1071" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 305.72 &lt;= EMA21 309.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D1072" t="n">
+        <v>1835</v>
+      </c>
+      <c r="E1072" t="n">
+        <v>1957.41</v>
+      </c>
+      <c r="F1072" t="n">
+        <v>1957.41</v>
+      </c>
+      <c r="G1072" t="n">
+        <v>1840.16</v>
+      </c>
+      <c r="H1072" t="n">
+        <v>1864.12</v>
+      </c>
+      <c r="I1072" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="J1072" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1072" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1840.16 &lt;= EMA21 1864.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D1073" t="n">
+        <v>47555</v>
+      </c>
+      <c r="E1073" t="n">
+        <v>49900.7</v>
+      </c>
+      <c r="F1073" t="n">
+        <v>49900.7</v>
+      </c>
+      <c r="G1073" t="n">
+        <v>47988.02</v>
+      </c>
+      <c r="H1073" t="n">
+        <v>47529.96</v>
+      </c>
+      <c r="I1073" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1073" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1073" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47555.00 &lt;= Upper 49900.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D1074" t="n">
+        <v>4999.5</v>
+      </c>
+      <c r="E1074" t="n">
+        <v>5539.91</v>
+      </c>
+      <c r="F1074" t="n">
+        <v>5539.91</v>
+      </c>
+      <c r="G1074" t="n">
+        <v>5048.18</v>
+      </c>
+      <c r="H1074" t="n">
+        <v>5166.43</v>
+      </c>
+      <c r="I1074" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1074" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1074" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5048.18 &lt;= EMA21 5166.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D1075" t="n">
+        <v>851.55</v>
+      </c>
+      <c r="E1075" t="n">
+        <v>931.13</v>
+      </c>
+      <c r="F1075" t="n">
+        <v>931.13</v>
+      </c>
+      <c r="G1075" t="n">
+        <v>887.03</v>
+      </c>
+      <c r="H1075" t="n">
+        <v>889.53</v>
+      </c>
+      <c r="I1075" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1075" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1075" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 887.03 &lt;= EMA21 889.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D1076" t="n">
+        <v>123.2</v>
+      </c>
+      <c r="E1076" t="n">
+        <v>130.76</v>
+      </c>
+      <c r="F1076" t="n">
+        <v>130.76</v>
+      </c>
+      <c r="G1076" t="n">
+        <v>124.16</v>
+      </c>
+      <c r="H1076" t="n">
+        <v>125.64</v>
+      </c>
+      <c r="I1076" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J1076" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1076" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.16 &lt;= EMA21 125.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D1077" t="n">
+        <v>1765.6</v>
+      </c>
+      <c r="E1077" t="n">
+        <v>1905.07</v>
+      </c>
+      <c r="F1077" t="n">
+        <v>1905.07</v>
+      </c>
+      <c r="G1077" t="n">
+        <v>1820.49</v>
+      </c>
+      <c r="H1077" t="n">
+        <v>1836.62</v>
+      </c>
+      <c r="I1077" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J1077" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1077" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1820.49 &lt;= EMA21 1836.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D1078" t="n">
+        <v>1358</v>
+      </c>
+      <c r="E1078" t="n">
+        <v>1456.66</v>
+      </c>
+      <c r="F1078" t="n">
+        <v>1456.66</v>
+      </c>
+      <c r="G1078" t="n">
+        <v>1372.52</v>
+      </c>
+      <c r="H1078" t="n">
+        <v>1394.64</v>
+      </c>
+      <c r="I1078" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1078" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1078" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1372.52 &lt;= EMA21 1394.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D1079" t="n">
+        <v>422.25</v>
+      </c>
+      <c r="E1079" t="n">
+        <v>437.27</v>
+      </c>
+      <c r="F1079" t="n">
+        <v>437.27</v>
+      </c>
+      <c r="G1079" t="n">
+        <v>421.13</v>
+      </c>
+      <c r="H1079" t="n">
+        <v>415.4</v>
+      </c>
+      <c r="I1079" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J1079" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1079" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 422.25 &lt;= Upper 437.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D1080" t="n">
+        <v>4940</v>
+      </c>
+      <c r="E1080" t="n">
+        <v>5343.46</v>
+      </c>
+      <c r="F1080" t="n">
+        <v>5343.46</v>
+      </c>
+      <c r="G1080" t="n">
+        <v>5041.8</v>
+      </c>
+      <c r="H1080" t="n">
+        <v>5138.17</v>
+      </c>
+      <c r="I1080" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1080" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1080" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5041.80 &lt;= EMA21 5138.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D1081" t="n">
+        <v>622.8</v>
+      </c>
+      <c r="E1081" t="n">
+        <v>707.8</v>
+      </c>
+      <c r="F1081" t="n">
+        <v>707.8</v>
+      </c>
+      <c r="G1081" t="n">
+        <v>646.79</v>
+      </c>
+      <c r="H1081" t="n">
+        <v>657.85</v>
+      </c>
+      <c r="I1081" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J1081" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1081" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 646.79 &lt;= EMA21 657.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D1082" t="n">
+        <v>9158</v>
+      </c>
+      <c r="E1082" t="n">
+        <v>9761.219999999999</v>
+      </c>
+      <c r="F1082" t="n">
+        <v>9761.219999999999</v>
+      </c>
+      <c r="G1082" t="n">
+        <v>9263.469999999999</v>
+      </c>
+      <c r="H1082" t="n">
+        <v>9069.889999999999</v>
+      </c>
+      <c r="I1082" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J1082" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1082" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9158.00 &lt;= Upper 9761.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D1083" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E1083" t="n">
+        <v>1196.65</v>
+      </c>
+      <c r="F1083" t="n">
+        <v>1196.65</v>
+      </c>
+      <c r="G1083" t="n">
+        <v>1152.17</v>
+      </c>
+      <c r="H1083" t="n">
+        <v>1161.76</v>
+      </c>
+      <c r="I1083" t="n">
+        <v>1</v>
+      </c>
+      <c r="J1083" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1083" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1152.17 &lt;= EMA21 1161.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D1084" t="n">
+        <v>7500</v>
+      </c>
+      <c r="E1084" t="n">
+        <v>8279.129999999999</v>
+      </c>
+      <c r="F1084" t="n">
+        <v>8279.129999999999</v>
+      </c>
+      <c r="G1084" t="n">
+        <v>7643</v>
+      </c>
+      <c r="H1084" t="n">
+        <v>7762.24</v>
+      </c>
+      <c r="I1084" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J1084" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1084" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7643.00 &lt;= EMA21 7762.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D1085" t="n">
+        <v>317</v>
+      </c>
+      <c r="E1085" t="n">
+        <v>333</v>
+      </c>
+      <c r="F1085" t="n">
+        <v>333</v>
+      </c>
+      <c r="G1085" t="n">
+        <v>320.91</v>
+      </c>
+      <c r="H1085" t="n">
+        <v>320.63</v>
+      </c>
+      <c r="I1085" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="J1085" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1085" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 317.00 &lt;= Upper 333.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D1086" t="n">
+        <v>170.65</v>
+      </c>
+      <c r="E1086" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="F1086" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="G1086" t="n">
+        <v>172.9</v>
+      </c>
+      <c r="H1086" t="n">
+        <v>173.36</v>
+      </c>
+      <c r="I1086" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J1086" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1086" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 172.90 &lt;= EMA21 173.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D1087" t="n">
+        <v>863</v>
+      </c>
+      <c r="E1087" t="n">
+        <v>953.8</v>
+      </c>
+      <c r="F1087" t="n">
+        <v>953.8</v>
+      </c>
+      <c r="G1087" t="n">
+        <v>870.09</v>
+      </c>
+      <c r="H1087" t="n">
+        <v>897.6799999999999</v>
+      </c>
+      <c r="I1087" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1087" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1087" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 870.09 &lt;= EMA21 897.68)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D1088" t="n">
+        <v>3187</v>
+      </c>
+      <c r="E1088" t="n">
+        <v>3375</v>
+      </c>
+      <c r="F1088" t="n">
+        <v>3375</v>
+      </c>
+      <c r="G1088" t="n">
+        <v>3255.71</v>
+      </c>
+      <c r="H1088" t="n">
+        <v>3267.63</v>
+      </c>
+      <c r="I1088" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1088" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1088" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3255.71 &lt;= EMA21 3267.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D1089" t="n">
+        <v>1253</v>
+      </c>
+      <c r="E1089" t="n">
+        <v>1372.25</v>
+      </c>
+      <c r="F1089" t="n">
+        <v>1372.25</v>
+      </c>
+      <c r="G1089" t="n">
+        <v>1250.1</v>
+      </c>
+      <c r="H1089" t="n">
+        <v>1273.41</v>
+      </c>
+      <c r="I1089" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J1089" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1089" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1250.10 &lt;= EMA21 1273.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D1090" t="n">
+        <v>2373.1</v>
+      </c>
+      <c r="E1090" t="n">
+        <v>2720.64</v>
+      </c>
+      <c r="F1090" t="n">
+        <v>2720.64</v>
+      </c>
+      <c r="G1090" t="n">
+        <v>2434.83</v>
+      </c>
+      <c r="H1090" t="n">
+        <v>2488.95</v>
+      </c>
+      <c r="I1090" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J1090" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1090" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2434.83 &lt;= EMA21 2488.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D1091" t="n">
+        <v>721.5</v>
+      </c>
+      <c r="E1091" t="n">
+        <v>735.98</v>
+      </c>
+      <c r="F1091" t="n">
+        <v>735.98</v>
+      </c>
+      <c r="G1091" t="n">
+        <v>710.3099999999999</v>
+      </c>
+      <c r="H1091" t="n">
+        <v>714.8200000000001</v>
+      </c>
+      <c r="I1091" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1091" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1091" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 710.31 &lt;= EMA21 714.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D1092" t="n">
+        <v>530.2</v>
+      </c>
+      <c r="E1092" t="n">
+        <v>561.15</v>
+      </c>
+      <c r="F1092" t="n">
+        <v>561.15</v>
+      </c>
+      <c r="G1092" t="n">
+        <v>528.8</v>
+      </c>
+      <c r="H1092" t="n">
+        <v>534.73</v>
+      </c>
+      <c r="I1092" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J1092" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1092" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 528.80 &lt;= EMA21 534.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D1093" t="n">
+        <v>972.7</v>
+      </c>
+      <c r="E1093" t="n">
+        <v>1070.43</v>
+      </c>
+      <c r="F1093" t="n">
+        <v>1070.43</v>
+      </c>
+      <c r="G1093" t="n">
+        <v>991.4400000000001</v>
+      </c>
+      <c r="H1093" t="n">
+        <v>1006.16</v>
+      </c>
+      <c r="I1093" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J1093" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1093" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 991.44 &lt;= EMA21 1006.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D1094" t="n">
+        <v>4695.6</v>
+      </c>
+      <c r="E1094" t="n">
+        <v>5085.01</v>
+      </c>
+      <c r="F1094" t="n">
+        <v>5085.01</v>
+      </c>
+      <c r="G1094" t="n">
+        <v>4832.73</v>
+      </c>
+      <c r="H1094" t="n">
+        <v>4850.5</v>
+      </c>
+      <c r="I1094" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J1094" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1094" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4832.73 &lt;= EMA21 4850.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D1095" t="n">
+        <v>1962</v>
+      </c>
+      <c r="E1095" t="n">
+        <v>2053.79</v>
+      </c>
+      <c r="F1095" t="n">
+        <v>2053.79</v>
+      </c>
+      <c r="G1095" t="n">
+        <v>1954.37</v>
+      </c>
+      <c r="H1095" t="n">
+        <v>1985.18</v>
+      </c>
+      <c r="I1095" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1095" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1095" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1954.37 &lt;= EMA21 1985.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D1096" t="n">
+        <v>567.5</v>
+      </c>
+      <c r="E1096" t="n">
+        <v>626.28</v>
+      </c>
+      <c r="F1096" t="n">
+        <v>626.28</v>
+      </c>
+      <c r="G1096" t="n">
+        <v>580.33</v>
+      </c>
+      <c r="H1096" t="n">
+        <v>583.83</v>
+      </c>
+      <c r="I1096" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J1096" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1096" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 580.33 &lt;= EMA21 583.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D1097" t="n">
+        <v>2155</v>
+      </c>
+      <c r="E1097" t="n">
+        <v>2272.61</v>
+      </c>
+      <c r="F1097" t="n">
+        <v>2272.61</v>
+      </c>
+      <c r="G1097" t="n">
+        <v>2175.53</v>
+      </c>
+      <c r="H1097" t="n">
+        <v>2180.49</v>
+      </c>
+      <c r="I1097" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1097" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1097" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2175.53 &lt;= EMA21 2180.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D1098" t="n">
+        <v>1358.8</v>
+      </c>
+      <c r="E1098" t="n">
+        <v>1466.6</v>
+      </c>
+      <c r="F1098" t="n">
+        <v>1466.6</v>
+      </c>
+      <c r="G1098" t="n">
+        <v>1383.09</v>
+      </c>
+      <c r="H1098" t="n">
+        <v>1401.09</v>
+      </c>
+      <c r="I1098" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1098" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1098" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1383.09 &lt;= EMA21 1401.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D1099" t="n">
+        <v>264.15</v>
+      </c>
+      <c r="E1099" t="n">
+        <v>274.05</v>
+      </c>
+      <c r="F1099" t="n">
+        <v>274.05</v>
+      </c>
+      <c r="G1099" t="n">
+        <v>261.78</v>
+      </c>
+      <c r="H1099" t="n">
+        <v>265.33</v>
+      </c>
+      <c r="I1099" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="J1099" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1099" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 261.78 &lt;= EMA21 265.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D1100" t="n">
+        <v>713.4</v>
+      </c>
+      <c r="E1100" t="n">
+        <v>738.55</v>
+      </c>
+      <c r="F1100" t="n">
+        <v>738.55</v>
+      </c>
+      <c r="G1100" t="n">
+        <v>717.98</v>
+      </c>
+      <c r="H1100" t="n">
+        <v>721.21</v>
+      </c>
+      <c r="I1100" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1100" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1100" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 717.98 &lt;= EMA21 721.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D1101" t="n">
+        <v>134.75</v>
+      </c>
+      <c r="E1101" t="n">
+        <v>140.21</v>
+      </c>
+      <c r="F1101" t="n">
+        <v>140.21</v>
+      </c>
+      <c r="G1101" t="n">
+        <v>134.96</v>
+      </c>
+      <c r="H1101" t="n">
+        <v>136.25</v>
+      </c>
+      <c r="I1101" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1101" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1101" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 134.96 &lt;= EMA21 136.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D1102" t="n">
+        <v>78.95</v>
+      </c>
+      <c r="E1102" t="n">
+        <v>87.73999999999999</v>
+      </c>
+      <c r="F1102" t="n">
+        <v>87.73999999999999</v>
+      </c>
+      <c r="G1102" t="n">
+        <v>80.98</v>
+      </c>
+      <c r="H1102" t="n">
+        <v>82.95999999999999</v>
+      </c>
+      <c r="I1102" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="J1102" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1102" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 80.98 &lt;= EMA21 82.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1103" t="n">
+        <v>1060</v>
+      </c>
+      <c r="E1103" t="n">
+        <v>1185.34</v>
+      </c>
+      <c r="F1103" t="n">
+        <v>1185.34</v>
+      </c>
+      <c r="G1103" t="n">
+        <v>1068.94</v>
+      </c>
+      <c r="H1103" t="n">
+        <v>1092.81</v>
+      </c>
+      <c r="I1103" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1103" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1103" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1068.94 &lt;= EMA21 1092.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D1104" t="n">
+        <v>4733.5</v>
+      </c>
+      <c r="E1104" t="n">
+        <v>5340.2</v>
+      </c>
+      <c r="F1104" t="n">
+        <v>5340.2</v>
+      </c>
+      <c r="G1104" t="n">
+        <v>4916.3</v>
+      </c>
+      <c r="H1104" t="n">
+        <v>5027.66</v>
+      </c>
+      <c r="I1104" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1104" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1104" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4916.30 &lt;= EMA21 5027.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D1105" t="n">
+        <v>1248.9</v>
+      </c>
+      <c r="E1105" t="n">
+        <v>1360.88</v>
+      </c>
+      <c r="F1105" t="n">
+        <v>1360.88</v>
+      </c>
+      <c r="G1105" t="n">
+        <v>1273.81</v>
+      </c>
+      <c r="H1105" t="n">
+        <v>1287.31</v>
+      </c>
+      <c r="I1105" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J1105" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1105" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1273.81 &lt;= EMA21 1287.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D1106" t="n">
+        <v>1103</v>
+      </c>
+      <c r="E1106" t="n">
+        <v>1196.84</v>
+      </c>
+      <c r="F1106" t="n">
+        <v>1196.84</v>
+      </c>
+      <c r="G1106" t="n">
+        <v>1124.63</v>
+      </c>
+      <c r="H1106" t="n">
+        <v>1129.6</v>
+      </c>
+      <c r="I1106" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J1106" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1106" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1124.63 &lt;= EMA21 1129.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D1107" t="n">
+        <v>224.84</v>
+      </c>
+      <c r="E1107" t="n">
+        <v>248.85</v>
+      </c>
+      <c r="F1107" t="n">
+        <v>248.85</v>
+      </c>
+      <c r="G1107" t="n">
+        <v>230.51</v>
+      </c>
+      <c r="H1107" t="n">
+        <v>235.84</v>
+      </c>
+      <c r="I1107" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1107" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1107" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 230.51 &lt;= EMA21 235.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D1108" t="n">
+        <v>415</v>
+      </c>
+      <c r="E1108" t="n">
+        <v>433.12</v>
+      </c>
+      <c r="F1108" t="n">
+        <v>433.12</v>
+      </c>
+      <c r="G1108" t="n">
+        <v>416.25</v>
+      </c>
+      <c r="H1108" t="n">
+        <v>413</v>
+      </c>
+      <c r="I1108" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J1108" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1108" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 415.00 &lt;= Upper 433.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D1109" t="n">
+        <v>4233</v>
+      </c>
+      <c r="E1109" t="n">
+        <v>4708.69</v>
+      </c>
+      <c r="F1109" t="n">
+        <v>4708.69</v>
+      </c>
+      <c r="G1109" t="n">
+        <v>4359.56</v>
+      </c>
+      <c r="H1109" t="n">
+        <v>4430.31</v>
+      </c>
+      <c r="I1109" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J1109" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1109" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4359.56 &lt;= EMA21 4430.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D1110" t="n">
+        <v>3807.7</v>
+      </c>
+      <c r="E1110" t="n">
+        <v>4150.55</v>
+      </c>
+      <c r="F1110" t="n">
+        <v>4150.55</v>
+      </c>
+      <c r="G1110" t="n">
+        <v>3911.24</v>
+      </c>
+      <c r="H1110" t="n">
+        <v>3958.5</v>
+      </c>
+      <c r="I1110" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="J1110" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1110" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3911.24 &lt;= EMA21 3958.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D1111" t="n">
+        <v>1087.4</v>
+      </c>
+      <c r="E1111" t="n">
+        <v>1325.25</v>
+      </c>
+      <c r="F1111" t="n">
+        <v>1325.25</v>
+      </c>
+      <c r="G1111" t="n">
+        <v>1137.91</v>
+      </c>
+      <c r="H1111" t="n">
+        <v>1176.2</v>
+      </c>
+      <c r="I1111" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1111" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1111" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1137.91 &lt;= EMA21 1176.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D1112" t="n">
+        <v>3070</v>
+      </c>
+      <c r="E1112" t="n">
+        <v>3502.3</v>
+      </c>
+      <c r="F1112" t="n">
+        <v>3502.3</v>
+      </c>
+      <c r="G1112" t="n">
+        <v>3121.83</v>
+      </c>
+      <c r="H1112" t="n">
+        <v>3200.81</v>
+      </c>
+      <c r="I1112" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="J1112" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1112" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3121.83 &lt;= EMA21 3200.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D1113" t="n">
+        <v>12166</v>
+      </c>
+      <c r="E1113" t="n">
+        <v>14048.32</v>
+      </c>
+      <c r="F1113" t="n">
+        <v>14048.32</v>
+      </c>
+      <c r="G1113" t="n">
+        <v>12505.77</v>
+      </c>
+      <c r="H1113" t="n">
+        <v>12886.59</v>
+      </c>
+      <c r="I1113" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1113" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1113" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12505.77 &lt;= EMA21 12886.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D1114" t="n">
+        <v>1025</v>
+      </c>
+      <c r="E1114" t="n">
+        <v>1047.69</v>
+      </c>
+      <c r="F1114" t="n">
+        <v>1047.69</v>
+      </c>
+      <c r="G1114" t="n">
+        <v>1021.88</v>
+      </c>
+      <c r="H1114" t="n">
+        <v>1022.62</v>
+      </c>
+      <c r="I1114" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1114" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1114" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1021.88 &lt;= EMA21 1022.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D1115" t="n">
+        <v>2231.9</v>
+      </c>
+      <c r="E1115" t="n">
+        <v>2699.1</v>
+      </c>
+      <c r="F1115" t="n">
+        <v>2699.1</v>
+      </c>
+      <c r="G1115" t="n">
+        <v>2350.95</v>
+      </c>
+      <c r="H1115" t="n">
+        <v>2421.37</v>
+      </c>
+      <c r="I1115" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1115" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1115" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2350.95 &lt;= EMA21 2421.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D1116" t="n">
+        <v>2771.4</v>
+      </c>
+      <c r="E1116" t="n">
+        <v>3241.16</v>
+      </c>
+      <c r="F1116" t="n">
+        <v>3241.16</v>
+      </c>
+      <c r="G1116" t="n">
+        <v>2833.78</v>
+      </c>
+      <c r="H1116" t="n">
+        <v>2899.52</v>
+      </c>
+      <c r="I1116" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1116" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1116" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2833.78 &lt;= EMA21 2899.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D1117" t="n">
+        <v>327</v>
+      </c>
+      <c r="E1117" t="n">
+        <v>338.92</v>
+      </c>
+      <c r="F1117" t="n">
+        <v>338.92</v>
+      </c>
+      <c r="G1117" t="n">
+        <v>330.97</v>
+      </c>
+      <c r="H1117" t="n">
+        <v>332.3</v>
+      </c>
+      <c r="I1117" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J1117" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1117" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 330.97 &lt;= EMA21 332.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D1118" t="n">
+        <v>1384.5</v>
+      </c>
+      <c r="E1118" t="n">
+        <v>1504.83</v>
+      </c>
+      <c r="F1118" t="n">
+        <v>1504.83</v>
+      </c>
+      <c r="G1118" t="n">
+        <v>1392.25</v>
+      </c>
+      <c r="H1118" t="n">
+        <v>1419.33</v>
+      </c>
+      <c r="I1118" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J1118" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1118" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1392.25 &lt;= EMA21 1419.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D1119" t="n">
+        <v>236.8</v>
+      </c>
+      <c r="E1119" t="n">
+        <v>238.67</v>
+      </c>
+      <c r="F1119" t="n">
+        <v>238.67</v>
+      </c>
+      <c r="G1119" t="n">
+        <v>234.96</v>
+      </c>
+      <c r="H1119" t="n">
+        <v>235.33</v>
+      </c>
+      <c r="I1119" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1119" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1119" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.96 &lt;= EMA21 235.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D1120" t="n">
+        <v>1543.8</v>
+      </c>
+      <c r="E1120" t="n">
+        <v>1708.46</v>
+      </c>
+      <c r="F1120" t="n">
+        <v>1708.46</v>
+      </c>
+      <c r="G1120" t="n">
+        <v>1570.36</v>
+      </c>
+      <c r="H1120" t="n">
+        <v>1600.71</v>
+      </c>
+      <c r="I1120" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1120" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1120" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1570.36 &lt;= EMA21 1600.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D1121" t="n">
+        <v>346</v>
+      </c>
+      <c r="E1121" t="n">
+        <v>366.04</v>
+      </c>
+      <c r="F1121" t="n">
+        <v>366.04</v>
+      </c>
+      <c r="G1121" t="n">
+        <v>350.19</v>
+      </c>
+      <c r="H1121" t="n">
+        <v>357</v>
+      </c>
+      <c r="I1121" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J1121" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1121" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 350.19 &lt;= EMA21 357.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D1122" t="n">
+        <v>262.8</v>
+      </c>
+      <c r="E1122" t="n">
+        <v>272.77</v>
+      </c>
+      <c r="F1122" t="n">
+        <v>272.77</v>
+      </c>
+      <c r="G1122" t="n">
+        <v>266.06</v>
+      </c>
+      <c r="H1122" t="n">
+        <v>267.75</v>
+      </c>
+      <c r="I1122" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1122" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1122" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.06 &lt;= EMA21 267.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D1123" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="E1123" t="n">
+        <v>117.94</v>
+      </c>
+      <c r="F1123" t="n">
+        <v>117.94</v>
+      </c>
+      <c r="G1123" t="n">
+        <v>116.18</v>
+      </c>
+      <c r="H1123" t="n">
+        <v>115.84</v>
+      </c>
+      <c r="I1123" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J1123" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1123" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.80 &lt;= Upper 117.94)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D1124" t="n">
+        <v>312.65</v>
+      </c>
+      <c r="E1124" t="n">
+        <v>329.79</v>
+      </c>
+      <c r="F1124" t="n">
+        <v>329.79</v>
+      </c>
+      <c r="G1124" t="n">
+        <v>313.9</v>
+      </c>
+      <c r="H1124" t="n">
+        <v>320.7</v>
+      </c>
+      <c r="I1124" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1124" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1124" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 313.90 &lt;= EMA21 320.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D1125" t="n">
+        <v>1240</v>
+      </c>
+      <c r="E1125" t="n">
+        <v>1342.24</v>
+      </c>
+      <c r="F1125" t="n">
+        <v>1342.24</v>
+      </c>
+      <c r="G1125" t="n">
+        <v>1265.51</v>
+      </c>
+      <c r="H1125" t="n">
+        <v>1283.28</v>
+      </c>
+      <c r="I1125" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1125" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1125" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1265.51 &lt;= EMA21 1283.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D1126" t="n">
+        <v>1697.9</v>
+      </c>
+      <c r="E1126" t="n">
+        <v>1810.55</v>
+      </c>
+      <c r="F1126" t="n">
+        <v>1810.55</v>
+      </c>
+      <c r="G1126" t="n">
+        <v>1697.68</v>
+      </c>
+      <c r="H1126" t="n">
+        <v>1730.16</v>
+      </c>
+      <c r="I1126" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1126" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1126" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1697.68 &lt;= EMA21 1730.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D1127" t="n">
+        <v>158.27</v>
+      </c>
+      <c r="E1127" t="n">
+        <v>171.48</v>
+      </c>
+      <c r="F1127" t="n">
+        <v>171.48</v>
+      </c>
+      <c r="G1127" t="n">
+        <v>161.93</v>
+      </c>
+      <c r="H1127" t="n">
+        <v>162.75</v>
+      </c>
+      <c r="I1127" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1127" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1127" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 161.93 &lt;= EMA21 162.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>21795</v>
+      </c>
+      <c r="E1128" t="n">
+        <v>25271.83</v>
+      </c>
+      <c r="F1128" t="n">
+        <v>25271.83</v>
+      </c>
+      <c r="G1128" t="n">
+        <v>22734.31</v>
+      </c>
+      <c r="H1128" t="n">
+        <v>23553.23</v>
+      </c>
+      <c r="I1128" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1128" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1128" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 22734.31 &lt;= EMA21 23553.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>979</v>
+      </c>
+      <c r="E1129" t="n">
+        <v>1161.78</v>
+      </c>
+      <c r="F1129" t="n">
+        <v>1161.78</v>
+      </c>
+      <c r="G1129" t="n">
+        <v>1019.47</v>
+      </c>
+      <c r="H1129" t="n">
+        <v>1047.93</v>
+      </c>
+      <c r="I1129" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="J1129" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1129" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1019.47 &lt;= EMA21 1047.93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D1130" t="n">
+        <v>3013.4</v>
+      </c>
+      <c r="E1130" t="n">
+        <v>3485.41</v>
+      </c>
+      <c r="F1130" t="n">
+        <v>3485.41</v>
+      </c>
+      <c r="G1130" t="n">
+        <v>3128.47</v>
+      </c>
+      <c r="H1130" t="n">
+        <v>3212.35</v>
+      </c>
+      <c r="I1130" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1130" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1130" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3128.47 &lt;= EMA21 3212.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D1131" t="n">
+        <v>3742</v>
+      </c>
+      <c r="E1131" t="n">
+        <v>4175.54</v>
+      </c>
+      <c r="F1131" t="n">
+        <v>4175.54</v>
+      </c>
+      <c r="G1131" t="n">
+        <v>3892.11</v>
+      </c>
+      <c r="H1131" t="n">
+        <v>3928.13</v>
+      </c>
+      <c r="I1131" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="J1131" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1131" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3892.11 &lt;= EMA21 3928.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D1132" t="n">
+        <v>18900</v>
+      </c>
+      <c r="E1132" t="n">
+        <v>23129.13</v>
+      </c>
+      <c r="F1132" t="n">
+        <v>23129.13</v>
+      </c>
+      <c r="G1132" t="n">
+        <v>20853.4</v>
+      </c>
+      <c r="H1132" t="n">
+        <v>20689.57</v>
+      </c>
+      <c r="I1132" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="J1132" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1132" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 18900.00 &lt;= Upper 23129.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D1133" t="n">
+        <v>991.4</v>
+      </c>
+      <c r="E1133" t="n">
+        <v>1073.68</v>
+      </c>
+      <c r="F1133" t="n">
+        <v>1073.68</v>
+      </c>
+      <c r="G1133" t="n">
+        <v>999.4299999999999</v>
+      </c>
+      <c r="H1133" t="n">
+        <v>1017.03</v>
+      </c>
+      <c r="I1133" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J1133" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1133" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 999.43 &lt;= EMA21 1017.03)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D1134" t="n">
+        <v>1853.5</v>
+      </c>
+      <c r="E1134" t="n">
+        <v>1970.2</v>
+      </c>
+      <c r="F1134" t="n">
+        <v>1970.2</v>
+      </c>
+      <c r="G1134" t="n">
+        <v>1863.48</v>
+      </c>
+      <c r="H1134" t="n">
+        <v>1887.4</v>
+      </c>
+      <c r="I1134" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1134" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1134" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1863.48 &lt;= EMA21 1887.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D1135" t="n">
+        <v>4033</v>
+      </c>
+      <c r="E1135" t="n">
+        <v>4506.65</v>
+      </c>
+      <c r="F1135" t="n">
+        <v>4506.65</v>
+      </c>
+      <c r="G1135" t="n">
+        <v>4118.87</v>
+      </c>
+      <c r="H1135" t="n">
+        <v>4178.78</v>
+      </c>
+      <c r="I1135" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="J1135" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1135" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4118.87 &lt;= EMA21 4178.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D1136" t="n">
+        <v>343.5</v>
+      </c>
+      <c r="E1136" t="n">
+        <v>380.88</v>
+      </c>
+      <c r="F1136" t="n">
+        <v>380.88</v>
+      </c>
+      <c r="G1136" t="n">
+        <v>359.73</v>
+      </c>
+      <c r="H1136" t="n">
+        <v>363.3</v>
+      </c>
+      <c r="I1136" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="J1136" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1136" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 359.73 &lt;= EMA21 363.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D1137" t="n">
+        <v>2188.8</v>
+      </c>
+      <c r="E1137" t="n">
+        <v>2397.88</v>
+      </c>
+      <c r="F1137" t="n">
+        <v>2397.88</v>
+      </c>
+      <c r="G1137" t="n">
+        <v>2234.02</v>
+      </c>
+      <c r="H1137" t="n">
+        <v>2268.4</v>
+      </c>
+      <c r="I1137" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1137" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1137" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2234.02 &lt;= EMA21 2268.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D1138" t="n">
+        <v>1000.1</v>
+      </c>
+      <c r="E1138" t="n">
+        <v>1072.86</v>
+      </c>
+      <c r="F1138" t="n">
+        <v>1072.86</v>
+      </c>
+      <c r="G1138" t="n">
+        <v>1002.26</v>
+      </c>
+      <c r="H1138" t="n">
+        <v>1022.37</v>
+      </c>
+      <c r="I1138" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="J1138" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1138" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1002.26 &lt;= EMA21 1022.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D1139" t="n">
+        <v>424.25</v>
+      </c>
+      <c r="E1139" t="n">
+        <v>493.29</v>
+      </c>
+      <c r="F1139" t="n">
+        <v>493.29</v>
+      </c>
+      <c r="G1139" t="n">
+        <v>439.39</v>
+      </c>
+      <c r="H1139" t="n">
+        <v>448.52</v>
+      </c>
+      <c r="I1139" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1139" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1139" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 439.39 &lt;= EMA21 448.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D1140" t="n">
+        <v>301</v>
+      </c>
+      <c r="E1140" t="n">
+        <v>322.63</v>
+      </c>
+      <c r="F1140" t="n">
+        <v>322.63</v>
+      </c>
+      <c r="G1140" t="n">
+        <v>304.28</v>
+      </c>
+      <c r="H1140" t="n">
+        <v>311.27</v>
+      </c>
+      <c r="I1140" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="J1140" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1140" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 304.28 &lt;= EMA21 311.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D1141" t="n">
+        <v>360.4</v>
+      </c>
+      <c r="E1141" t="n">
+        <v>379.86</v>
+      </c>
+      <c r="F1141" t="n">
+        <v>379.86</v>
+      </c>
+      <c r="G1141" t="n">
+        <v>363.88</v>
+      </c>
+      <c r="H1141" t="n">
+        <v>366.17</v>
+      </c>
+      <c r="I1141" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J1141" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1141" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 363.88 &lt;= EMA21 366.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D1142" t="n">
+        <v>183</v>
+      </c>
+      <c r="E1142" t="n">
+        <v>189.19</v>
+      </c>
+      <c r="F1142" t="n">
+        <v>189.19</v>
+      </c>
+      <c r="G1142" t="n">
+        <v>184.42</v>
+      </c>
+      <c r="H1142" t="n">
+        <v>185.23</v>
+      </c>
+      <c r="I1142" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1142" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1142" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 184.42 &lt;= EMA21 185.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D1143" t="n">
+        <v>1558</v>
+      </c>
+      <c r="E1143" t="n">
+        <v>1653.09</v>
+      </c>
+      <c r="F1143" t="n">
+        <v>1653.09</v>
+      </c>
+      <c r="G1143" t="n">
+        <v>1562.37</v>
+      </c>
+      <c r="H1143" t="n">
+        <v>1577.4</v>
+      </c>
+      <c r="I1143" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1143" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1143" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1562.37 &lt;= EMA21 1577.40)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D1144" t="n">
+        <v>4908.5</v>
+      </c>
+      <c r="E1144" t="n">
+        <v>5191.56</v>
+      </c>
+      <c r="F1144" t="n">
+        <v>5191.56</v>
+      </c>
+      <c r="G1144" t="n">
+        <v>4973.08</v>
+      </c>
+      <c r="H1144" t="n">
+        <v>4997.38</v>
+      </c>
+      <c r="I1144" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1144" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1144" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4973.08 &lt;= EMA21 4997.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D1145" t="n">
+        <v>4812.5</v>
+      </c>
+      <c r="E1145" t="n">
+        <v>5072.48</v>
+      </c>
+      <c r="F1145" t="n">
+        <v>5072.48</v>
+      </c>
+      <c r="G1145" t="n">
+        <v>4905.59</v>
+      </c>
+      <c r="H1145" t="n">
+        <v>4925.96</v>
+      </c>
+      <c r="I1145" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="J1145" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1145" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4905.59 &lt;= EMA21 4925.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D1146" t="n">
+        <v>2769.7</v>
+      </c>
+      <c r="E1146" t="n">
+        <v>2972.09</v>
+      </c>
+      <c r="F1146" t="n">
+        <v>2972.09</v>
+      </c>
+      <c r="G1146" t="n">
+        <v>2798.49</v>
+      </c>
+      <c r="H1146" t="n">
+        <v>2846.97</v>
+      </c>
+      <c r="I1146" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1146" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1146" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2798.49 &lt;= EMA21 2846.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D1147" t="n">
+        <v>10700</v>
+      </c>
+      <c r="E1147" t="n">
+        <v>11927.38</v>
+      </c>
+      <c r="F1147" t="n">
+        <v>11927.38</v>
+      </c>
+      <c r="G1147" t="n">
+        <v>10968.38</v>
+      </c>
+      <c r="H1147" t="n">
+        <v>11209.85</v>
+      </c>
+      <c r="I1147" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1147" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1147" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 10968.38 &lt;= EMA21 11209.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D1148" t="n">
+        <v>178.2</v>
+      </c>
+      <c r="E1148" t="n">
+        <v>191.74</v>
+      </c>
+      <c r="F1148" t="n">
+        <v>191.74</v>
+      </c>
+      <c r="G1148" t="n">
+        <v>180.14</v>
+      </c>
+      <c r="H1148" t="n">
+        <v>181.8</v>
+      </c>
+      <c r="I1148" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J1148" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1148" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 180.14 &lt;= EMA21 181.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D1149" t="n">
+        <v>1389.5</v>
+      </c>
+      <c r="E1149" t="n">
+        <v>1595.5</v>
+      </c>
+      <c r="F1149" t="n">
+        <v>1595.5</v>
+      </c>
+      <c r="G1149" t="n">
+        <v>1412.11</v>
+      </c>
+      <c r="H1149" t="n">
+        <v>1448.04</v>
+      </c>
+      <c r="I1149" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J1149" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1149" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1412.11 &lt;= EMA21 1448.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D1150" t="n">
+        <v>410.4</v>
+      </c>
+      <c r="E1150" t="n">
+        <v>437.05</v>
+      </c>
+      <c r="F1150" t="n">
+        <v>437.05</v>
+      </c>
+      <c r="G1150" t="n">
+        <v>411.63</v>
+      </c>
+      <c r="H1150" t="n">
+        <v>417.53</v>
+      </c>
+      <c r="I1150" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J1150" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1150" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 411.63 &lt;= EMA21 417.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D1151" t="n">
+        <v>256</v>
+      </c>
+      <c r="E1151" t="n">
+        <v>288.86</v>
+      </c>
+      <c r="F1151" t="n">
+        <v>288.86</v>
+      </c>
+      <c r="G1151" t="n">
+        <v>264.54</v>
+      </c>
+      <c r="H1151" t="n">
+        <v>268.85</v>
+      </c>
+      <c r="I1151" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="J1151" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1151" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 264.54 &lt;= EMA21 268.85)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D1152" t="n">
+        <v>166.89</v>
+      </c>
+      <c r="E1152" t="n">
+        <v>187.12</v>
+      </c>
+      <c r="F1152" t="n">
+        <v>187.12</v>
+      </c>
+      <c r="G1152" t="n">
+        <v>169.94</v>
+      </c>
+      <c r="H1152" t="n">
+        <v>173.77</v>
+      </c>
+      <c r="I1152" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J1152" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1152" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 169.94 &lt;= EMA21 173.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D1153" t="n">
+        <v>1107.5</v>
+      </c>
+      <c r="E1153" t="n">
+        <v>1191.01</v>
+      </c>
+      <c r="F1153" t="n">
+        <v>1191.01</v>
+      </c>
+      <c r="G1153" t="n">
+        <v>1121.52</v>
+      </c>
+      <c r="H1153" t="n">
+        <v>1130.64</v>
+      </c>
+      <c r="I1153" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J1153" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1153" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1121.52 &lt;= EMA21 1130.64)</t>
         </is>
       </c>
     </row>
@@ -46019,7 +50319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46100,10 +50400,10 @@
         <v>19685.95</v>
       </c>
       <c r="F2" t="n">
-        <v>419.25</v>
+        <v>422.25</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H2" t="n">
         <v>416.67</v>
@@ -46112,50 +50412,9 @@
         <v>436.2999877929688</v>
       </c>
       <c r="J2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>ADANIPORTS</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>1775</v>
-      </c>
-      <c r="D3" t="n">
-        <v>11</v>
-      </c>
-      <c r="E3" t="n">
-        <v>19525</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1713.8</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-3.45</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1710.79</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1791.400024414062</v>
-      </c>
-      <c r="J3" t="n">
-        <v>4</v>
-      </c>
-      <c r="K3" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -46172,7 +50431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47155,6 +51414,57 @@
         <v>4</v>
       </c>
       <c r="M20" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1775</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1710.79</v>
+      </c>
+      <c r="F21" t="n">
+        <v>11</v>
+      </c>
+      <c r="G21" t="n">
+        <v>19525</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-3.617</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-3.917</v>
+      </c>
+      <c r="J21" t="n">
+        <v>-764.79</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>5</v>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -47171,7 +51481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K149"/>
+  <dimension ref="A1:K150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52504,6 +56814,55 @@
         </is>
       </c>
       <c r="K149" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-16 20:29:37</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>6019EAC875</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>1710.79</v>
+      </c>
+      <c r="G150" t="n">
+        <v>1710.79</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" t="n">
+        <v>11</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
         <is>
           <t>HARD_STOP_LOSS</t>
         </is>
@@ -52588,7 +56947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53100,6 +57459,39 @@
         <v>2</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20:29:38</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>176592.45</v>
+      </c>
+      <c r="D16" t="n">
+        <v>19685.95</v>
+      </c>
+      <c r="E16" t="n">
+        <v>196278.4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-3635.96</v>
+      </c>
+      <c r="G16" t="n">
+        <v>20</v>
+      </c>
+      <c r="H16" t="n">
+        <v>20</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-17T20:31 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1153"/>
+  <dimension ref="A1:K1253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50006,6 +50006,4306 @@
       <c r="K1153" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1121.52 &lt;= EMA21 1130.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D1154" t="n">
+        <v>7130.5</v>
+      </c>
+      <c r="E1154" t="n">
+        <v>7752.09</v>
+      </c>
+      <c r="F1154" t="n">
+        <v>7752.09</v>
+      </c>
+      <c r="G1154" t="n">
+        <v>7212.89</v>
+      </c>
+      <c r="H1154" t="n">
+        <v>7329.36</v>
+      </c>
+      <c r="I1154" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1154" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1154" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7212.89 &lt;= EMA21 7329.36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D1155" t="n">
+        <v>1386.8</v>
+      </c>
+      <c r="E1155" t="n">
+        <v>1628.11</v>
+      </c>
+      <c r="F1155" t="n">
+        <v>1628.11</v>
+      </c>
+      <c r="G1155" t="n">
+        <v>1386.16</v>
+      </c>
+      <c r="H1155" t="n">
+        <v>1439.64</v>
+      </c>
+      <c r="I1155" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="J1155" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1155" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1386.16 &lt;= EMA21 1439.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D1156" t="n">
+        <v>2923.2</v>
+      </c>
+      <c r="E1156" t="n">
+        <v>3200.1</v>
+      </c>
+      <c r="F1156" t="n">
+        <v>3200.1</v>
+      </c>
+      <c r="G1156" t="n">
+        <v>2975.43</v>
+      </c>
+      <c r="H1156" t="n">
+        <v>2992.73</v>
+      </c>
+      <c r="I1156" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J1156" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1156" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2975.43 &lt;= EMA21 2992.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D1157" t="n">
+        <v>1274.2</v>
+      </c>
+      <c r="E1157" t="n">
+        <v>1345.38</v>
+      </c>
+      <c r="F1157" t="n">
+        <v>1345.38</v>
+      </c>
+      <c r="G1157" t="n">
+        <v>1279.89</v>
+      </c>
+      <c r="H1157" t="n">
+        <v>1297.12</v>
+      </c>
+      <c r="I1157" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J1157" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1157" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1279.89 &lt;= EMA21 1297.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D1158" t="n">
+        <v>1738.3</v>
+      </c>
+      <c r="E1158" t="n">
+        <v>1795.07</v>
+      </c>
+      <c r="F1158" t="n">
+        <v>1795.07</v>
+      </c>
+      <c r="G1158" t="n">
+        <v>1731.28</v>
+      </c>
+      <c r="H1158" t="n">
+        <v>1719.52</v>
+      </c>
+      <c r="I1158" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="J1158" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1158" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1738.30 &lt;= Upper 1795.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D1159" t="n">
+        <v>205.92</v>
+      </c>
+      <c r="E1159" t="n">
+        <v>216.26</v>
+      </c>
+      <c r="F1159" t="n">
+        <v>216.26</v>
+      </c>
+      <c r="G1159" t="n">
+        <v>206.74</v>
+      </c>
+      <c r="H1159" t="n">
+        <v>207.55</v>
+      </c>
+      <c r="I1159" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J1159" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1159" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 206.74 &lt;= EMA21 207.55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D1160" t="n">
+        <v>383.25</v>
+      </c>
+      <c r="E1160" t="n">
+        <v>422.64</v>
+      </c>
+      <c r="F1160" t="n">
+        <v>422.64</v>
+      </c>
+      <c r="G1160" t="n">
+        <v>390.17</v>
+      </c>
+      <c r="H1160" t="n">
+        <v>399.52</v>
+      </c>
+      <c r="I1160" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1160" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1160" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 390.17 &lt;= EMA21 399.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D1161" t="n">
+        <v>8768.5</v>
+      </c>
+      <c r="E1161" t="n">
+        <v>8959.15</v>
+      </c>
+      <c r="F1161" t="n">
+        <v>8959.15</v>
+      </c>
+      <c r="G1161" t="n">
+        <v>8780.219999999999</v>
+      </c>
+      <c r="H1161" t="n">
+        <v>8790.799999999999</v>
+      </c>
+      <c r="I1161" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1161" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1161" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 8780.22 &lt;= EMA21 8790.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D1162" t="n">
+        <v>2454</v>
+      </c>
+      <c r="E1162" t="n">
+        <v>2702.2</v>
+      </c>
+      <c r="F1162" t="n">
+        <v>2702.2</v>
+      </c>
+      <c r="G1162" t="n">
+        <v>2469.52</v>
+      </c>
+      <c r="H1162" t="n">
+        <v>2530.82</v>
+      </c>
+      <c r="I1162" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="J1162" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1162" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2469.52 &lt;= EMA21 2530.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D1163" t="n">
+        <v>3711.2</v>
+      </c>
+      <c r="E1163" t="n">
+        <v>3954.74</v>
+      </c>
+      <c r="F1163" t="n">
+        <v>3954.74</v>
+      </c>
+      <c r="G1163" t="n">
+        <v>3720.78</v>
+      </c>
+      <c r="H1163" t="n">
+        <v>3783.52</v>
+      </c>
+      <c r="I1163" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="J1163" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1163" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3720.78 &lt;= EMA21 3783.52)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D1164" t="n">
+        <v>1240</v>
+      </c>
+      <c r="E1164" t="n">
+        <v>1284.21</v>
+      </c>
+      <c r="F1164" t="n">
+        <v>1284.21</v>
+      </c>
+      <c r="G1164" t="n">
+        <v>1243.33</v>
+      </c>
+      <c r="H1164" t="n">
+        <v>1247.75</v>
+      </c>
+      <c r="I1164" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1164" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1164" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1243.33 &lt;= EMA21 1247.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D1165" t="n">
+        <v>11500</v>
+      </c>
+      <c r="E1165" t="n">
+        <v>12256.93</v>
+      </c>
+      <c r="F1165" t="n">
+        <v>12256.93</v>
+      </c>
+      <c r="G1165" t="n">
+        <v>11658.52</v>
+      </c>
+      <c r="H1165" t="n">
+        <v>11705.71</v>
+      </c>
+      <c r="I1165" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J1165" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1165" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11658.52 &lt;= EMA21 11705.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D1166" t="n">
+        <v>1015</v>
+      </c>
+      <c r="E1166" t="n">
+        <v>1105.93</v>
+      </c>
+      <c r="F1166" t="n">
+        <v>1105.93</v>
+      </c>
+      <c r="G1166" t="n">
+        <v>1029.51</v>
+      </c>
+      <c r="H1166" t="n">
+        <v>1047.7</v>
+      </c>
+      <c r="I1166" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1166" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1166" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1029.51 &lt;= EMA21 1047.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D1167" t="n">
+        <v>1859.2</v>
+      </c>
+      <c r="E1167" t="n">
+        <v>2072.88</v>
+      </c>
+      <c r="F1167" t="n">
+        <v>2072.88</v>
+      </c>
+      <c r="G1167" t="n">
+        <v>1898.08</v>
+      </c>
+      <c r="H1167" t="n">
+        <v>1936.74</v>
+      </c>
+      <c r="I1167" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="J1167" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1167" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1898.08 &lt;= EMA21 1936.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D1168" t="n">
+        <v>11010</v>
+      </c>
+      <c r="E1168" t="n">
+        <v>11570.21</v>
+      </c>
+      <c r="F1168" t="n">
+        <v>11570.21</v>
+      </c>
+      <c r="G1168" t="n">
+        <v>11069.13</v>
+      </c>
+      <c r="H1168" t="n">
+        <v>11139.37</v>
+      </c>
+      <c r="I1168" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1168" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1168" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11069.13 &lt;= EMA21 11139.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D1169" t="n">
+        <v>232.3</v>
+      </c>
+      <c r="E1169" t="n">
+        <v>245.83</v>
+      </c>
+      <c r="F1169" t="n">
+        <v>245.83</v>
+      </c>
+      <c r="G1169" t="n">
+        <v>235.76</v>
+      </c>
+      <c r="H1169" t="n">
+        <v>238.64</v>
+      </c>
+      <c r="I1169" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="J1169" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1169" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 235.76 &lt;= EMA21 238.64)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D1170" t="n">
+        <v>395.45</v>
+      </c>
+      <c r="E1170" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="F1170" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="G1170" t="n">
+        <v>397.82</v>
+      </c>
+      <c r="H1170" t="n">
+        <v>402.35</v>
+      </c>
+      <c r="I1170" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1170" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1170" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 397.82 &lt;= EMA21 402.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D1171" t="n">
+        <v>307</v>
+      </c>
+      <c r="E1171" t="n">
+        <v>326.84</v>
+      </c>
+      <c r="F1171" t="n">
+        <v>326.84</v>
+      </c>
+      <c r="G1171" t="n">
+        <v>305.98</v>
+      </c>
+      <c r="H1171" t="n">
+        <v>309.71</v>
+      </c>
+      <c r="I1171" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1171" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1171" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 305.98 &lt;= EMA21 309.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D1172" t="n">
+        <v>1836</v>
+      </c>
+      <c r="E1172" t="n">
+        <v>1946.2</v>
+      </c>
+      <c r="F1172" t="n">
+        <v>1946.2</v>
+      </c>
+      <c r="G1172" t="n">
+        <v>1839.33</v>
+      </c>
+      <c r="H1172" t="n">
+        <v>1861.57</v>
+      </c>
+      <c r="I1172" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1172" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1172" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1839.33 &lt;= EMA21 1861.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D1173" t="n">
+        <v>47735</v>
+      </c>
+      <c r="E1173" t="n">
+        <v>49881</v>
+      </c>
+      <c r="F1173" t="n">
+        <v>49881</v>
+      </c>
+      <c r="G1173" t="n">
+        <v>47937.42</v>
+      </c>
+      <c r="H1173" t="n">
+        <v>47548.6</v>
+      </c>
+      <c r="I1173" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J1173" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1173" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47735.00 &lt;= Upper 49881.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D1174" t="n">
+        <v>4982</v>
+      </c>
+      <c r="E1174" t="n">
+        <v>5439.07</v>
+      </c>
+      <c r="F1174" t="n">
+        <v>5439.07</v>
+      </c>
+      <c r="G1174" t="n">
+        <v>5021.98</v>
+      </c>
+      <c r="H1174" t="n">
+        <v>5132.95</v>
+      </c>
+      <c r="I1174" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J1174" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1174" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5021.98 &lt;= EMA21 5132.95)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D1175" t="n">
+        <v>880</v>
+      </c>
+      <c r="E1175" t="n">
+        <v>931.09</v>
+      </c>
+      <c r="F1175" t="n">
+        <v>931.09</v>
+      </c>
+      <c r="G1175" t="n">
+        <v>885.62</v>
+      </c>
+      <c r="H1175" t="n">
+        <v>888.66</v>
+      </c>
+      <c r="I1175" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1175" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1175" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 885.62 &lt;= EMA21 888.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D1176" t="n">
+        <v>123.9</v>
+      </c>
+      <c r="E1176" t="n">
+        <v>130.27</v>
+      </c>
+      <c r="F1176" t="n">
+        <v>130.27</v>
+      </c>
+      <c r="G1176" t="n">
+        <v>124.1</v>
+      </c>
+      <c r="H1176" t="n">
+        <v>125.48</v>
+      </c>
+      <c r="I1176" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="J1176" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1176" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.10 &lt;= EMA21 125.48)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D1177" t="n">
+        <v>1764.5</v>
+      </c>
+      <c r="E1177" t="n">
+        <v>1907.89</v>
+      </c>
+      <c r="F1177" t="n">
+        <v>1907.89</v>
+      </c>
+      <c r="G1177" t="n">
+        <v>1809.29</v>
+      </c>
+      <c r="H1177" t="n">
+        <v>1830.06</v>
+      </c>
+      <c r="I1177" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J1177" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1177" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1809.29 &lt;= EMA21 1830.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D1178" t="n">
+        <v>1376.3</v>
+      </c>
+      <c r="E1178" t="n">
+        <v>1454.19</v>
+      </c>
+      <c r="F1178" t="n">
+        <v>1454.19</v>
+      </c>
+      <c r="G1178" t="n">
+        <v>1373.27</v>
+      </c>
+      <c r="H1178" t="n">
+        <v>1392.97</v>
+      </c>
+      <c r="I1178" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1178" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1178" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1373.27 &lt;= EMA21 1392.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D1179" t="n">
+        <v>418</v>
+      </c>
+      <c r="E1179" t="n">
+        <v>437.66</v>
+      </c>
+      <c r="F1179" t="n">
+        <v>437.66</v>
+      </c>
+      <c r="G1179" t="n">
+        <v>420.5</v>
+      </c>
+      <c r="H1179" t="n">
+        <v>415.63</v>
+      </c>
+      <c r="I1179" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="J1179" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1179" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 418.00 &lt;= Upper 437.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D1180" t="n">
+        <v>5020</v>
+      </c>
+      <c r="E1180" t="n">
+        <v>5304.65</v>
+      </c>
+      <c r="F1180" t="n">
+        <v>5304.65</v>
+      </c>
+      <c r="G1180" t="n">
+        <v>5037.44</v>
+      </c>
+      <c r="H1180" t="n">
+        <v>5127.43</v>
+      </c>
+      <c r="I1180" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J1180" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1180" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5037.44 &lt;= EMA21 5127.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D1181" t="n">
+        <v>640</v>
+      </c>
+      <c r="E1181" t="n">
+        <v>708.08</v>
+      </c>
+      <c r="F1181" t="n">
+        <v>708.08</v>
+      </c>
+      <c r="G1181" t="n">
+        <v>645.4299999999999</v>
+      </c>
+      <c r="H1181" t="n">
+        <v>656.23</v>
+      </c>
+      <c r="I1181" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1181" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1181" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 645.43 &lt;= EMA21 656.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D1182" t="n">
+        <v>9323</v>
+      </c>
+      <c r="E1182" t="n">
+        <v>9743.040000000001</v>
+      </c>
+      <c r="F1182" t="n">
+        <v>9743.040000000001</v>
+      </c>
+      <c r="G1182" t="n">
+        <v>9275.370000000001</v>
+      </c>
+      <c r="H1182" t="n">
+        <v>9092.9</v>
+      </c>
+      <c r="I1182" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1182" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1182" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9323.00 &lt;= Upper 9743.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D1183" t="n">
+        <v>1175</v>
+      </c>
+      <c r="E1183" t="n">
+        <v>1195.94</v>
+      </c>
+      <c r="F1183" t="n">
+        <v>1195.94</v>
+      </c>
+      <c r="G1183" t="n">
+        <v>1156.73</v>
+      </c>
+      <c r="H1183" t="n">
+        <v>1162.96</v>
+      </c>
+      <c r="I1183" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1183" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1183" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1156.73 &lt;= EMA21 1162.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D1184" t="n">
+        <v>7493.5</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>8272.85</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>8272.85</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>7613.1</v>
+      </c>
+      <c r="H1184" t="n">
+        <v>7737.81</v>
+      </c>
+      <c r="I1184" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J1184" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1184" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7613.10 &lt;= EMA21 7737.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D1185" t="n">
+        <v>322.35</v>
+      </c>
+      <c r="E1185" t="n">
+        <v>332.91</v>
+      </c>
+      <c r="F1185" t="n">
+        <v>332.91</v>
+      </c>
+      <c r="G1185" t="n">
+        <v>321.2</v>
+      </c>
+      <c r="H1185" t="n">
+        <v>320.79</v>
+      </c>
+      <c r="I1185" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="J1185" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1185" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 322.35 &lt;= Upper 332.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D1186" t="n">
+        <v>172</v>
+      </c>
+      <c r="E1186" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="F1186" t="n">
+        <v>176.99</v>
+      </c>
+      <c r="G1186" t="n">
+        <v>172.72</v>
+      </c>
+      <c r="H1186" t="n">
+        <v>173.24</v>
+      </c>
+      <c r="I1186" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="J1186" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1186" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 172.72 &lt;= EMA21 173.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D1187" t="n">
+        <v>873</v>
+      </c>
+      <c r="E1187" t="n">
+        <v>945.24</v>
+      </c>
+      <c r="F1187" t="n">
+        <v>945.24</v>
+      </c>
+      <c r="G1187" t="n">
+        <v>870.67</v>
+      </c>
+      <c r="H1187" t="n">
+        <v>895.4400000000001</v>
+      </c>
+      <c r="I1187" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J1187" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1187" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 870.67 &lt;= EMA21 895.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D1188" t="n">
+        <v>3173.1</v>
+      </c>
+      <c r="E1188" t="n">
+        <v>3383.96</v>
+      </c>
+      <c r="F1188" t="n">
+        <v>3383.96</v>
+      </c>
+      <c r="G1188" t="n">
+        <v>3239.19</v>
+      </c>
+      <c r="H1188" t="n">
+        <v>3259.04</v>
+      </c>
+      <c r="I1188" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1188" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1188" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3239.19 &lt;= EMA21 3259.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D1189" t="n">
+        <v>1258.3</v>
+      </c>
+      <c r="E1189" t="n">
+        <v>1368.39</v>
+      </c>
+      <c r="F1189" t="n">
+        <v>1368.39</v>
+      </c>
+      <c r="G1189" t="n">
+        <v>1251.74</v>
+      </c>
+      <c r="H1189" t="n">
+        <v>1272.04</v>
+      </c>
+      <c r="I1189" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="J1189" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1189" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1251.74 &lt;= EMA21 1272.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D1190" t="n">
+        <v>2387.7</v>
+      </c>
+      <c r="E1190" t="n">
+        <v>2721.14</v>
+      </c>
+      <c r="F1190" t="n">
+        <v>2721.14</v>
+      </c>
+      <c r="G1190" t="n">
+        <v>2425.4</v>
+      </c>
+      <c r="H1190" t="n">
+        <v>2479.75</v>
+      </c>
+      <c r="I1190" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J1190" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1190" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2425.40 &lt;= EMA21 2479.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D1191" t="n">
+        <v>713</v>
+      </c>
+      <c r="E1191" t="n">
+        <v>734.65</v>
+      </c>
+      <c r="F1191" t="n">
+        <v>734.65</v>
+      </c>
+      <c r="G1191" t="n">
+        <v>710.85</v>
+      </c>
+      <c r="H1191" t="n">
+        <v>714.65</v>
+      </c>
+      <c r="I1191" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J1191" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1191" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 710.85 &lt;= EMA21 714.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D1192" t="n">
+        <v>557</v>
+      </c>
+      <c r="E1192" t="n">
+        <v>563.39</v>
+      </c>
+      <c r="F1192" t="n">
+        <v>563.39</v>
+      </c>
+      <c r="G1192" t="n">
+        <v>534.4400000000001</v>
+      </c>
+      <c r="H1192" t="n">
+        <v>536.76</v>
+      </c>
+      <c r="I1192" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="J1192" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1192" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 534.44 &lt;= EMA21 536.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D1193" t="n">
+        <v>980.5</v>
+      </c>
+      <c r="E1193" t="n">
+        <v>1068.73</v>
+      </c>
+      <c r="F1193" t="n">
+        <v>1068.73</v>
+      </c>
+      <c r="G1193" t="n">
+        <v>989.25</v>
+      </c>
+      <c r="H1193" t="n">
+        <v>1003.83</v>
+      </c>
+      <c r="I1193" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="J1193" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1193" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 989.25 &lt;= EMA21 1003.83)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D1194" t="n">
+        <v>4788</v>
+      </c>
+      <c r="E1194" t="n">
+        <v>5067.23</v>
+      </c>
+      <c r="F1194" t="n">
+        <v>5067.23</v>
+      </c>
+      <c r="G1194" t="n">
+        <v>4823.78</v>
+      </c>
+      <c r="H1194" t="n">
+        <v>4844.82</v>
+      </c>
+      <c r="I1194" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="J1194" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1194" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4823.78 &lt;= EMA21 4844.82)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D1195" t="n">
+        <v>1942.2</v>
+      </c>
+      <c r="E1195" t="n">
+        <v>2049.68</v>
+      </c>
+      <c r="F1195" t="n">
+        <v>2049.68</v>
+      </c>
+      <c r="G1195" t="n">
+        <v>1951.94</v>
+      </c>
+      <c r="H1195" t="n">
+        <v>1981.27</v>
+      </c>
+      <c r="I1195" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1195" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1195" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1951.94 &lt;= EMA21 1981.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D1196" t="n">
+        <v>572.3</v>
+      </c>
+      <c r="E1196" t="n">
+        <v>626.4</v>
+      </c>
+      <c r="F1196" t="n">
+        <v>626.4</v>
+      </c>
+      <c r="G1196" t="n">
+        <v>578.72</v>
+      </c>
+      <c r="H1196" t="n">
+        <v>582.78</v>
+      </c>
+      <c r="I1196" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J1196" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1196" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 578.72 &lt;= EMA21 582.78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D1197" t="n">
+        <v>2160</v>
+      </c>
+      <c r="E1197" t="n">
+        <v>2270.31</v>
+      </c>
+      <c r="F1197" t="n">
+        <v>2270.31</v>
+      </c>
+      <c r="G1197" t="n">
+        <v>2172.42</v>
+      </c>
+      <c r="H1197" t="n">
+        <v>2178.62</v>
+      </c>
+      <c r="I1197" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="J1197" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1197" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2172.42 &lt;= EMA21 2178.62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D1198" t="n">
+        <v>1347.6</v>
+      </c>
+      <c r="E1198" t="n">
+        <v>1469.95</v>
+      </c>
+      <c r="F1198" t="n">
+        <v>1469.95</v>
+      </c>
+      <c r="G1198" t="n">
+        <v>1375.99</v>
+      </c>
+      <c r="H1198" t="n">
+        <v>1396.23</v>
+      </c>
+      <c r="I1198" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1198" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1198" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1375.99 &lt;= EMA21 1396.23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D1199" t="n">
+        <v>266.2</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>273.22</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>273.22</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>262.66</v>
+      </c>
+      <c r="H1199" t="n">
+        <v>265.41</v>
+      </c>
+      <c r="I1199" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="J1199" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1199" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.66 &lt;= EMA21 265.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D1200" t="n">
+        <v>726.65</v>
+      </c>
+      <c r="E1200" t="n">
+        <v>736.96</v>
+      </c>
+      <c r="F1200" t="n">
+        <v>736.96</v>
+      </c>
+      <c r="G1200" t="n">
+        <v>719.72</v>
+      </c>
+      <c r="H1200" t="n">
+        <v>721.71</v>
+      </c>
+      <c r="I1200" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="J1200" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1200" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 719.72 &lt;= EMA21 721.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D1201" t="n">
+        <v>134.27</v>
+      </c>
+      <c r="E1201" t="n">
+        <v>140.24</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>140.24</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>134.82</v>
+      </c>
+      <c r="H1201" t="n">
+        <v>136.07</v>
+      </c>
+      <c r="I1201" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J1201" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1201" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 134.82 &lt;= EMA21 136.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D1202" t="n">
+        <v>79.31</v>
+      </c>
+      <c r="E1202" t="n">
+        <v>87.65000000000001</v>
+      </c>
+      <c r="F1202" t="n">
+        <v>87.65000000000001</v>
+      </c>
+      <c r="G1202" t="n">
+        <v>80.65000000000001</v>
+      </c>
+      <c r="H1202" t="n">
+        <v>82.63</v>
+      </c>
+      <c r="I1202" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1202" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1202" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 80.65 &lt;= EMA21 82.63)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1203" t="n">
+        <v>1058.6</v>
+      </c>
+      <c r="E1203" t="n">
+        <v>1182.86</v>
+      </c>
+      <c r="F1203" t="n">
+        <v>1182.86</v>
+      </c>
+      <c r="G1203" t="n">
+        <v>1066.87</v>
+      </c>
+      <c r="H1203" t="n">
+        <v>1089.7</v>
+      </c>
+      <c r="I1203" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1203" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1203" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1066.87 &lt;= EMA21 1089.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D1204" t="n">
+        <v>4845</v>
+      </c>
+      <c r="E1204" t="n">
+        <v>5328.98</v>
+      </c>
+      <c r="F1204" t="n">
+        <v>5328.98</v>
+      </c>
+      <c r="G1204" t="n">
+        <v>4902.04</v>
+      </c>
+      <c r="H1204" t="n">
+        <v>5011.05</v>
+      </c>
+      <c r="I1204" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="J1204" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1204" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4902.04 &lt;= EMA21 5011.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D1205" t="n">
+        <v>1253.4</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>1362.41</v>
+      </c>
+      <c r="F1205" t="n">
+        <v>1362.41</v>
+      </c>
+      <c r="G1205" t="n">
+        <v>1269.73</v>
+      </c>
+      <c r="H1205" t="n">
+        <v>1284.22</v>
+      </c>
+      <c r="I1205" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1205" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1205" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1269.73 &lt;= EMA21 1284.22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D1206" t="n">
+        <v>1128.4</v>
+      </c>
+      <c r="E1206" t="n">
+        <v>1196.2</v>
+      </c>
+      <c r="F1206" t="n">
+        <v>1196.2</v>
+      </c>
+      <c r="G1206" t="n">
+        <v>1125.39</v>
+      </c>
+      <c r="H1206" t="n">
+        <v>1129.49</v>
+      </c>
+      <c r="I1206" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1206" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1206" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1125.39 &lt;= EMA21 1129.49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D1207" t="n">
+        <v>229.3</v>
+      </c>
+      <c r="E1207" t="n">
+        <v>248.14</v>
+      </c>
+      <c r="F1207" t="n">
+        <v>248.14</v>
+      </c>
+      <c r="G1207" t="n">
+        <v>230.27</v>
+      </c>
+      <c r="H1207" t="n">
+        <v>235.24</v>
+      </c>
+      <c r="I1207" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J1207" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1207" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 230.27 &lt;= EMA21 235.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D1208" t="n">
+        <v>416.5</v>
+      </c>
+      <c r="E1208" t="n">
+        <v>431.74</v>
+      </c>
+      <c r="F1208" t="n">
+        <v>431.74</v>
+      </c>
+      <c r="G1208" t="n">
+        <v>416.3</v>
+      </c>
+      <c r="H1208" t="n">
+        <v>413.32</v>
+      </c>
+      <c r="I1208" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1208" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1208" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 416.50 &lt;= Upper 431.74)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D1209" t="n">
+        <v>4265.3</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>4706.88</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>4706.88</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>4340.71</v>
+      </c>
+      <c r="H1209" t="n">
+        <v>4415.31</v>
+      </c>
+      <c r="I1209" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J1209" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1209" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4340.71 &lt;= EMA21 4415.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D1210" t="n">
+        <v>3836.2</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>4145.9</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>4145.9</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>3896.23</v>
+      </c>
+      <c r="H1210" t="n">
+        <v>3947.38</v>
+      </c>
+      <c r="I1210" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1210" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1210" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3896.23 &lt;= EMA21 3947.38)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D1211" t="n">
+        <v>1103.1</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>1327.04</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>1327.04</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>1130.95</v>
+      </c>
+      <c r="H1211" t="n">
+        <v>1169.56</v>
+      </c>
+      <c r="I1211" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J1211" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1211" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1130.95 &lt;= EMA21 1169.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D1212" t="n">
+        <v>3076.5</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>3478.31</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>3478.31</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>3112.76</v>
+      </c>
+      <c r="H1212" t="n">
+        <v>3189.51</v>
+      </c>
+      <c r="I1212" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J1212" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1212" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3112.76 &lt;= EMA21 3189.51)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D1213" t="n">
+        <v>12338</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>13937.78</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>13937.78</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>12472.22</v>
+      </c>
+      <c r="H1213" t="n">
+        <v>12836.71</v>
+      </c>
+      <c r="I1213" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="J1213" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1213" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12472.22 &lt;= EMA21 12836.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D1214" t="n">
+        <v>1037</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>1050.6</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>1050.6</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>1024.91</v>
+      </c>
+      <c r="H1214" t="n">
+        <v>1023.93</v>
+      </c>
+      <c r="I1214" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J1214" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1214" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1037.00 &lt;= Upper 1050.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D1215" t="n">
+        <v>2210</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>2704.6</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>2704.6</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>2322.76</v>
+      </c>
+      <c r="H1215" t="n">
+        <v>2402.15</v>
+      </c>
+      <c r="I1215" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="J1215" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1215" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2322.76 &lt;= EMA21 2402.15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D1216" t="n">
+        <v>2770.2</v>
+      </c>
+      <c r="E1216" t="n">
+        <v>3245.27</v>
+      </c>
+      <c r="F1216" t="n">
+        <v>3245.27</v>
+      </c>
+      <c r="G1216" t="n">
+        <v>2821.06</v>
+      </c>
+      <c r="H1216" t="n">
+        <v>2887.76</v>
+      </c>
+      <c r="I1216" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1216" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1216" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2821.06 &lt;= EMA21 2887.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D1217" t="n">
+        <v>329.6</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>338.63</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>338.63</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>330.69</v>
+      </c>
+      <c r="H1217" t="n">
+        <v>332.05</v>
+      </c>
+      <c r="I1217" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J1217" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1217" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 330.69 &lt;= EMA21 332.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D1218" t="n">
+        <v>1370.6</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>1502.63</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>1502.63</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>1387.92</v>
+      </c>
+      <c r="H1218" t="n">
+        <v>1414.9</v>
+      </c>
+      <c r="I1218" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1218" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1218" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1387.92 &lt;= EMA21 1414.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D1219" t="n">
+        <v>232.43</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>238.22</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>238.22</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>234.45</v>
+      </c>
+      <c r="H1219" t="n">
+        <v>235.07</v>
+      </c>
+      <c r="I1219" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="J1219" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1219" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.45 &lt;= EMA21 235.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D1220" t="n">
+        <v>1551.5</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>1704.61</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>1704.61</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>1566.59</v>
+      </c>
+      <c r="H1220" t="n">
+        <v>1596.24</v>
+      </c>
+      <c r="I1220" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="J1220" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1220" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1566.59 &lt;= EMA21 1596.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D1221" t="n">
+        <v>344.95</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>365.22</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>365.22</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>349.14</v>
+      </c>
+      <c r="H1221" t="n">
+        <v>355.91</v>
+      </c>
+      <c r="I1221" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1221" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1221" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 349.14 &lt;= EMA21 355.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D1222" t="n">
+        <v>263.75</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>272.75</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>272.75</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>265.59</v>
+      </c>
+      <c r="H1222" t="n">
+        <v>267.39</v>
+      </c>
+      <c r="I1222" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J1222" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1222" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 265.59 &lt;= EMA21 267.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D1223" t="n">
+        <v>116.47</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>117.65</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>117.65</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>116.24</v>
+      </c>
+      <c r="H1223" t="n">
+        <v>115.9</v>
+      </c>
+      <c r="I1223" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1223" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1223" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 116.47 &lt;= Upper 117.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D1224" t="n">
+        <v>310.5</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>328.4</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>328.4</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>313.22</v>
+      </c>
+      <c r="H1224" t="n">
+        <v>319.77</v>
+      </c>
+      <c r="I1224" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1224" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1224" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 313.22 &lt;= EMA21 319.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D1225" t="n">
+        <v>1243.9</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>1341.33</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>1341.33</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>1261.18</v>
+      </c>
+      <c r="H1225" t="n">
+        <v>1279.7</v>
+      </c>
+      <c r="I1225" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1225" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1225" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1261.18 &lt;= EMA21 1279.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D1226" t="n">
+        <v>1766.9</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>1808.02</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>1808.02</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>1711.52</v>
+      </c>
+      <c r="H1226" t="n">
+        <v>1733.5</v>
+      </c>
+      <c r="I1226" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="J1226" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1226" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1711.52 &lt;= EMA21 1733.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D1227" t="n">
+        <v>161.87</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>170.77</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>170.77</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>161.92</v>
+      </c>
+      <c r="H1227" t="n">
+        <v>162.67</v>
+      </c>
+      <c r="I1227" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1227" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1227" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 161.92 &lt;= EMA21 162.67)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D1228" t="n">
+        <v>21960</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>25255.68</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>25255.68</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>22579.45</v>
+      </c>
+      <c r="H1228" t="n">
+        <v>23408.39</v>
+      </c>
+      <c r="I1228" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J1228" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1228" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 22579.45 &lt;= EMA21 23408.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D1229" t="n">
+        <v>995</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>1154.73</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>1154.73</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>1014.57</v>
+      </c>
+      <c r="H1229" t="n">
+        <v>1043.12</v>
+      </c>
+      <c r="I1229" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J1229" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1229" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1014.57 &lt;= EMA21 1043.12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D1230" t="n">
+        <v>3109.1</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>3453.56</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>3453.56</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>3124.6</v>
+      </c>
+      <c r="H1230" t="n">
+        <v>3202.97</v>
+      </c>
+      <c r="I1230" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="J1230" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1230" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3124.60 &lt;= EMA21 3202.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D1231" t="n">
+        <v>3763.5</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>4187.57</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>4187.57</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>3866.39</v>
+      </c>
+      <c r="H1231" t="n">
+        <v>3913.17</v>
+      </c>
+      <c r="I1231" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J1231" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1231" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3866.39 &lt;= EMA21 3913.17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D1232" t="n">
+        <v>18815</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>23206</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>23206</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>20445.72</v>
+      </c>
+      <c r="H1232" t="n">
+        <v>20519.16</v>
+      </c>
+      <c r="I1232" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="J1232" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1232" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 20445.72 &lt;= EMA21 20519.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D1233" t="n">
+        <v>988.7</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>1071.44</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>1071.44</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>997.28</v>
+      </c>
+      <c r="H1233" t="n">
+        <v>1014.46</v>
+      </c>
+      <c r="I1233" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="J1233" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1233" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 997.28 &lt;= EMA21 1014.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D1234" t="n">
+        <v>1867.3</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>1969.26</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>1969.26</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>1864.24</v>
+      </c>
+      <c r="H1234" t="n">
+        <v>1885.57</v>
+      </c>
+      <c r="I1234" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1234" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1234" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1864.24 &lt;= EMA21 1885.57)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D1235" t="n">
+        <v>4101.7</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>4488.06</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>4488.06</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>4115.44</v>
+      </c>
+      <c r="H1235" t="n">
+        <v>4171.77</v>
+      </c>
+      <c r="I1235" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="J1235" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1235" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4115.44 &lt;= EMA21 4171.77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D1236" t="n">
+        <v>343.65</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>382.65</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>382.65</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>356.16</v>
+      </c>
+      <c r="H1236" t="n">
+        <v>361.27</v>
+      </c>
+      <c r="I1236" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1236" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1236" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 356.16 &lt;= EMA21 361.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D1237" t="n">
+        <v>2190</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>2398.28</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>2398.28</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>2225.22</v>
+      </c>
+      <c r="H1237" t="n">
+        <v>2261.27</v>
+      </c>
+      <c r="I1237" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1237" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1237" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2225.22 &lt;= EMA21 2261.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D1238" t="n">
+        <v>1013.7</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>1068.36</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>1068.36</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>1004.55</v>
+      </c>
+      <c r="H1238" t="n">
+        <v>1021.58</v>
+      </c>
+      <c r="I1238" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J1238" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1238" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1004.55 &lt;= EMA21 1021.58)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D1239" t="n">
+        <v>436.1</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>491.06</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>491.06</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>438.73</v>
+      </c>
+      <c r="H1239" t="n">
+        <v>447.39</v>
+      </c>
+      <c r="I1239" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1239" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1239" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 438.73 &lt;= EMA21 447.39)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D1240" t="n">
+        <v>314.5</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>321.59</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>321.59</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>306.32</v>
+      </c>
+      <c r="H1240" t="n">
+        <v>311.56</v>
+      </c>
+      <c r="I1240" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="J1240" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1240" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 306.32 &lt;= EMA21 311.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D1241" t="n">
+        <v>369</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>378.84</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>378.84</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>364.9</v>
+      </c>
+      <c r="H1241" t="n">
+        <v>366.42</v>
+      </c>
+      <c r="I1241" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J1241" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1241" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 364.90 &lt;= EMA21 366.42)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D1242" t="n">
+        <v>187.29</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>189.4</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>189.4</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>185</v>
+      </c>
+      <c r="H1242" t="n">
+        <v>185.41</v>
+      </c>
+      <c r="I1242" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="J1242" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1242" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.00 &lt;= EMA21 185.41)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D1243" t="n">
+        <v>1561</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>1652.25</v>
+      </c>
+      <c r="F1243" t="n">
+        <v>1652.25</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>1562.1</v>
+      </c>
+      <c r="H1243" t="n">
+        <v>1575.9</v>
+      </c>
+      <c r="I1243" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1243" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1243" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1562.10 &lt;= EMA21 1575.90)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D1244" t="n">
+        <v>4841</v>
+      </c>
+      <c r="E1244" t="n">
+        <v>5204.22</v>
+      </c>
+      <c r="F1244" t="n">
+        <v>5204.22</v>
+      </c>
+      <c r="G1244" t="n">
+        <v>4946.67</v>
+      </c>
+      <c r="H1244" t="n">
+        <v>4983.16</v>
+      </c>
+      <c r="I1244" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J1244" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1244" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4946.67 &lt;= EMA21 4983.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D1245" t="n">
+        <v>4875</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>5065.23</v>
+      </c>
+      <c r="F1245" t="n">
+        <v>5065.23</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>4899.47</v>
+      </c>
+      <c r="H1245" t="n">
+        <v>4921.32</v>
+      </c>
+      <c r="I1245" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J1245" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1245" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4899.47 &lt;= EMA21 4921.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D1246" t="n">
+        <v>2789</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>2952.17</v>
+      </c>
+      <c r="F1246" t="n">
+        <v>2952.17</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>2796.59</v>
+      </c>
+      <c r="H1246" t="n">
+        <v>2841.7</v>
+      </c>
+      <c r="I1246" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1246" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1246" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2796.59 &lt;= EMA21 2841.70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D1247" t="n">
+        <v>10764</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>11910.18</v>
+      </c>
+      <c r="F1247" t="n">
+        <v>11910.18</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>10927.5</v>
+      </c>
+      <c r="H1247" t="n">
+        <v>11169.32</v>
+      </c>
+      <c r="I1247" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J1247" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1247" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 10927.50 &lt;= EMA21 11169.32)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D1248" t="n">
+        <v>178.09</v>
+      </c>
+      <c r="E1248" t="n">
+        <v>191.79</v>
+      </c>
+      <c r="F1248" t="n">
+        <v>191.79</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>179.73</v>
+      </c>
+      <c r="H1248" t="n">
+        <v>181.46</v>
+      </c>
+      <c r="I1248" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="J1248" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1248" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 179.73 &lt;= EMA21 181.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D1249" t="n">
+        <v>1390</v>
+      </c>
+      <c r="E1249" t="n">
+        <v>1587.59</v>
+      </c>
+      <c r="F1249" t="n">
+        <v>1587.59</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>1407.69</v>
+      </c>
+      <c r="H1249" t="n">
+        <v>1442.76</v>
+      </c>
+      <c r="I1249" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J1249" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1249" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1407.69 &lt;= EMA21 1442.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D1250" t="n">
+        <v>415.45</v>
+      </c>
+      <c r="E1250" t="n">
+        <v>433.03</v>
+      </c>
+      <c r="F1250" t="n">
+        <v>433.03</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>412.39</v>
+      </c>
+      <c r="H1250" t="n">
+        <v>417.34</v>
+      </c>
+      <c r="I1250" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J1250" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1250" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 412.39 &lt;= EMA21 417.34)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D1251" t="n">
+        <v>257.45</v>
+      </c>
+      <c r="E1251" t="n">
+        <v>289.5</v>
+      </c>
+      <c r="F1251" t="n">
+        <v>289.5</v>
+      </c>
+      <c r="G1251" t="n">
+        <v>263.12</v>
+      </c>
+      <c r="H1251" t="n">
+        <v>267.81</v>
+      </c>
+      <c r="I1251" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="J1251" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1251" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 263.12 &lt;= EMA21 267.81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D1252" t="n">
+        <v>166.4</v>
+      </c>
+      <c r="E1252" t="n">
+        <v>186.66</v>
+      </c>
+      <c r="F1252" t="n">
+        <v>186.66</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>169.23</v>
+      </c>
+      <c r="H1252" t="n">
+        <v>173.1</v>
+      </c>
+      <c r="I1252" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1252" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1252" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 169.23 &lt;= EMA21 173.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D1253" t="n">
+        <v>1135.1</v>
+      </c>
+      <c r="E1253" t="n">
+        <v>1190.72</v>
+      </c>
+      <c r="F1253" t="n">
+        <v>1190.72</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>1124.24</v>
+      </c>
+      <c r="H1253" t="n">
+        <v>1131.05</v>
+      </c>
+      <c r="I1253" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1253" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1253" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1124.24 &lt;= EMA21 1131.05)</t>
         </is>
       </c>
     </row>
@@ -50319,7 +54619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -50376,47 +54676,6 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>418.85</v>
-      </c>
-      <c r="D2" t="n">
-        <v>47</v>
-      </c>
-      <c r="E2" t="n">
-        <v>19685.95</v>
-      </c>
-      <c r="F2" t="n">
-        <v>422.25</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="H2" t="n">
-        <v>416.67</v>
-      </c>
-      <c r="I2" t="n">
-        <v>436.2999877929688</v>
-      </c>
-      <c r="J2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
         </is>
       </c>
     </row>
@@ -50431,7 +54690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51465,6 +55724,57 @@
         <v>5</v>
       </c>
       <c r="M21" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>418.85</v>
+      </c>
+      <c r="E22" t="n">
+        <v>416.67</v>
+      </c>
+      <c r="F22" t="n">
+        <v>47</v>
+      </c>
+      <c r="G22" t="n">
+        <v>19685.95</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="J22" t="n">
+        <v>-161.42</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>7</v>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
@@ -51481,7 +55791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K150"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56863,6 +61173,55 @@
         </is>
       </c>
       <c r="K150" t="inlineStr">
+        <is>
+          <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-17 20:31:27</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>EDF9249AD8</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>416.67</v>
+      </c>
+      <c r="G151" t="n">
+        <v>416.67</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>47</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
         <is>
           <t>HARD_STOP_LOSS</t>
         </is>
@@ -56947,7 +61306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57492,6 +61851,39 @@
         <v>1</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20:31:28</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>196116.98</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>196116.98</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-3797.38</v>
+      </c>
+      <c r="G17" t="n">
+        <v>19</v>
+      </c>
+      <c r="H17" t="n">
+        <v>21</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: bot run 2026-09-18T20:02 IST
</commit_message>
<xml_diff>
--- a/data/trade_log_india.xlsx
+++ b/data/trade_log_india.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1253"/>
+  <dimension ref="A1:K1353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54306,6 +54306,4306 @@
       <c r="K1253" t="inlineStr">
         <is>
           <t>EMA_BEARISH (EMA9 1124.24 &lt;= EMA21 1131.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D1254" t="n">
+        <v>7270.5</v>
+      </c>
+      <c r="E1254" t="n">
+        <v>7739.4</v>
+      </c>
+      <c r="F1254" t="n">
+        <v>7739.4</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>7239.45</v>
+      </c>
+      <c r="H1254" t="n">
+        <v>7339.97</v>
+      </c>
+      <c r="I1254" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="J1254" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1254" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7239.45 &lt;= EMA21 7339.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>ADANIENSOL</t>
+        </is>
+      </c>
+      <c r="D1255" t="n">
+        <v>1436.1</v>
+      </c>
+      <c r="E1255" t="n">
+        <v>1617.03</v>
+      </c>
+      <c r="F1255" t="n">
+        <v>1617.03</v>
+      </c>
+      <c r="G1255" t="n">
+        <v>1396.14</v>
+      </c>
+      <c r="H1255" t="n">
+        <v>1439.31</v>
+      </c>
+      <c r="I1255" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J1255" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1255" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1396.14 &lt;= EMA21 1439.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>ADANIENT</t>
+        </is>
+      </c>
+      <c r="D1256" t="n">
+        <v>3020</v>
+      </c>
+      <c r="E1256" t="n">
+        <v>3201.45</v>
+      </c>
+      <c r="F1256" t="n">
+        <v>3201.45</v>
+      </c>
+      <c r="G1256" t="n">
+        <v>2984.34</v>
+      </c>
+      <c r="H1256" t="n">
+        <v>2995.21</v>
+      </c>
+      <c r="I1256" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J1256" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1256" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2984.34 &lt;= EMA21 2995.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>ADANIGREEN</t>
+        </is>
+      </c>
+      <c r="D1257" t="n">
+        <v>1334.5</v>
+      </c>
+      <c r="E1257" t="n">
+        <v>1351.11</v>
+      </c>
+      <c r="F1257" t="n">
+        <v>1351.11</v>
+      </c>
+      <c r="G1257" t="n">
+        <v>1291.95</v>
+      </c>
+      <c r="H1257" t="n">
+        <v>1302.6</v>
+      </c>
+      <c r="I1257" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="J1257" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1257" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1291.95 &lt;= EMA21 1302.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D1258" t="n">
+        <v>1824</v>
+      </c>
+      <c r="E1258" t="n">
+        <v>1815.32</v>
+      </c>
+      <c r="F1258" t="n">
+        <v>1815.32</v>
+      </c>
+      <c r="G1258" t="n">
+        <v>1750.1</v>
+      </c>
+      <c r="H1258" t="n">
+        <v>1729.09</v>
+      </c>
+      <c r="I1258" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="J1258" t="b">
+        <v>1</v>
+      </c>
+      <c r="K1258" t="inlineStr">
+        <is>
+          <t>QUALIFIED_BREAKOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>ADANIPOWER</t>
+        </is>
+      </c>
+      <c r="D1259" t="n">
+        <v>206.6</v>
+      </c>
+      <c r="E1259" t="n">
+        <v>216.28</v>
+      </c>
+      <c r="F1259" t="n">
+        <v>216.28</v>
+      </c>
+      <c r="G1259" t="n">
+        <v>206.72</v>
+      </c>
+      <c r="H1259" t="n">
+        <v>207.46</v>
+      </c>
+      <c r="I1259" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="J1259" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1259" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 206.72 &lt;= EMA21 207.46)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>AMBUJACEM</t>
+        </is>
+      </c>
+      <c r="D1260" t="n">
+        <v>388.3</v>
+      </c>
+      <c r="E1260" t="n">
+        <v>420.99</v>
+      </c>
+      <c r="F1260" t="n">
+        <v>420.99</v>
+      </c>
+      <c r="G1260" t="n">
+        <v>389.8</v>
+      </c>
+      <c r="H1260" t="n">
+        <v>398.5</v>
+      </c>
+      <c r="I1260" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="J1260" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1260" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 389.80 &lt;= EMA21 398.50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="D1261" t="n">
+        <v>8944.5</v>
+      </c>
+      <c r="E1261" t="n">
+        <v>8979.75</v>
+      </c>
+      <c r="F1261" t="n">
+        <v>8979.75</v>
+      </c>
+      <c r="G1261" t="n">
+        <v>8813.51</v>
+      </c>
+      <c r="H1261" t="n">
+        <v>8804.219999999999</v>
+      </c>
+      <c r="I1261" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J1261" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1261" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 8944.50 &lt;= Upper 8979.75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="D1262" t="n">
+        <v>2451.3</v>
+      </c>
+      <c r="E1262" t="n">
+        <v>2690.21</v>
+      </c>
+      <c r="F1262" t="n">
+        <v>2690.21</v>
+      </c>
+      <c r="G1262" t="n">
+        <v>2465.87</v>
+      </c>
+      <c r="H1262" t="n">
+        <v>2523.59</v>
+      </c>
+      <c r="I1262" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="J1262" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1262" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2465.87 &lt;= EMA21 2523.59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>DMART</t>
+        </is>
+      </c>
+      <c r="D1263" t="n">
+        <v>3749.9</v>
+      </c>
+      <c r="E1263" t="n">
+        <v>3937.41</v>
+      </c>
+      <c r="F1263" t="n">
+        <v>3937.41</v>
+      </c>
+      <c r="G1263" t="n">
+        <v>3726.6</v>
+      </c>
+      <c r="H1263" t="n">
+        <v>3780.47</v>
+      </c>
+      <c r="I1263" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J1263" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1263" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3726.60 &lt;= EMA21 3780.47)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
+      <c r="D1264" t="n">
+        <v>1257</v>
+      </c>
+      <c r="E1264" t="n">
+        <v>1286.14</v>
+      </c>
+      <c r="F1264" t="n">
+        <v>1286.14</v>
+      </c>
+      <c r="G1264" t="n">
+        <v>1246.16</v>
+      </c>
+      <c r="H1264" t="n">
+        <v>1248.96</v>
+      </c>
+      <c r="I1264" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1264" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1264" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1246.16 &lt;= EMA21 1248.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="D1265" t="n">
+        <v>11414</v>
+      </c>
+      <c r="E1265" t="n">
+        <v>12267.16</v>
+      </c>
+      <c r="F1265" t="n">
+        <v>12267.16</v>
+      </c>
+      <c r="G1265" t="n">
+        <v>11641.32</v>
+      </c>
+      <c r="H1265" t="n">
+        <v>11697.89</v>
+      </c>
+      <c r="I1265" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="J1265" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1265" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11641.32 &lt;= EMA21 11697.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>BAJFINANCE</t>
+        </is>
+      </c>
+      <c r="D1266" t="n">
+        <v>1040.3</v>
+      </c>
+      <c r="E1266" t="n">
+        <v>1104.35</v>
+      </c>
+      <c r="F1266" t="n">
+        <v>1104.35</v>
+      </c>
+      <c r="G1266" t="n">
+        <v>1034.57</v>
+      </c>
+      <c r="H1266" t="n">
+        <v>1050</v>
+      </c>
+      <c r="I1266" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="J1266" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1266" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1034.57 &lt;= EMA21 1050.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>BAJAJFINSV</t>
+        </is>
+      </c>
+      <c r="D1267" t="n">
+        <v>1852.5</v>
+      </c>
+      <c r="E1267" t="n">
+        <v>2073.76</v>
+      </c>
+      <c r="F1267" t="n">
+        <v>2073.76</v>
+      </c>
+      <c r="G1267" t="n">
+        <v>1896.74</v>
+      </c>
+      <c r="H1267" t="n">
+        <v>1936.13</v>
+      </c>
+      <c r="I1267" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1267" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1267" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1896.74 &lt;= EMA21 1936.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="D1268" t="n">
+        <v>11282</v>
+      </c>
+      <c r="E1268" t="n">
+        <v>11576.34</v>
+      </c>
+      <c r="F1268" t="n">
+        <v>11576.34</v>
+      </c>
+      <c r="G1268" t="n">
+        <v>11123.53</v>
+      </c>
+      <c r="H1268" t="n">
+        <v>11164.1</v>
+      </c>
+      <c r="I1268" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="J1268" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1268" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 11123.53 &lt;= EMA21 11164.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
+      <c r="D1269" t="n">
+        <v>234.94</v>
+      </c>
+      <c r="E1269" t="n">
+        <v>245.55</v>
+      </c>
+      <c r="F1269" t="n">
+        <v>245.55</v>
+      </c>
+      <c r="G1269" t="n">
+        <v>236.29</v>
+      </c>
+      <c r="H1269" t="n">
+        <v>238.88</v>
+      </c>
+      <c r="I1269" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J1269" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1269" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 236.29 &lt;= EMA21 238.88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="D1270" t="n">
+        <v>393.3</v>
+      </c>
+      <c r="E1270" t="n">
+        <v>421.79</v>
+      </c>
+      <c r="F1270" t="n">
+        <v>421.79</v>
+      </c>
+      <c r="G1270" t="n">
+        <v>396.92</v>
+      </c>
+      <c r="H1270" t="n">
+        <v>401.53</v>
+      </c>
+      <c r="I1270" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J1270" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1270" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 396.92 &lt;= EMA21 401.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>BPCL</t>
+        </is>
+      </c>
+      <c r="D1271" t="n">
+        <v>314</v>
+      </c>
+      <c r="E1271" t="n">
+        <v>327.02</v>
+      </c>
+      <c r="F1271" t="n">
+        <v>327.02</v>
+      </c>
+      <c r="G1271" t="n">
+        <v>307.58</v>
+      </c>
+      <c r="H1271" t="n">
+        <v>310.1</v>
+      </c>
+      <c r="I1271" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="J1271" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1271" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 307.58 &lt;= EMA21 310.10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="D1272" t="n">
+        <v>1893.3</v>
+      </c>
+      <c r="E1272" t="n">
+        <v>1935.45</v>
+      </c>
+      <c r="F1272" t="n">
+        <v>1935.45</v>
+      </c>
+      <c r="G1272" t="n">
+        <v>1850.12</v>
+      </c>
+      <c r="H1272" t="n">
+        <v>1864.45</v>
+      </c>
+      <c r="I1272" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="J1272" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1272" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1850.12 &lt;= EMA21 1864.45)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="D1273" t="n">
+        <v>47000</v>
+      </c>
+      <c r="E1273" t="n">
+        <v>49924.92</v>
+      </c>
+      <c r="F1273" t="n">
+        <v>49924.92</v>
+      </c>
+      <c r="G1273" t="n">
+        <v>47790.42</v>
+      </c>
+      <c r="H1273" t="n">
+        <v>47481.78</v>
+      </c>
+      <c r="I1273" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="J1273" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1273" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 47000.00 &lt;= Upper 49924.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="D1274" t="n">
+        <v>4998</v>
+      </c>
+      <c r="E1274" t="n">
+        <v>5407.96</v>
+      </c>
+      <c r="F1274" t="n">
+        <v>5407.96</v>
+      </c>
+      <c r="G1274" t="n">
+        <v>5017.18</v>
+      </c>
+      <c r="H1274" t="n">
+        <v>5120.69</v>
+      </c>
+      <c r="I1274" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J1274" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1274" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5017.18 &lt;= EMA21 5120.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>CGPOWER</t>
+        </is>
+      </c>
+      <c r="D1275" t="n">
+        <v>892</v>
+      </c>
+      <c r="E1275" t="n">
+        <v>930.9400000000001</v>
+      </c>
+      <c r="F1275" t="n">
+        <v>930.9400000000001</v>
+      </c>
+      <c r="G1275" t="n">
+        <v>886.9</v>
+      </c>
+      <c r="H1275" t="n">
+        <v>888.96</v>
+      </c>
+      <c r="I1275" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1275" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1275" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 886.90 &lt;= EMA21 888.96)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
+      <c r="D1276" t="n">
+        <v>123.78</v>
+      </c>
+      <c r="E1276" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="F1276" t="n">
+        <v>129.6</v>
+      </c>
+      <c r="G1276" t="n">
+        <v>124.04</v>
+      </c>
+      <c r="H1276" t="n">
+        <v>125.33</v>
+      </c>
+      <c r="I1276" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1276" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1276" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 124.04 &lt;= EMA21 125.33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>CHOLAFIN</t>
+        </is>
+      </c>
+      <c r="D1277" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E1277" t="n">
+        <v>1896.89</v>
+      </c>
+      <c r="F1277" t="n">
+        <v>1896.89</v>
+      </c>
+      <c r="G1277" t="n">
+        <v>1816.38</v>
+      </c>
+      <c r="H1277" t="n">
+        <v>1833.07</v>
+      </c>
+      <c r="I1277" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="J1277" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1277" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1816.38 &lt;= EMA21 1833.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="D1278" t="n">
+        <v>1394.5</v>
+      </c>
+      <c r="E1278" t="n">
+        <v>1448.89</v>
+      </c>
+      <c r="F1278" t="n">
+        <v>1448.89</v>
+      </c>
+      <c r="G1278" t="n">
+        <v>1376.42</v>
+      </c>
+      <c r="H1278" t="n">
+        <v>1393.43</v>
+      </c>
+      <c r="I1278" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="J1278" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1278" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1376.42 &lt;= EMA21 1393.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="D1279" t="n">
+        <v>409.9</v>
+      </c>
+      <c r="E1279" t="n">
+        <v>437.56</v>
+      </c>
+      <c r="F1279" t="n">
+        <v>437.56</v>
+      </c>
+      <c r="G1279" t="n">
+        <v>418.38</v>
+      </c>
+      <c r="H1279" t="n">
+        <v>415.11</v>
+      </c>
+      <c r="I1279" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J1279" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1279" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 409.90 &lt;= Upper 437.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="D1280" t="n">
+        <v>5099.5</v>
+      </c>
+      <c r="E1280" t="n">
+        <v>5277.99</v>
+      </c>
+      <c r="F1280" t="n">
+        <v>5277.99</v>
+      </c>
+      <c r="G1280" t="n">
+        <v>5043.59</v>
+      </c>
+      <c r="H1280" t="n">
+        <v>5110.26</v>
+      </c>
+      <c r="I1280" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J1280" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1280" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 5043.59 &lt;= EMA21 5110.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>DLF</t>
+        </is>
+      </c>
+      <c r="D1281" t="n">
+        <v>644.35</v>
+      </c>
+      <c r="E1281" t="n">
+        <v>706.67</v>
+      </c>
+      <c r="F1281" t="n">
+        <v>706.67</v>
+      </c>
+      <c r="G1281" t="n">
+        <v>645.05</v>
+      </c>
+      <c r="H1281" t="n">
+        <v>655.16</v>
+      </c>
+      <c r="I1281" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="J1281" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1281" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 645.05 &lt;= EMA21 655.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>DIVISLAB</t>
+        </is>
+      </c>
+      <c r="D1282" t="n">
+        <v>9375</v>
+      </c>
+      <c r="E1282" t="n">
+        <v>9718.200000000001</v>
+      </c>
+      <c r="F1282" t="n">
+        <v>9718.200000000001</v>
+      </c>
+      <c r="G1282" t="n">
+        <v>9295.299999999999</v>
+      </c>
+      <c r="H1282" t="n">
+        <v>9118.549999999999</v>
+      </c>
+      <c r="I1282" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="J1282" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1282" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 9375.00 &lt;= Upper 9718.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="D1283" t="n">
+        <v>1185</v>
+      </c>
+      <c r="E1283" t="n">
+        <v>1197.5</v>
+      </c>
+      <c r="F1283" t="n">
+        <v>1197.5</v>
+      </c>
+      <c r="G1283" t="n">
+        <v>1158.73</v>
+      </c>
+      <c r="H1283" t="n">
+        <v>1163.87</v>
+      </c>
+      <c r="I1283" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="J1283" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1283" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1158.73 &lt;= EMA21 1163.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="D1284" t="n">
+        <v>7516</v>
+      </c>
+      <c r="E1284" t="n">
+        <v>8207.27</v>
+      </c>
+      <c r="F1284" t="n">
+        <v>8207.27</v>
+      </c>
+      <c r="G1284" t="n">
+        <v>7572.15</v>
+      </c>
+      <c r="H1284" t="n">
+        <v>7690.98</v>
+      </c>
+      <c r="I1284" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1284" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1284" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 7572.15 &lt;= EMA21 7690.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>ETERNAL</t>
+        </is>
+      </c>
+      <c r="D1285" t="n">
+        <v>326.85</v>
+      </c>
+      <c r="E1285" t="n">
+        <v>332.43</v>
+      </c>
+      <c r="F1285" t="n">
+        <v>332.43</v>
+      </c>
+      <c r="G1285" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="H1285" t="n">
+        <v>321.33</v>
+      </c>
+      <c r="I1285" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="J1285" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1285" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 326.85 &lt;= Upper 332.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>GAIL</t>
+        </is>
+      </c>
+      <c r="D1286" t="n">
+        <v>173.9</v>
+      </c>
+      <c r="E1286" t="n">
+        <v>177</v>
+      </c>
+      <c r="F1286" t="n">
+        <v>177</v>
+      </c>
+      <c r="G1286" t="n">
+        <v>172.95</v>
+      </c>
+      <c r="H1286" t="n">
+        <v>173.3</v>
+      </c>
+      <c r="I1286" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J1286" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1286" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 172.95 &lt;= EMA21 173.30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>GODREJCP</t>
+        </is>
+      </c>
+      <c r="D1287" t="n">
+        <v>880</v>
+      </c>
+      <c r="E1287" t="n">
+        <v>945.22</v>
+      </c>
+      <c r="F1287" t="n">
+        <v>945.22</v>
+      </c>
+      <c r="G1287" t="n">
+        <v>872.0700000000001</v>
+      </c>
+      <c r="H1287" t="n">
+        <v>896.0700000000001</v>
+      </c>
+      <c r="I1287" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J1287" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1287" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 872.07 &lt;= EMA21 896.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="D1288" t="n">
+        <v>3209.2</v>
+      </c>
+      <c r="E1288" t="n">
+        <v>3378.75</v>
+      </c>
+      <c r="F1288" t="n">
+        <v>3378.75</v>
+      </c>
+      <c r="G1288" t="n">
+        <v>3246.29</v>
+      </c>
+      <c r="H1288" t="n">
+        <v>3263.28</v>
+      </c>
+      <c r="I1288" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="J1288" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1288" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3246.29 &lt;= EMA21 3263.28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="D1289" t="n">
+        <v>1249.3</v>
+      </c>
+      <c r="E1289" t="n">
+        <v>1366.2</v>
+      </c>
+      <c r="F1289" t="n">
+        <v>1366.2</v>
+      </c>
+      <c r="G1289" t="n">
+        <v>1251.25</v>
+      </c>
+      <c r="H1289" t="n">
+        <v>1269.97</v>
+      </c>
+      <c r="I1289" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="J1289" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1289" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1251.25 &lt;= EMA21 1269.97)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>HDFCAMC</t>
+        </is>
+      </c>
+      <c r="D1290" t="n">
+        <v>2425</v>
+      </c>
+      <c r="E1290" t="n">
+        <v>2706.11</v>
+      </c>
+      <c r="F1290" t="n">
+        <v>2706.11</v>
+      </c>
+      <c r="G1290" t="n">
+        <v>2429.14</v>
+      </c>
+      <c r="H1290" t="n">
+        <v>2477.61</v>
+      </c>
+      <c r="I1290" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="J1290" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1290" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2429.14 &lt;= EMA21 2477.61)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="D1291" t="n">
+        <v>731</v>
+      </c>
+      <c r="E1291" t="n">
+        <v>735.48</v>
+      </c>
+      <c r="F1291" t="n">
+        <v>735.48</v>
+      </c>
+      <c r="G1291" t="n">
+        <v>714.88</v>
+      </c>
+      <c r="H1291" t="n">
+        <v>716.14</v>
+      </c>
+      <c r="I1291" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J1291" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1291" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 714.88 &lt;= EMA21 716.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="D1292" t="n">
+        <v>550.95</v>
+      </c>
+      <c r="E1292" t="n">
+        <v>562.72</v>
+      </c>
+      <c r="F1292" t="n">
+        <v>562.72</v>
+      </c>
+      <c r="G1292" t="n">
+        <v>537.74</v>
+      </c>
+      <c r="H1292" t="n">
+        <v>538.05</v>
+      </c>
+      <c r="I1292" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="J1292" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1292" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 537.74 &lt;= EMA21 538.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>HINDALCO</t>
+        </is>
+      </c>
+      <c r="D1293" t="n">
+        <v>986.5</v>
+      </c>
+      <c r="E1293" t="n">
+        <v>1066.71</v>
+      </c>
+      <c r="F1293" t="n">
+        <v>1066.71</v>
+      </c>
+      <c r="G1293" t="n">
+        <v>989.95</v>
+      </c>
+      <c r="H1293" t="n">
+        <v>1003.65</v>
+      </c>
+      <c r="I1293" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="J1293" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1293" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 989.95 &lt;= EMA21 1003.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>HAL</t>
+        </is>
+      </c>
+      <c r="D1294" t="n">
+        <v>4800.3</v>
+      </c>
+      <c r="E1294" t="n">
+        <v>5031.15</v>
+      </c>
+      <c r="F1294" t="n">
+        <v>5031.15</v>
+      </c>
+      <c r="G1294" t="n">
+        <v>4819.46</v>
+      </c>
+      <c r="H1294" t="n">
+        <v>4841.31</v>
+      </c>
+      <c r="I1294" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1294" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1294" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4819.46 &lt;= EMA21 4841.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="D1295" t="n">
+        <v>1932</v>
+      </c>
+      <c r="E1295" t="n">
+        <v>2038.54</v>
+      </c>
+      <c r="F1295" t="n">
+        <v>2038.54</v>
+      </c>
+      <c r="G1295" t="n">
+        <v>1947.12</v>
+      </c>
+      <c r="H1295" t="n">
+        <v>1974.35</v>
+      </c>
+      <c r="I1295" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J1295" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1295" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1947.12 &lt;= EMA21 1974.35)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="D1296" t="n">
+        <v>596</v>
+      </c>
+      <c r="E1296" t="n">
+        <v>626.47</v>
+      </c>
+      <c r="F1296" t="n">
+        <v>626.47</v>
+      </c>
+      <c r="G1296" t="n">
+        <v>582.1799999999999</v>
+      </c>
+      <c r="H1296" t="n">
+        <v>583.98</v>
+      </c>
+      <c r="I1296" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J1296" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1296" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 582.18 &lt;= EMA21 583.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="D1297" t="n">
+        <v>2208.8</v>
+      </c>
+      <c r="E1297" t="n">
+        <v>2269.32</v>
+      </c>
+      <c r="F1297" t="n">
+        <v>2269.32</v>
+      </c>
+      <c r="G1297" t="n">
+        <v>2179.7</v>
+      </c>
+      <c r="H1297" t="n">
+        <v>2181.37</v>
+      </c>
+      <c r="I1297" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="J1297" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1297" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2179.70 &lt;= EMA21 2181.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="D1298" t="n">
+        <v>1338.9</v>
+      </c>
+      <c r="E1298" t="n">
+        <v>1472.49</v>
+      </c>
+      <c r="F1298" t="n">
+        <v>1472.49</v>
+      </c>
+      <c r="G1298" t="n">
+        <v>1368.57</v>
+      </c>
+      <c r="H1298" t="n">
+        <v>1391.02</v>
+      </c>
+      <c r="I1298" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="J1298" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1298" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1368.57 &lt;= EMA21 1391.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="D1299" t="n">
+        <v>262.3</v>
+      </c>
+      <c r="E1299" t="n">
+        <v>272.57</v>
+      </c>
+      <c r="F1299" t="n">
+        <v>272.57</v>
+      </c>
+      <c r="G1299" t="n">
+        <v>262.59</v>
+      </c>
+      <c r="H1299" t="n">
+        <v>265.13</v>
+      </c>
+      <c r="I1299" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="J1299" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1299" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 262.59 &lt;= EMA21 265.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>INDHOTEL</t>
+        </is>
+      </c>
+      <c r="D1300" t="n">
+        <v>732.75</v>
+      </c>
+      <c r="E1300" t="n">
+        <v>737.46</v>
+      </c>
+      <c r="F1300" t="n">
+        <v>737.46</v>
+      </c>
+      <c r="G1300" t="n">
+        <v>722.3200000000001</v>
+      </c>
+      <c r="H1300" t="n">
+        <v>722.71</v>
+      </c>
+      <c r="I1300" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="J1300" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1300" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 722.32 &lt;= EMA21 722.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="D1301" t="n">
+        <v>137</v>
+      </c>
+      <c r="E1301" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="F1301" t="n">
+        <v>140.3</v>
+      </c>
+      <c r="G1301" t="n">
+        <v>135.26</v>
+      </c>
+      <c r="H1301" t="n">
+        <v>136.16</v>
+      </c>
+      <c r="I1301" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="J1301" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1301" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 135.26 &lt;= EMA21 136.16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="D1302" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="E1302" t="n">
+        <v>86.58</v>
+      </c>
+      <c r="F1302" t="n">
+        <v>86.58</v>
+      </c>
+      <c r="G1302" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="H1302" t="n">
+        <v>82.44</v>
+      </c>
+      <c r="I1302" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J1302" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1302" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 80.80 &lt;= EMA21 82.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="D1303" t="n">
+        <v>1051.4</v>
+      </c>
+      <c r="E1303" t="n">
+        <v>1181.22</v>
+      </c>
+      <c r="F1303" t="n">
+        <v>1181.22</v>
+      </c>
+      <c r="G1303" t="n">
+        <v>1063.78</v>
+      </c>
+      <c r="H1303" t="n">
+        <v>1086.21</v>
+      </c>
+      <c r="I1303" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="J1303" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1303" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1063.78 &lt;= EMA21 1086.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>INDIGO</t>
+        </is>
+      </c>
+      <c r="D1304" t="n">
+        <v>4920</v>
+      </c>
+      <c r="E1304" t="n">
+        <v>5306.04</v>
+      </c>
+      <c r="F1304" t="n">
+        <v>5306.04</v>
+      </c>
+      <c r="G1304" t="n">
+        <v>4903.38</v>
+      </c>
+      <c r="H1304" t="n">
+        <v>4996.87</v>
+      </c>
+      <c r="I1304" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="J1304" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1304" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4903.38 &lt;= EMA21 4996.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>JSWSTEEL</t>
+        </is>
+      </c>
+      <c r="D1305" t="n">
+        <v>1275.6</v>
+      </c>
+      <c r="E1305" t="n">
+        <v>1360.83</v>
+      </c>
+      <c r="F1305" t="n">
+        <v>1360.83</v>
+      </c>
+      <c r="G1305" t="n">
+        <v>1274.17</v>
+      </c>
+      <c r="H1305" t="n">
+        <v>1286.24</v>
+      </c>
+      <c r="I1305" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="J1305" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1305" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1274.17 &lt;= EMA21 1286.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>JINDALSTEL</t>
+        </is>
+      </c>
+      <c r="D1306" t="n">
+        <v>1119.5</v>
+      </c>
+      <c r="E1306" t="n">
+        <v>1196.51</v>
+      </c>
+      <c r="F1306" t="n">
+        <v>1196.51</v>
+      </c>
+      <c r="G1306" t="n">
+        <v>1123.27</v>
+      </c>
+      <c r="H1306" t="n">
+        <v>1129.06</v>
+      </c>
+      <c r="I1306" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="J1306" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1306" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1123.27 &lt;= EMA21 1129.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>JIOFIN</t>
+        </is>
+      </c>
+      <c r="D1307" t="n">
+        <v>229.89</v>
+      </c>
+      <c r="E1307" t="n">
+        <v>245.69</v>
+      </c>
+      <c r="F1307" t="n">
+        <v>245.69</v>
+      </c>
+      <c r="G1307" t="n">
+        <v>230.05</v>
+      </c>
+      <c r="H1307" t="n">
+        <v>234.44</v>
+      </c>
+      <c r="I1307" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="J1307" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1307" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 230.05 &lt;= EMA21 234.44)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="D1308" t="n">
+        <v>412.5</v>
+      </c>
+      <c r="E1308" t="n">
+        <v>430.89</v>
+      </c>
+      <c r="F1308" t="n">
+        <v>430.89</v>
+      </c>
+      <c r="G1308" t="n">
+        <v>415.54</v>
+      </c>
+      <c r="H1308" t="n">
+        <v>413.24</v>
+      </c>
+      <c r="I1308" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1308" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1308" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 412.50 &lt;= Upper 430.89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>LTM</t>
+        </is>
+      </c>
+      <c r="D1309" t="n">
+        <v>4275.1</v>
+      </c>
+      <c r="E1309" t="n">
+        <v>4707.74</v>
+      </c>
+      <c r="F1309" t="n">
+        <v>4707.74</v>
+      </c>
+      <c r="G1309" t="n">
+        <v>4327.59</v>
+      </c>
+      <c r="H1309" t="n">
+        <v>4402.56</v>
+      </c>
+      <c r="I1309" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J1309" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1309" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4327.59 &lt;= EMA21 4402.56)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="D1310" t="n">
+        <v>3885</v>
+      </c>
+      <c r="E1310" t="n">
+        <v>4130.94</v>
+      </c>
+      <c r="F1310" t="n">
+        <v>4130.94</v>
+      </c>
+      <c r="G1310" t="n">
+        <v>3893.98</v>
+      </c>
+      <c r="H1310" t="n">
+        <v>3941.71</v>
+      </c>
+      <c r="I1310" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="J1310" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1310" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3893.98 &lt;= EMA21 3941.71)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>LODHA</t>
+        </is>
+      </c>
+      <c r="D1311" t="n">
+        <v>1144.7</v>
+      </c>
+      <c r="E1311" t="n">
+        <v>1318.01</v>
+      </c>
+      <c r="F1311" t="n">
+        <v>1318.01</v>
+      </c>
+      <c r="G1311" t="n">
+        <v>1132.96</v>
+      </c>
+      <c r="H1311" t="n">
+        <v>1166.31</v>
+      </c>
+      <c r="I1311" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="J1311" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1311" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1132.96 &lt;= EMA21 1166.31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>M&amp;M</t>
+        </is>
+      </c>
+      <c r="D1312" t="n">
+        <v>3052</v>
+      </c>
+      <c r="E1312" t="n">
+        <v>3453.56</v>
+      </c>
+      <c r="F1312" t="n">
+        <v>3453.56</v>
+      </c>
+      <c r="G1312" t="n">
+        <v>3100.61</v>
+      </c>
+      <c r="H1312" t="n">
+        <v>3177</v>
+      </c>
+      <c r="I1312" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="J1312" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1312" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3100.61 &lt;= EMA21 3177.00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="D1313" t="n">
+        <v>12103</v>
+      </c>
+      <c r="E1313" t="n">
+        <v>13877.04</v>
+      </c>
+      <c r="F1313" t="n">
+        <v>13877.04</v>
+      </c>
+      <c r="G1313" t="n">
+        <v>12398.37</v>
+      </c>
+      <c r="H1313" t="n">
+        <v>12770.01</v>
+      </c>
+      <c r="I1313" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J1313" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1313" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 12398.37 &lt;= EMA21 12770.01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>MAXHEALTH</t>
+        </is>
+      </c>
+      <c r="D1314" t="n">
+        <v>1049.3</v>
+      </c>
+      <c r="E1314" t="n">
+        <v>1058.66</v>
+      </c>
+      <c r="F1314" t="n">
+        <v>1058.66</v>
+      </c>
+      <c r="G1314" t="n">
+        <v>1031.04</v>
+      </c>
+      <c r="H1314" t="n">
+        <v>1026.21</v>
+      </c>
+      <c r="I1314" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="J1314" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1314" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 1049.30 &lt;= Upper 1058.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>MAZDOCK</t>
+        </is>
+      </c>
+      <c r="D1315" t="n">
+        <v>2280</v>
+      </c>
+      <c r="E1315" t="n">
+        <v>2684.23</v>
+      </c>
+      <c r="F1315" t="n">
+        <v>2684.23</v>
+      </c>
+      <c r="G1315" t="n">
+        <v>2312.82</v>
+      </c>
+      <c r="H1315" t="n">
+        <v>2388.92</v>
+      </c>
+      <c r="I1315" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="J1315" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1315" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2312.82 &lt;= EMA21 2388.92)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>MUTHOOTFIN</t>
+        </is>
+      </c>
+      <c r="D1316" t="n">
+        <v>2841.1</v>
+      </c>
+      <c r="E1316" t="n">
+        <v>3241.57</v>
+      </c>
+      <c r="F1316" t="n">
+        <v>3241.57</v>
+      </c>
+      <c r="G1316" t="n">
+        <v>2835.24</v>
+      </c>
+      <c r="H1316" t="n">
+        <v>2894.21</v>
+      </c>
+      <c r="I1316" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J1316" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1316" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2835.24 &lt;= EMA21 2894.21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="D1317" t="n">
+        <v>323.65</v>
+      </c>
+      <c r="E1317" t="n">
+        <v>338.22</v>
+      </c>
+      <c r="F1317" t="n">
+        <v>338.22</v>
+      </c>
+      <c r="G1317" t="n">
+        <v>329.28</v>
+      </c>
+      <c r="H1317" t="n">
+        <v>331.29</v>
+      </c>
+      <c r="I1317" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1317" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1317" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 329.28 &lt;= EMA21 331.29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="D1318" t="n">
+        <v>1372.4</v>
+      </c>
+      <c r="E1318" t="n">
+        <v>1502.49</v>
+      </c>
+      <c r="F1318" t="n">
+        <v>1502.49</v>
+      </c>
+      <c r="G1318" t="n">
+        <v>1388.28</v>
+      </c>
+      <c r="H1318" t="n">
+        <v>1415.06</v>
+      </c>
+      <c r="I1318" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="J1318" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1318" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1388.28 &lt;= EMA21 1415.06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="D1319" t="n">
+        <v>232.8</v>
+      </c>
+      <c r="E1319" t="n">
+        <v>238.08</v>
+      </c>
+      <c r="F1319" t="n">
+        <v>238.08</v>
+      </c>
+      <c r="G1319" t="n">
+        <v>234.12</v>
+      </c>
+      <c r="H1319" t="n">
+        <v>234.86</v>
+      </c>
+      <c r="I1319" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J1319" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1319" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 234.12 &lt;= EMA21 234.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="D1320" t="n">
+        <v>1572.1</v>
+      </c>
+      <c r="E1320" t="n">
+        <v>1700.27</v>
+      </c>
+      <c r="F1320" t="n">
+        <v>1700.27</v>
+      </c>
+      <c r="G1320" t="n">
+        <v>1567.69</v>
+      </c>
+      <c r="H1320" t="n">
+        <v>1594.04</v>
+      </c>
+      <c r="I1320" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J1320" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1320" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1567.69 &lt;= EMA21 1594.04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="D1321" t="n">
+        <v>342.55</v>
+      </c>
+      <c r="E1321" t="n">
+        <v>365.39</v>
+      </c>
+      <c r="F1321" t="n">
+        <v>365.39</v>
+      </c>
+      <c r="G1321" t="n">
+        <v>348.66</v>
+      </c>
+      <c r="H1321" t="n">
+        <v>355.69</v>
+      </c>
+      <c r="I1321" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J1321" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1321" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 348.66 &lt;= EMA21 355.69)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="D1322" t="n">
+        <v>270.3</v>
+      </c>
+      <c r="E1322" t="n">
+        <v>273.13</v>
+      </c>
+      <c r="F1322" t="n">
+        <v>273.13</v>
+      </c>
+      <c r="G1322" t="n">
+        <v>266.91</v>
+      </c>
+      <c r="H1322" t="n">
+        <v>267.87</v>
+      </c>
+      <c r="I1322" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="J1322" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1322" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 266.91 &lt;= EMA21 267.87)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
+      <c r="D1323" t="n">
+        <v>117.27</v>
+      </c>
+      <c r="E1323" t="n">
+        <v>117.76</v>
+      </c>
+      <c r="F1323" t="n">
+        <v>117.76</v>
+      </c>
+      <c r="G1323" t="n">
+        <v>116.45</v>
+      </c>
+      <c r="H1323" t="n">
+        <v>116.02</v>
+      </c>
+      <c r="I1323" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="J1323" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1323" t="inlineStr">
+        <is>
+          <t>BELOW_BAND (Close 117.27 &lt;= Upper 117.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>RECLTD</t>
+        </is>
+      </c>
+      <c r="D1324" t="n">
+        <v>312</v>
+      </c>
+      <c r="E1324" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="F1324" t="n">
+        <v>328.3</v>
+      </c>
+      <c r="G1324" t="n">
+        <v>313.52</v>
+      </c>
+      <c r="H1324" t="n">
+        <v>319.91</v>
+      </c>
+      <c r="I1324" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="J1324" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1324" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 313.52 &lt;= EMA21 319.91)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="D1325" t="n">
+        <v>1226.4</v>
+      </c>
+      <c r="E1325" t="n">
+        <v>1341.08</v>
+      </c>
+      <c r="F1325" t="n">
+        <v>1341.08</v>
+      </c>
+      <c r="G1325" t="n">
+        <v>1254.23</v>
+      </c>
+      <c r="H1325" t="n">
+        <v>1274.86</v>
+      </c>
+      <c r="I1325" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="J1325" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1325" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1254.23 &lt;= EMA21 1274.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="D1326" t="n">
+        <v>1731</v>
+      </c>
+      <c r="E1326" t="n">
+        <v>1799.13</v>
+      </c>
+      <c r="F1326" t="n">
+        <v>1799.13</v>
+      </c>
+      <c r="G1326" t="n">
+        <v>1715.42</v>
+      </c>
+      <c r="H1326" t="n">
+        <v>1733.27</v>
+      </c>
+      <c r="I1326" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1326" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1326" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1715.42 &lt;= EMA21 1733.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>MOTHERSON</t>
+        </is>
+      </c>
+      <c r="D1327" t="n">
+        <v>162.57</v>
+      </c>
+      <c r="E1327" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="F1327" t="n">
+        <v>169.99</v>
+      </c>
+      <c r="G1327" t="n">
+        <v>162.05</v>
+      </c>
+      <c r="H1327" t="n">
+        <v>162.66</v>
+      </c>
+      <c r="I1327" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J1327" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1327" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 162.05 &lt;= EMA21 162.66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="D1328" t="n">
+        <v>22600</v>
+      </c>
+      <c r="E1328" t="n">
+        <v>25056.23</v>
+      </c>
+      <c r="F1328" t="n">
+        <v>25056.23</v>
+      </c>
+      <c r="G1328" t="n">
+        <v>22529.07</v>
+      </c>
+      <c r="H1328" t="n">
+        <v>23251.6</v>
+      </c>
+      <c r="I1328" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="J1328" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1328" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 22529.07 &lt;= EMA21 23251.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>SHRIRAMFIN</t>
+        </is>
+      </c>
+      <c r="D1329" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E1329" t="n">
+        <v>1144.48</v>
+      </c>
+      <c r="F1329" t="n">
+        <v>1144.48</v>
+      </c>
+      <c r="G1329" t="n">
+        <v>1013.66</v>
+      </c>
+      <c r="H1329" t="n">
+        <v>1040.11</v>
+      </c>
+      <c r="I1329" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="J1329" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1329" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1013.66 &lt;= EMA21 1040.11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>ENRIN</t>
+        </is>
+      </c>
+      <c r="D1330" t="n">
+        <v>3228</v>
+      </c>
+      <c r="E1330" t="n">
+        <v>3418.88</v>
+      </c>
+      <c r="F1330" t="n">
+        <v>3418.88</v>
+      </c>
+      <c r="G1330" t="n">
+        <v>3145.28</v>
+      </c>
+      <c r="H1330" t="n">
+        <v>3205.24</v>
+      </c>
+      <c r="I1330" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J1330" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1330" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3145.28 &lt;= EMA21 3205.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>SIEMENS</t>
+        </is>
+      </c>
+      <c r="D1331" t="n">
+        <v>3913.9</v>
+      </c>
+      <c r="E1331" t="n">
+        <v>4174.34</v>
+      </c>
+      <c r="F1331" t="n">
+        <v>4174.34</v>
+      </c>
+      <c r="G1331" t="n">
+        <v>3896.47</v>
+      </c>
+      <c r="H1331" t="n">
+        <v>3926.84</v>
+      </c>
+      <c r="I1331" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="J1331" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1331" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 3896.47 &lt;= EMA21 3926.84)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>SOLARINDS</t>
+        </is>
+      </c>
+      <c r="D1332" t="n">
+        <v>18555</v>
+      </c>
+      <c r="E1332" t="n">
+        <v>23305.56</v>
+      </c>
+      <c r="F1332" t="n">
+        <v>23305.56</v>
+      </c>
+      <c r="G1332" t="n">
+        <v>20067.58</v>
+      </c>
+      <c r="H1332" t="n">
+        <v>20340.6</v>
+      </c>
+      <c r="I1332" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="J1332" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1332" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 20067.58 &lt;= EMA21 20340.60)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="D1333" t="n">
+        <v>996.2</v>
+      </c>
+      <c r="E1333" t="n">
+        <v>1067.97</v>
+      </c>
+      <c r="F1333" t="n">
+        <v>1067.97</v>
+      </c>
+      <c r="G1333" t="n">
+        <v>997.0700000000001</v>
+      </c>
+      <c r="H1333" t="n">
+        <v>1012.8</v>
+      </c>
+      <c r="I1333" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="J1333" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1333" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 997.07 &lt;= EMA21 1012.80)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="D1334" t="n">
+        <v>1837.3</v>
+      </c>
+      <c r="E1334" t="n">
+        <v>1969.89</v>
+      </c>
+      <c r="F1334" t="n">
+        <v>1969.89</v>
+      </c>
+      <c r="G1334" t="n">
+        <v>1858.86</v>
+      </c>
+      <c r="H1334" t="n">
+        <v>1881.19</v>
+      </c>
+      <c r="I1334" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="J1334" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1334" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1858.86 &lt;= EMA21 1881.19)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>TVSMOTOR</t>
+        </is>
+      </c>
+      <c r="D1335" t="n">
+        <v>4171.3</v>
+      </c>
+      <c r="E1335" t="n">
+        <v>4465.53</v>
+      </c>
+      <c r="F1335" t="n">
+        <v>4465.53</v>
+      </c>
+      <c r="G1335" t="n">
+        <v>4126.61</v>
+      </c>
+      <c r="H1335" t="n">
+        <v>4171.73</v>
+      </c>
+      <c r="I1335" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="J1335" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1335" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4126.61 &lt;= EMA21 4171.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>TATACAP</t>
+        </is>
+      </c>
+      <c r="D1336" t="n">
+        <v>351.35</v>
+      </c>
+      <c r="E1336" t="n">
+        <v>382.92</v>
+      </c>
+      <c r="F1336" t="n">
+        <v>382.92</v>
+      </c>
+      <c r="G1336" t="n">
+        <v>355.2</v>
+      </c>
+      <c r="H1336" t="n">
+        <v>360.37</v>
+      </c>
+      <c r="I1336" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="J1336" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1336" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 355.20 &lt;= EMA21 360.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="D1337" t="n">
+        <v>2105</v>
+      </c>
+      <c r="E1337" t="n">
+        <v>2408.07</v>
+      </c>
+      <c r="F1337" t="n">
+        <v>2408.07</v>
+      </c>
+      <c r="G1337" t="n">
+        <v>2201.18</v>
+      </c>
+      <c r="H1337" t="n">
+        <v>2247.07</v>
+      </c>
+      <c r="I1337" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="J1337" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1337" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2201.18 &lt;= EMA21 2247.07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="D1338" t="n">
+        <v>996</v>
+      </c>
+      <c r="E1338" t="n">
+        <v>1065.06</v>
+      </c>
+      <c r="F1338" t="n">
+        <v>1065.06</v>
+      </c>
+      <c r="G1338" t="n">
+        <v>1002.84</v>
+      </c>
+      <c r="H1338" t="n">
+        <v>1019.26</v>
+      </c>
+      <c r="I1338" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="J1338" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1338" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1002.84 &lt;= EMA21 1019.26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>TMCV</t>
+        </is>
+      </c>
+      <c r="D1339" t="n">
+        <v>442.9</v>
+      </c>
+      <c r="E1339" t="n">
+        <v>489</v>
+      </c>
+      <c r="F1339" t="n">
+        <v>489</v>
+      </c>
+      <c r="G1339" t="n">
+        <v>439.57</v>
+      </c>
+      <c r="H1339" t="n">
+        <v>446.98</v>
+      </c>
+      <c r="I1339" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="J1339" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1339" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 439.57 &lt;= EMA21 446.98)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>TMPV</t>
+        </is>
+      </c>
+      <c r="D1340" t="n">
+        <v>303.8</v>
+      </c>
+      <c r="E1340" t="n">
+        <v>320.44</v>
+      </c>
+      <c r="F1340" t="n">
+        <v>320.44</v>
+      </c>
+      <c r="G1340" t="n">
+        <v>305.82</v>
+      </c>
+      <c r="H1340" t="n">
+        <v>310.86</v>
+      </c>
+      <c r="I1340" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="J1340" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1340" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 305.82 &lt;= EMA21 310.86)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>TATAPOWER</t>
+        </is>
+      </c>
+      <c r="D1341" t="n">
+        <v>374.8</v>
+      </c>
+      <c r="E1341" t="n">
+        <v>378.94</v>
+      </c>
+      <c r="F1341" t="n">
+        <v>378.94</v>
+      </c>
+      <c r="G1341" t="n">
+        <v>366.88</v>
+      </c>
+      <c r="H1341" t="n">
+        <v>367.18</v>
+      </c>
+      <c r="I1341" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="J1341" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1341" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 366.88 &lt;= EMA21 367.18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>TATASTEEL</t>
+        </is>
+      </c>
+      <c r="D1342" t="n">
+        <v>185.54</v>
+      </c>
+      <c r="E1342" t="n">
+        <v>189.36</v>
+      </c>
+      <c r="F1342" t="n">
+        <v>189.36</v>
+      </c>
+      <c r="G1342" t="n">
+        <v>185.1</v>
+      </c>
+      <c r="H1342" t="n">
+        <v>185.43</v>
+      </c>
+      <c r="I1342" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="J1342" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1342" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 185.10 &lt;= EMA21 185.43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>TECHM</t>
+        </is>
+      </c>
+      <c r="D1343" t="n">
+        <v>1537.1</v>
+      </c>
+      <c r="E1343" t="n">
+        <v>1653.31</v>
+      </c>
+      <c r="F1343" t="n">
+        <v>1653.31</v>
+      </c>
+      <c r="G1343" t="n">
+        <v>1557.32</v>
+      </c>
+      <c r="H1343" t="n">
+        <v>1573.73</v>
+      </c>
+      <c r="I1343" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J1343" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1343" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1557.32 &lt;= EMA21 1573.73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="D1344" t="n">
+        <v>4798.5</v>
+      </c>
+      <c r="E1344" t="n">
+        <v>5215.97</v>
+      </c>
+      <c r="F1344" t="n">
+        <v>5215.97</v>
+      </c>
+      <c r="G1344" t="n">
+        <v>4917.03</v>
+      </c>
+      <c r="H1344" t="n">
+        <v>4966.37</v>
+      </c>
+      <c r="I1344" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="J1344" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1344" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4917.03 &lt;= EMA21 4966.37)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="D1345" t="n">
+        <v>4840</v>
+      </c>
+      <c r="E1345" t="n">
+        <v>5067.59</v>
+      </c>
+      <c r="F1345" t="n">
+        <v>5067.59</v>
+      </c>
+      <c r="G1345" t="n">
+        <v>4892.47</v>
+      </c>
+      <c r="H1345" t="n">
+        <v>4918.14</v>
+      </c>
+      <c r="I1345" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="J1345" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1345" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 4892.47 &lt;= EMA21 4918.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>TRENT</t>
+        </is>
+      </c>
+      <c r="D1346" t="n">
+        <v>2824</v>
+      </c>
+      <c r="E1346" t="n">
+        <v>2940.36</v>
+      </c>
+      <c r="F1346" t="n">
+        <v>2940.36</v>
+      </c>
+      <c r="G1346" t="n">
+        <v>2802.07</v>
+      </c>
+      <c r="H1346" t="n">
+        <v>2840.09</v>
+      </c>
+      <c r="I1346" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="J1346" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1346" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 2802.07 &lt;= EMA21 2840.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="D1347" t="n">
+        <v>11014</v>
+      </c>
+      <c r="E1347" t="n">
+        <v>11870.66</v>
+      </c>
+      <c r="F1347" t="n">
+        <v>11870.66</v>
+      </c>
+      <c r="G1347" t="n">
+        <v>10944.8</v>
+      </c>
+      <c r="H1347" t="n">
+        <v>11155.2</v>
+      </c>
+      <c r="I1347" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="J1347" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1347" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 10944.80 &lt;= EMA21 11155.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D1348" t="n">
+        <v>176.56</v>
+      </c>
+      <c r="E1348" t="n">
+        <v>191.99</v>
+      </c>
+      <c r="F1348" t="n">
+        <v>191.99</v>
+      </c>
+      <c r="G1348" t="n">
+        <v>179.1</v>
+      </c>
+      <c r="H1348" t="n">
+        <v>181.02</v>
+      </c>
+      <c r="I1348" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="J1348" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1348" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 179.10 &lt;= EMA21 181.02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>UNITDSPR</t>
+        </is>
+      </c>
+      <c r="D1349" t="n">
+        <v>1371</v>
+      </c>
+      <c r="E1349" t="n">
+        <v>1576.53</v>
+      </c>
+      <c r="F1349" t="n">
+        <v>1576.53</v>
+      </c>
+      <c r="G1349" t="n">
+        <v>1400.35</v>
+      </c>
+      <c r="H1349" t="n">
+        <v>1436.24</v>
+      </c>
+      <c r="I1349" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J1349" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1349" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1400.35 &lt;= EMA21 1436.24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>VBL</t>
+        </is>
+      </c>
+      <c r="D1350" t="n">
+        <v>421.95</v>
+      </c>
+      <c r="E1350" t="n">
+        <v>431.49</v>
+      </c>
+      <c r="F1350" t="n">
+        <v>431.49</v>
+      </c>
+      <c r="G1350" t="n">
+        <v>414.3</v>
+      </c>
+      <c r="H1350" t="n">
+        <v>417.76</v>
+      </c>
+      <c r="I1350" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="J1350" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1350" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 414.30 &lt;= EMA21 417.76)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>VEDL</t>
+        </is>
+      </c>
+      <c r="D1351" t="n">
+        <v>267.6</v>
+      </c>
+      <c r="E1351" t="n">
+        <v>288.65</v>
+      </c>
+      <c r="F1351" t="n">
+        <v>288.65</v>
+      </c>
+      <c r="G1351" t="n">
+        <v>264.02</v>
+      </c>
+      <c r="H1351" t="n">
+        <v>267.79</v>
+      </c>
+      <c r="I1351" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="J1351" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1351" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 264.02 &lt;= EMA21 267.79)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="D1352" t="n">
+        <v>166.83</v>
+      </c>
+      <c r="E1352" t="n">
+        <v>186.02</v>
+      </c>
+      <c r="F1352" t="n">
+        <v>186.02</v>
+      </c>
+      <c r="G1352" t="n">
+        <v>168.75</v>
+      </c>
+      <c r="H1352" t="n">
+        <v>172.53</v>
+      </c>
+      <c r="I1352" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="J1352" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1352" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 168.75 &lt;= EMA21 172.53)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>ZYDUSLIFE</t>
+        </is>
+      </c>
+      <c r="D1353" t="n">
+        <v>1160</v>
+      </c>
+      <c r="E1353" t="n">
+        <v>1192.94</v>
+      </c>
+      <c r="F1353" t="n">
+        <v>1192.94</v>
+      </c>
+      <c r="G1353" t="n">
+        <v>1131.39</v>
+      </c>
+      <c r="H1353" t="n">
+        <v>1133.68</v>
+      </c>
+      <c r="I1353" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="J1353" t="b">
+        <v>0</v>
+      </c>
+      <c r="K1353" t="inlineStr">
+        <is>
+          <t>EMA_BEARISH (EMA9 1131.39 &lt;= EMA21 1133.68)</t>
         </is>
       </c>
     </row>
@@ -54320,7 +58620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54603,6 +58903,37 @@
         <v>2.08</v>
       </c>
       <c r="G9" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1824</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1741.92</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>
@@ -54619,7 +58950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -54676,6 +59007,47 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1824</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" t="n">
+        <v>18240</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1824</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1741.92</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1824</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
         </is>
       </c>
     </row>
@@ -55791,7 +60163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K151"/>
+  <dimension ref="A1:K152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61224,6 +65596,55 @@
       <c r="K151" t="inlineStr">
         <is>
           <t>HARD_STOP_LOSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-18 20:02:11</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>D0431998D6</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>1824</v>
+      </c>
+      <c r="G152" t="n">
+        <v>1824</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" t="n">
+        <v>10</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>FILLED</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Entry Breakout</t>
         </is>
       </c>
     </row>
@@ -61306,7 +65727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -61884,6 +66305,39 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20:02:12</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>177876.98</v>
+      </c>
+      <c r="D18" t="n">
+        <v>18240</v>
+      </c>
+      <c r="E18" t="n">
+        <v>196116.98</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-3797.38</v>
+      </c>
+      <c r="G18" t="n">
+        <v>19</v>
+      </c>
+      <c r="H18" t="n">
+        <v>21</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>